<commit_message>
chore(editais): atualizacao automatica 2026-06-10 11:23
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -884,25 +892,32 @@
           <t>EDITAL FAPES Nº 12/2026 - EXTENSÃO TECNOLÓGICA</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 10/06/2026</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09: Data limite para submissão das propostas (até 17h59, via Sigfapes)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
+          <t>2026-06-30: Submissão de propostas (Até as 17h59 via Sigfapes)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas, coordenados por profissionais de Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) localizadas no Espírito Santo. O objetivo é promover o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, visando a inclusão social e produtiva nas microrregiões do estado." → "Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas. Os projetos devem ser coordenados por profissionais vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) no Espírito Santo, visando o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, com foco na inclusão social e produtiva nas microrregiões do estado."
+Público-alvo: "Profissionais vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T), públicas e privadas, com atividades de extensão regulamentadas, localizadas no estado do Espírito Santo. O proponente deve ser coordenador do projeto, possuir vínculo empregatício (ou termo de adesão a trabalho voluntário se aposentado), ter graduação concluída com 3 anos de experiência em projetos de extensão ou titulação mínima de mestre, currículo Lattes atualizado há menos de 6 meses, não integrar outra equipe executora neste edital, estar adimplente com a Fapes, ser brasileiro ou estrangeiro com visto permanente e residir no Espírito Santo ou municípios limítrofes." → "Profissionais (coordenadores de projeto) vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) públicas e privadas, localizadas no Espírito Santo, que possuam vínculo empregatício ou termo de adesão a trabalho voluntário, experiência em projetos de extensão ou titulação mínima de mestre, currículo Lattes atualizado, e que apresentem parceria com organização externa (empresa pública ou privada, cooperativa ou organização sem fins lucrativos)."
+Submissão (nova): Submissão de propostas — ? a 2026-06-30
+Submissão (removida): Data limite para submissão das propostas — ? a 2026-06-09</t>
+        </is>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas, coordenados por profissionais de Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) localizadas no Espírito Santo. O objetivo é promover o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, visando a inclusão social e produtiva nas microrregiões do estado.</t>
+          <t>Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas. Os projetos devem ser coordenados por profissionais vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) no Espírito Santo, visando o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, com foco na inclusão social e produtiva nas microrregiões do estado.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Profissionais vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T), públicas e privadas, com atividades de extensão regulamentadas, localizadas no estado do Espírito Santo. O proponente deve ser coordenador do projeto, possuir vínculo empregatício (ou termo de adesão a trabalho voluntário se aposentado), ter graduação concluída com 3 anos de experiência em projetos de extensão ou titulação mínima de mestre, currículo Lattes atualizado há menos de 6 meses, não integrar outra equipe executora neste edital, estar adimplente com a Fapes, ser brasileiro ou estrangeiro com visto permanente e residir no Espírito Santo ou municípios limítrofes.</t>
+          <t>Profissionais (coordenadores de projeto) vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) públicas e privadas, localizadas no Espírito Santo, que possuam vínculo empregatício ou termo de adesão a trabalho voluntário, experiência em projetos de extensão ou titulação mínima de mestre, currículo Lattes atualizado, e que apresentem parceria com organização externa (empresa pública ou privada, cooperativa ou organização sem fins lucrativos).</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -922,15 +937,16 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09: Data limite para submissão das propostas (até 17h59, via Sigfapes)
-?: Prazo para submissão de recursos administrativos (habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
-?: Prazo para submissão de recursos administrativos (mérito) (05 (cinco) dias úteis a partir da publicação do resultado preliminar do mérito)
-?: Início da contratação / Assinatura do Termo de Outorga (Até 5 (cinco) dias úteis da publicação do resultado homologado)</t>
+          <t>2026-06-30: Submissão de propostas (Até as 17h59 via Sigfapes)
+2026-06-27 a 2026-07-03: Prazo para submissão de recursos administrativos da habilitação (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
+2026-09-26 a 2026-10-01: Prazo para submissão de recursos administrativos da análise de mérito (05 (cinco) dias úteis a partir da publicação do resultado preliminar do mérito)
+2026-10-28: Assinatura do Termo de Outorga e Projeto Aprovado (Proponentes aprovados devem assinar eletronicamente via E-Docs. Prazo para assinatura será divulgado junto ao resultado final homologado.)
+?: Contratação de suplentes (Período a ser definido, se aplicável. Até as 17h00.)</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Serão apoiados 4 projetos oriundos das IES/P/T para cada microrregião e 10 projetos na ampla concorrência. Recursos remanescentes da não contratação de projetos em uma microrregião serão redistribuídos para os projetos mais bem classificados da ampla concorrência. O orçamento do projeto poderá ser aprovado na íntegra ou parcialmente. Cada proponente poderá ser coordenador(a) de somente uma proposta; em caso de mais de uma submissão, a última será considerada para análise. Não será permitida a participação de Empresário Individual, Microempreendedor individual (MEI) ou Empresa Júnior como empresa parceira do projeto.</t>
+          <t>O prazo de execução do projeto será de 24 meses. As propostas devem ser submetidas para desenvolvimento em apenas uma das 10 microrregiões listadas no Quadro 2. Serão apoiados 4 projetos por microrregião e 10 projetos na ampla concorrência. É obrigatória a permanência de no mínimo 1 bolsista EXT-E ou EXT-F a partir do 3º mês de vigência do projeto, pelo prazo mínimo de 22 meses. A soma dos serviços de terceiros é limitada a 30% do valor total do projeto aprovado (incluído DOACI). As despesas operacionais e administrativas (DOACI) são limitadas a 10% do valor total do projeto, descontados os valores de bolsa. Os valores destinados a diárias não poderão superar 50% do valor máximo permitido para o projeto. A proposta deve apresentar, pelo menos, uma parceria com organização externa. Cada proponente poderá ser coordenador de somente uma proposta. Propostas com Nota Final inferior a 70 pontos serão desclassificadas.</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-11 11:34
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -892,9 +884,9 @@
           <t>EDITAL FAPES Nº 12/2026 - EXTENSÃO TECNOLÓGICA</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 10/06/2026</t>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -902,14 +894,7 @@
           <t>2026-06-30: Submissão de propostas (Até as 17h59 via Sigfapes)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas, coordenados por profissionais de Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) localizadas no Espírito Santo. O objetivo é promover o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, visando a inclusão social e produtiva nas microrregiões do estado." → "Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas. Os projetos devem ser coordenados por profissionais vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) no Espírito Santo, visando o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, com foco na inclusão social e produtiva nas microrregiões do estado."
-Público-alvo: "Profissionais vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T), públicas e privadas, com atividades de extensão regulamentadas, localizadas no estado do Espírito Santo. O proponente deve ser coordenador do projeto, possuir vínculo empregatício (ou termo de adesão a trabalho voluntário se aposentado), ter graduação concluída com 3 anos de experiência em projetos de extensão ou titulação mínima de mestre, currículo Lattes atualizado há menos de 6 meses, não integrar outra equipe executora neste edital, estar adimplente com a Fapes, ser brasileiro ou estrangeiro com visto permanente e residir no Espírito Santo ou municípios limítrofes." → "Profissionais (coordenadores de projeto) vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) públicas e privadas, localizadas no Espírito Santo, que possuam vínculo empregatício ou termo de adesão a trabalho voluntário, experiência em projetos de extensão ou titulação mínima de mestre, currículo Lattes atualizado, e que apresentem parceria com organização externa (empresa pública ou privada, cooperativa ou organização sem fins lucrativos)."
-Submissão (nova): Submissão de propostas — ? a 2026-06-30
-Submissão (removida): Data limite para submissão das propostas — ? a 2026-06-09</t>
-        </is>
-      </c>
+      <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas. Os projetos devem ser coordenados por profissionais vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) no Espírito Santo, visando o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, com foco na inclusão social e produtiva nas microrregiões do estado.</t>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-20 09:25
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1257,28 +1265,28 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 20/06/2026</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
         </is>
       </c>
       <c r="H12" s="2" t="n"/>
@@ -1290,22 +1298,22 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1325,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1325,114 +1333,109 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
+          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-13: Prazo para envio de pré-propostas
-2026-04-13: Prazo para envio de propostas completas convidadas</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
-        </is>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
         </is>
       </c>
     </row>
@@ -1444,7 +1447,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
+          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1452,34 +1455,99 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-01 a 2026-11-15: Período para procedimento de recurso (Etapa 2)</t>
-        </is>
-      </c>
+      <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
+          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-13: Prazo para envio de pré-propostas
+2026-04-13: Prazo para envio de propostas completas convidadas</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 a 2026-11-15: Período para procedimento de recurso (Etapa 2)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
           <t>O edital visa impulsionar a digitalização e a inovação para ecossistemas marinhos, negócios e comunidades resilientes, fortalecendo a competitividade da Economia Azul da União Europeia. Serão financiados projetos de pesquisa e inovação que contribuam para a transição para uma economia azul sustentável, resiliente e neutra em carbono, com foco em áreas como Gêmeos Digitais do Oceano, transição de setores da economia azul, planejamento climático inteligente, bio-recursos azuis e comunidades costeiras resilientes. O objetivo é gerar conhecimento acionável e soluções para um oceano saudável e uma economia azul produtiva.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Consórcios compostos por parceiros elegíveis de pelo menos três países diferentes participantes da chamada, solicitando apoio financeiro de pelo menos três Organizações Financiadoras Participantes (PFOs) distintas. Adicionalmente, os projetos devem envolver pelo menos duas entidades legais independentes de dois Estados Membros da UE ou Países Associados ao Horizon Europe elegíveis para financiamento da UE. O Investigador Principal (PI) do coordenador do consórcio deve ser empregado por uma organização elegível em um dos países participantes da chamada.</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>32.045.000 Euro</t>
         </is>
       </c>
-      <c r="I15" s="2" t="n"/>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>sbep.call-secretariat@uefiscdi.ro, epss.sbep@g.etag.ee</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>2025-11-17: Prazo final para submissão de pré-propostas (Até as 15:00 CET)
 2026-03-15 a 2026-04-01: Período para procedimento de recurso (Etapa 1)
@@ -1488,77 +1556,77 @@
 ?: Negociações de subvenções nacionais/regionais para os projetos recomendados para financiamento</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>A chamada é co-patrocinada pela Década das Nações Unidas da Ciência Oceânica para o Desenvolvimento Sustentável. Os projetos devem ser orientados para o impacto, seguindo uma abordagem de via de impacto. É exigido o envolvimento de múltiplos stakeholders (quádrupla hélice), incluindo pelo menos um parceiro da indústria, governo, institutos de pesquisa ou público. Atividades de participação cidadã e literacia oceânica são encorajadas. As propostas são fortemente recomendadas a cobrir um mínimo de duas bacias marítimas da UE (Oceano Atlântico, Mar Báltico, Mar Negro, Mar Mediterrâneo, Mar do Norte). Todas as propostas devem estar alinhadas com a Taxonomia da UE e cumprir os princípios éticos. Um processo de submissão em duas etapas é obrigatório (pré-proposta e, em seguida, proposta completa mediante convite). As informações fornecidas nas pré-propostas são vinculativas para as propostas completas; nenhuma alteração importante no conteúdo é permitida. O coordenador do consórcio pode ser Investigador Principal (PI) em apenas uma proposta. Parceiros do mesmo país não podem solicitar mais de 60% do financiamento total. A duração do projeto é de 36 meses. Os beneficiários do financiamento devem reconhecer o financiamento da SBEP e do Horizon Europe e aderir à Política de Ciência Aberta da CE para publicações.</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/SBEP%20Call%20text%202025.pdf</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/3a_CHAMADA_TRANSACIONAL_CONJUNTA_-_PARCERIA_ECONOMIA_AZUL_SUSTENTÁVEL.pdf</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>USD 20.000,00</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Serão apoiados até 20 projetos de pesquisa conjuntos. As propostas devem ser elaboradas em inglês (máximo 10 páginas) e incluir uma descrição clara da colaboração planejada, valor agregado e complementaridade das equipes. As áreas de pesquisa prioritárias são: Clima, Sustentabilidade, Agricultura; Saúde Pública e Medicina; e Democracia e Inclusão. Cada PI pode submeter apenas uma proposta. O apoio financeiro para o lado brasileiro (FAPs) destina-se a cobrir custos gerais, viagens internacionais, diárias, fundos semente para custos diretos de pesquisa e workshops. É exigido seguro médico para visitantes.</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Cooperative%20Program%20-U%20of%20I%20and%20Confap%20v%205%2024-03.docx.pdf</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_BRASIL–ILLINOIS_2026.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-21 10:03
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1268,9 +1260,9 @@
           <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 20/06/2026</t>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-22 12:50
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1431,199 +1431,6 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-13: Prazo para envio de pré-propostas
-2026-04-13: Prazo para envio de propostas completas convidadas</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-01 a 2026-11-15: Período para procedimento de recurso (Etapa 2)</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>O edital visa impulsionar a digitalização e a inovação para ecossistemas marinhos, negócios e comunidades resilientes, fortalecendo a competitividade da Economia Azul da União Europeia. Serão financiados projetos de pesquisa e inovação que contribuam para a transição para uma economia azul sustentável, resiliente e neutra em carbono, com foco em áreas como Gêmeos Digitais do Oceano, transição de setores da economia azul, planejamento climático inteligente, bio-recursos azuis e comunidades costeiras resilientes. O objetivo é gerar conhecimento acionável e soluções para um oceano saudável e uma economia azul produtiva.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>Consórcios compostos por parceiros elegíveis de pelo menos três países diferentes participantes da chamada, solicitando apoio financeiro de pelo menos três Organizações Financiadoras Participantes (PFOs) distintas. Adicionalmente, os projetos devem envolver pelo menos duas entidades legais independentes de dois Estados Membros da UE ou Países Associados ao Horizon Europe elegíveis para financiamento da UE. O Investigador Principal (PI) do coordenador do consórcio deve ser empregado por uma organização elegível em um dos países participantes da chamada.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>32.045.000 Euro</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="n"/>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>sbep.call-secretariat@uefiscdi.ro, epss.sbep@g.etag.ee</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-17: Prazo final para submissão de pré-propostas (Até as 15:00 CET)
-2026-03-15 a 2026-04-01: Período para procedimento de recurso (Etapa 1)
-2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)
-2026-11-01 a 2026-11-15: Período para procedimento de recurso (Etapa 2)
-?: Negociações de subvenções nacionais/regionais para os projetos recomendados para financiamento</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>A chamada é co-patrocinada pela Década das Nações Unidas da Ciência Oceânica para o Desenvolvimento Sustentável. Os projetos devem ser orientados para o impacto, seguindo uma abordagem de via de impacto. É exigido o envolvimento de múltiplos stakeholders (quádrupla hélice), incluindo pelo menos um parceiro da indústria, governo, institutos de pesquisa ou público. Atividades de participação cidadã e literacia oceânica são encorajadas. As propostas são fortemente recomendadas a cobrir um mínimo de duas bacias marítimas da UE (Oceano Atlântico, Mar Báltico, Mar Negro, Mar Mediterrâneo, Mar do Norte). Todas as propostas devem estar alinhadas com a Taxonomia da UE e cumprir os princípios éticos. Um processo de submissão em duas etapas é obrigatório (pré-proposta e, em seguida, proposta completa mediante convite). As informações fornecidas nas pré-propostas são vinculativas para as propostas completas; nenhuma alteração importante no conteúdo é permitida. O coordenador do consórcio pode ser Investigador Principal (PI) em apenas uma proposta. Parceiros do mesmo país não podem solicitar mais de 60% do financiamento total. A duração do projeto é de 36 meses. Os beneficiários do financiamento devem reconhecer o financiamento da SBEP e do Horizon Europe e aderir à Política de Ciência Aberta da CE para publicações.</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/SBEP%20Call%20text%202025.pdf</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/3a_CHAMADA_TRANSACIONAL_CONJUNTA_-_PARCERIA_ECONOMIA_AZUL_SUSTENTÁVEL.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>USD 20.000,00</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>Serão apoiados até 20 projetos de pesquisa conjuntos. As propostas devem ser elaboradas em inglês (máximo 10 páginas) e incluir uma descrição clara da colaboração planejada, valor agregado e complementaridade das equipes. As áreas de pesquisa prioritárias são: Clima, Sustentabilidade, Agricultura; Saúde Pública e Medicina; e Democracia e Inclusão. Cada PI pode submeter apenas uma proposta. O apoio financeiro para o lado brasileiro (FAPs) destina-se a cobrir custos gerais, viagens internacionais, diárias, fundos semente para custos diretos de pesquisa e workshops. É exigido seguro médico para visitantes.</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Cooperative%20Program%20-U%20of%20I%20and%20Confap%20v%205%2024-03.docx.pdf</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_BRASIL–ILLINOIS_2026.pdf</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-23 10:41
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -799,46 +807,118 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 23/06/2026</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30: Contratação / Assinatura do TO e envio de documentos - 2ª Chamada (Até 30 dias após a publicação do resultado final homologado.)</t>
+          <t>2026-06-22 a 2026-07-24: Envio das inscrições - Categorias Projetos e Destaque (Até as 17h59, via SigFapes)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
+          <t>Reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, além de matérias jornalísticas relacionadas à Fapes ou a projetos por ela fomentados, visando valorizar a ciência, tecnologia e inovação e ampliar sua divulgação no Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos por ela fomentados.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>R$ 308.000,00</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>R$ 12.000,00</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22 a 2026-07-24: Envio das inscrições - Categorias Projetos e Destaque (Até as 17h59, via SigFapes)
+2026-06-22 a 2026-09-15: Envio das inscrições - Categoria Jornalismo (Até as 17h59, via SigFapes)
+?: Interposição de recursos administrativos (Até 5 (cinco) dias úteis após a publicação dos resultados preliminares no DIO-ES, via E-Flow)
+2026-11-03 a 2026-11-09: Votação popular - Categoria Jornalismo (No site da Fapes, uma única vez por subcategoria)
+?: Solicitação de pagamento da premiação (Prazo máximo de 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES, mediante abertura de processo eletrônico no sistema E-Flow, via E-Docs)</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Não podem participar servidores da Fapes, membros do CCAF, cônjuges, companheiros e parentes até o segundo grau. É permitida apenas uma inscrição por pessoa. Os valores das premiações são brutos e sujeitos a IRRF, tendo caráter honorífico e não gerando vínculo empregatício. Solicitações de acessibilidade devem ser feitas com 10 dias de antecedência do prazo final de inscrição. O comparecimento à cerimônia de premiação é obrigatório, ou indicação de representante. Para a categoria Jornalismo, a matéria deve ter sido veiculada entre 01/09/2025 e 15/09/2026.</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30: Contratação / Assinatura do TO e envio de documentos - 2ª Chamada (Até 30 dias após a publicação do resultado final homologado.)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
 2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
@@ -857,70 +937,70 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 12/2026 - EXTENSÃO TECNOLÓGICA</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Submissão de propostas (Até as 17h59 via Sigfapes)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas. Os projetos devem ser coordenados por profissionais vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) no Espírito Santo, visando o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, com foco na inclusão social e produtiva nas microrregiões do estado.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Profissionais (coordenadores de projeto) vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) públicas e privadas, localizadas no Espírito Santo, que possuam vínculo empregatício ou termo de adesão a trabalho voluntário, experiência em projetos de extensão ou titulação mínima de mestre, currículo Lattes atualizado, e que apresentem parceria com organização externa (empresa pública ou privada, cooperativa ou organização sem fins lucrativos).</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>R$ 60.000,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Submissão de propostas (Até as 17h59 via Sigfapes)
 2026-06-27 a 2026-07-03: Prazo para submissão de recursos administrativos da habilitação (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
@@ -929,70 +1009,70 @@
 ?: Contratação de suplentes (Período a ser definido, se aplicável. Até as 17h00.)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução do projeto será de 24 meses. As propostas devem ser submetidas para desenvolvimento em apenas uma das 10 microrregiões listadas no Quadro 2. Serão apoiados 4 projetos por microrregião e 10 projetos na ampla concorrência. É obrigatória a permanência de no mínimo 1 bolsista EXT-E ou EXT-F a partir do 3º mês de vigência do projeto, pelo prazo mínimo de 22 meses. A soma dos serviços de terceiros é limitada a 30% do valor total do projeto aprovado (incluído DOACI). As despesas operacionais e administrativas (DOACI) são limitadas a 10% do valor total do projeto, descontados os valores de bolsa. Os valores destinados a diárias não poderão superar 50% do valor máximo permitido para o projeto. A proposta deve apresentar, pelo menos, uma parceria com organização externa. Cada proponente poderá ser coordenador de somente uma proposta. Propostas com Nota Final inferior a 70 pontos serão desclassificadas.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Extensão%20Tecnológica%20-%2012-2026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_12_2026_-_EXTENSÃO_TECNOLÓGICA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>2026-06-23: Prazo para impugnação do edital (Até 5 dias úteis antes da data limite de submissão das propostas)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do estado.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com titulação mínima de mestre, experiência comprovada em projetos de extensão nos últimos 3 anos, e vínculo empregatício, estatutário, temporário ou voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo. O proponente não deve ter sido contratado no Edital Fapes nº 04/2025 nem solicitado prorrogação de projeto do Edital FAPES nº 02/2024.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 5.000.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 80.000,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-06-23: Prazo para impugnação do edital (Até 5 dias úteis antes da data limite de submissão das propostas)
 2026-06-30: Submissão de propostas (Até as 17h59 via SigFapes)
@@ -1001,66 +1081,66 @@
 2026-10-29 a 2026-11-05: Início da contratação e envio de documentos (Até 5 dias úteis da publicação do resultado homologado para o início do processo de contratação. Inclui assinatura do Termo de Outorga e envio do Registro da Lista de Checagem de Documentação (e-Flow) até as 17h00.)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução dos projetos é de 24 meses. É obrigatória a previsão de pelo menos um bolsista EXT-E ou EXT-F por um período mínimo de 22 meses. As propostas devem ser submetidas para apenas uma das 10 microrregiões listadas no edital. Proponentes que declararem pertencimento a grupos de ações afirmativas (PcD, negra, quilombola, indígena, trans ou travesti) podem receber pontuação adicional. Propostas com nota final inferior a 70 pontos serão desclassificadas. É exigida a elaboração de um vídeo apresentando os resultados do projeto. É indispensável a menção explícita e destacada ao apoio da Fapes em todas as divulgações do trabalho.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -1074,70 +1154,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
 2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h (horário de Brasília) via SIGFAPES)
@@ -1160,70 +1240,70 @@
 2027-05-04: Período de contratação de suplentes (2ª chamada) (Se aplicável, até as 17h00min)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital, sendo responsabilidade do proponente acompanhar as atualizações no site da FAPES. O edital poderá ser suspenso, revogado ou anulado por interesse público ou exigência legal, sem direito a indenização. O proponente deve manter seus dados cadastrais atualizados no SIGFAPES. A FAPES não exigirá direitos de participação e propriedade intelectual sobre as pesquisas e projetos, mas deverá ser notificada em caso de registro de propriedade intelectual. Os participantes concordam em ceder direitos de imagem para divulgação das ações da FAPES.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana, no Espírito Santo. Ele oferece apoio técnico e financeiro para soluções inovadoras com potencial de se tornarem negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação para o desenvolvimento sustentável.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central-Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>R$ 30.000,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)
 ?: Prazo para recurso administrativo (Fase 1) (Até 5 dias úteis após divulgação do resultado preliminar)
@@ -1233,79 +1313,19 @@
 ?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>O edital será executado em duas fases. Na Fase 1, serão selecionadas 80 propostas de cada microrregião. Na Fase 2, serão selecionadas 25 propostas ou mais por microrregião. O valor total do edital de R$ 4.500.000,00 será distribuído entre as 6 microrregiões, com até R$ 750.000,00 para cada, visando financiar 25 projetos ou mais por microrregião. A participação em no mínimo 80% das oficinas e mentorias é obrigatória para o proponente ou membros da equipe, sob pena de desclassificação. Proponentes podem submeter mais de uma proposta na Fase 1, mas apenas a de maior nota avançará para a Fase 2. Propostas com nota final inferior a 70,0 serão desclassificadas. A Fapes pode alterar as datas e prazos do cronograma.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1337,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1327,18 +1347,18 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
         </is>
       </c>
       <c r="H13" s="2" t="n"/>
@@ -1350,22 +1370,22 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1397,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1385,47 +1405,107 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
+          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-24 10:15
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -608,7 +600,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23: Submissão das propostas (até as 17h59 (horário de Brasília))</t>
+          <t>2026-08-03: Contratação dos projetos</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
@@ -674,11 +666,7 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-25 a 2026-06-23: Submissão de candidaturas (O prazo de submissão vence às 17h59min do dia 23/06/2026. O Governo do Estado do Espírito Santo e o Instituto Trajetórias fornecem suporte e informações aos candidatos de 08h até às 18h. É considerado o horário oficial de Brasília/DF.)</t>
-        </is>
-      </c>
+      <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -748,7 +736,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25 a 2026-06-23: Submissão de candidatura (Prazo de submissão vence às 17h59min do dia 23/06/2026. Suporte e informações aos candidatos de 08h até às 18h (horário oficial de Brasília/DF).)</t>
+          <t>2026-07-01 a 2026-07-07: Interposição de recurso administrativo (Prazo de 05 (cinco) dias úteis após a divulgação do resultado preliminar. Interposto via formulário específico no Sistema E-Flow.)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -810,9 +798,9 @@
           <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 23/06/2026</t>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1043,7 +1031,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23: Prazo para impugnação do edital (Até 5 dias úteis antes da data limite de submissão das propostas)</t>
+          <t>2026-06-30: Submissão de propostas (Até as 17h59 via SigFapes)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-25 10:14
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -585,12 +585,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Formação Científica</t>
+          <t>Difusão do Conhecimento</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 13/2026  - PROGRAMA INSTITUCIONAL DE BOLSAS DE INICIAÇÃO CIENTÍFICA, TECNOLÓGICA E DE INOVAÇÃO DO ESPÍRITO SANTO (PIBICES 2026/2027)</t>
+          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -600,241 +600,36 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03: Contratação dos projetos</t>
+          <t>2026-06-22 a 2026-07-24: Envio das inscrições - Categorias Projetos e Destaque (Até as 17h59, via SigFapes)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>O Programa Institucional de Bolsas de Iniciação Científica, Tecnológica e de Inovação do Estado do Espírito Santo (PIBICES) visa fomentar a participação de estudantes de graduação em atividades sistemáticas de pesquisa científica, desenvolvimento tecnológico e inovação. O edital busca fortalecer o sistema capixaba de pesquisa e a formação de recursos humanos qualificados, contribuindo para a ampliação da cultura científica e a produção de conhecimento alinhada às demandas da sociedade. Serão concedidas cotas institucionais de bolsas para Programas Institucionais de Bolsas de Iniciação Científica, Tecnológica e de Inovação (PIBICTI) em Instituições de Ensino Superior e/ou Pesquisa.</t>
+          <t>Reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, além de matérias jornalísticas relacionadas à Fapes ou a projetos por ela fomentados, visando valorizar a ciência, tecnologia e inovação e ampliar sua divulgação no Espírito Santo.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Coordenadores Institucionais de Programas de Bolsas de Iniciação Científica, Tecnológica e de Inovação (PIBICTI) vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P), públicas ou privadas, localizadas no estado do Espírito Santo, que sejam pesquisadores/docentes com título de mestre ou doutor e vínculo empregatício indeterminado com a IES/P.</t>
+          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos por ela fomentados.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>R$ 8.640.000,00</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="n"/>
+          <t>R$ 308.000,00</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>R$ 12.000,00</t>
+        </is>
+      </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>bolsas.duvidas@fapes.es.gov.br</t>
+          <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-16: Impugnação do edital (até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)
-2026-06-23: Submissão das propostas (até as 17h59 (horário de Brasília))
-?: Interposição de recursos (habilitação) (até 5 dias úteis após a divulgação do resultado preliminar)
-2026-08-03: Contratação dos projetos
-?: Indicação dos bolsistas (a partir do início de vigência do Termo de Outorga)</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>Serão disponibilizadas 800 bolsas de Iniciação Científica e Tecnológica (ICT). Cada bolsa terá duração mínima de 4 e máxima de 12 meses, com valor mensal atual de R$ 900,00. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. É obrigatório mencionar o apoio da Fapes em todas as publicações ou divulgações de atividades, utilizando a citação padrão fornecida no edital. A Fapes pode alterar datas e prazos do cronograma ou reabrir prazos em casos de força maior ou falhas comprovadas nos sistemas.</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20PIBICES%20-%20Assinado.pdf</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>formacao_cientifica/EDITAL_FAPES_No_13_2026_-_PROGRAMA_INSTITUCIONAL_DE_BOLSAS_DE_INICIAÇÃO_CIENTÍFICA,_TECNOLÓGICA_E_DE_INOVAÇÃO_DO_ESPÍRITO_SANTO_(PIBICES_2026_2027).pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Formação Científica</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES/SEGER Nº 14/2026 - PROGRAMA TALENTOS GLOBAIS ESPÍRITO SANTO - MESTRADO INTERNACIONAL SERVIDORES PÚBLICOS 2026</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Este edital visa selecionar até 10 servidores públicos efetivos, estáveis e ativos do Poder Executivo do Estado do Espírito Santo para realizar cursos presenciais de mestrado em universidades estrangeiras de excelência. O programa busca fortalecer a capacidade institucional do Estado, apoiar projetos de pesquisa e desenvolver lideranças transformadoras no setor público, contribuindo para a geração de conhecimento, inovação e desenvolvimento.</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Servidores públicos estaduais efetivos, estáveis e ativos do Poder Executivo do Estado do Espírito Santo integrantes da administração pública direta, autárquica ou fundacional.</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>US$ 500.000,00</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Bolsa de estudo de mestrado internacional (BMI-TG) de US$ 5.000,00 por parcela trimestral (vigência de 12 a 24 meses) e Auxílio-Instalação (AI-TG) de US$ 10.000,00 em parcela única.</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>bolsas.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>?: Impugnação ao Edital (Até 5 (cinco) dias úteis anteriores ao encerramento do prazo de submissão das propostas.)
-2026-05-25 a 2026-06-23: Submissão de candidaturas (O prazo de submissão vence às 17h59min do dia 23/06/2026. O Governo do Estado do Espírito Santo e o Instituto Trajetórias fornecem suporte e informações aos candidatos de 08h até às 18h. É considerado o horário oficial de Brasília/DF.)
-?: Interposição de recurso administrativo do resultado preliminar de habilitação e de avaliação de mérito (Prazo de 05 (cinco) dias úteis após a divulgação do resultado preliminar.)
-?: Atualização documental para contratação (O cronograma do procedimento será informado oportunamente, após a publicação do resultado final. O candidato deve acessar o sistema Sigfapes e inserir os documentos pessoais listados no Anexo VII.)
-?: Assinatura do Termo de Concessão de Bolsa (O cronograma do procedimento será informado oportunamente, após a publicação do resultado final. A assinatura é eletrônica via E-Docs/Acesso Cidadão.)</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>As bolsas e o auxílio-instalação serão pagas em reais (BRL) conforme conversão a ser realizada através do Conversor de Moedas do Banco Central do Brasil. Todo o custeio do curso, incluindo anuidades e taxas de matrícula, moradia, passagens, visto, transporte, acomodação, realização da pesquisa e outras despesas, é de responsabilidade exclusiva do beneficiário. Os aprovados podem ser elegíveis a se candidatar a descontos de 15% a 100% nas anuidades e taxas de matrícula de universidades conveniadas, e financiamento para custeio do curso no exterior, oferecidos pelo Instituto Trajetórias. A aprovação no processo seletivo não garante autorização automática de afastamento remunerado, que é um ato discricionário e condicionado a processo próprio e autorização do Governador. O curso de mestrado deve se enquadrar em áreas como transformação digital, políticas de inovação, sustentabilidade, desenvolvimento econômico regional, saúde pública, educação pública ou planejamento governamental. As universidades de excelência são aquelas entre os 100 primeiros colocados nos rankings QS World University Rankings ou Times Higher Education World University Rankings (edições de 2026). Há vedações específicas para participação, incluindo servidores em cargo em comissão, com licenças sem vencimentos nos últimos 2 anos, ou que não concluíram cursos anteriores. O beneficiário deve retornar ao Brasil e permanecer a serviço do Estado do Espírito Santo pelo prazo correspondente ao período de licenciamento, aplicando o conhecimento adquirido. O reconhecimento (revalidação) do título de mestrado obtido no exterior é de competência exclusiva do beneficiário e deve ocorrer em até 1 (um) ano após a conclusão do curso.</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_SERVIDORES_ES_22.05.2026.pdf</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>formacao_cientifica/EDITAL_FAPES_SEGER_No_14_2026_-_PROGRAMA_TALENTOS_GLOBAIS_ESPÍRITO_SANTO_-_MESTRADO_INTERNACIONAL_SERVIDORES_PÚBLICOS_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Formação Científica</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES/SECTI Nº 15/2026 - PROGRAMA TALENTOS GLOBAIS ESPÍRITO SANTO - MESTRADO INTERNACIONAL PÚBLICO GERAL 2026</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-01 a 2026-07-07: Interposição de recurso administrativo (Prazo de 05 (cinco) dias úteis após a divulgação do resultado preliminar. Interposto via formulário específico no Sistema E-Flow.)</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>O edital visa selecionar até 10 candidatos para cursos presenciais de mestrado stricto sensu em instituições estrangeiras de excelência, no âmbito do Programa Talentos Globais Espírito Santo – Mestrado Internacional. O programa busca estimular a mobilidade acadêmica internacional, apoiar a formação de recursos humanos altamente qualificados para o desenvolvimento do Estado e promover o retorno e aplicação do conhecimento adquirido no Brasil.</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Candidatos brasileiros, com graduação completa e diploma reconhecido no Brasil, residentes no Estado do Espírito Santo, que tenham iniciado processo de candidatura ou possuam carta de aceite/admissão em programa presencial de mestrado em universidade estrangeira de excelência nas áreas do conhecimento destacadas no edital.</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>US$ 500.000,00</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>US$ 30.000,00 a US$ 50.000,00</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>bolsas.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-25 a 2026-06-23: Submissão de candidatura (Prazo de submissão vence às 17h59min do dia 23/06/2026. Suporte e informações aos candidatos de 08h até às 18h (horário oficial de Brasília/DF).)
-2026-07-01 a 2026-07-07: Interposição de recurso administrativo (Prazo de 05 (cinco) dias úteis após a divulgação do resultado preliminar. Interposto via formulário específico no Sistema E-Flow.)</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>O edital prevê duas etapas de seleção: Habilitação e Análise de Mérito, conduzidas por um Comitê de Avaliação. As universidades estrangeiras de excelência são aquelas entre as 100 primeiras colocadas nos rankings QS World University Rankings ou Times Higher Education World University Rankings (edições de 2026). O custeio total do curso, incluindo anuidades, taxas, moradia, passagens e visto, é de responsabilidade exclusiva do beneficiário. Os aprovados podem ser elegíveis a descontos de 15% a 100% nas anuidades/taxas de universidades conveniadas e financiamento para custeio do curso, oferecidos pelo Instituto Trajetórias. O cronograma para a assinatura do Termo de Concessão de Bolsa será informado após a publicação do resultado final. O beneficiário se compromete a residir e atuar no Brasil pelo mesmo período de vigência da bolsa, aplicando o conhecimento adquirido em atividades de ensino, pesquisa, inovação, extensão, gestão pública ou iniciativas de impacto social e econômico no Estado do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Talentos_Globais_Secti_22.05.2026.pdf</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>formacao_cientifica/EDITAL_FAPES_SECTI_No_15_2026_-_PROGRAMA_TALENTOS_GLOBAIS_ESPÍRITO_SANTO_-_MESTRADO_INTERNACIONAL_PÚBLICO_GERAL_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 a 2026-07-24: Envio das inscrições - Categorias Projetos e Destaque (Até as 17h59, via SigFapes)</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, além de matérias jornalísticas relacionadas à Fapes ou a projetos por ela fomentados, visando valorizar a ciência, tecnologia e inovação e ampliar sua divulgação no Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos por ela fomentados.</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>R$ 308.000,00</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>R$ 12.000,00</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-07-24: Envio das inscrições - Categorias Projetos e Destaque (Até as 17h59, via SigFapes)
 2026-06-22 a 2026-09-15: Envio das inscrições - Categoria Jornalismo (Até as 17h59, via SigFapes)
@@ -843,70 +638,70 @@
 ?: Solicitação de pagamento da premiação (Prazo máximo de 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES, mediante abertura de processo eletrônico no sistema E-Flow, via E-Docs)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Não podem participar servidores da Fapes, membros do CCAF, cônjuges, companheiros e parentes até o segundo grau. É permitida apenas uma inscrição por pessoa. Os valores das premiações são brutos e sujeitos a IRRF, tendo caráter honorífico e não gerando vínculo empregatício. Solicitações de acessibilidade devem ser feitas com 10 dias de antecedência do prazo final de inscrição. O comparecimento à cerimônia de premiação é obrigatório, ou indicação de representante. Para a categoria Jornalismo, a matéria deve ter sido veiculada entre 01/09/2025 e 15/09/2026.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>2026-07-30: Contratação / Assinatura do TO e envio de documentos - 2ª Chamada (Até 30 dias após a publicação do resultado final homologado.)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
 2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
@@ -925,70 +720,70 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 12/2026 - EXTENSÃO TECNOLÓGICA</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Submissão de propostas (Até as 17h59 via Sigfapes)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas. Os projetos devem ser coordenados por profissionais vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) no Espírito Santo, visando o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, com foco na inclusão social e produtiva nas microrregiões do estado.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Profissionais (coordenadores de projeto) vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) públicas e privadas, localizadas no Espírito Santo, que possuam vínculo empregatício ou termo de adesão a trabalho voluntário, experiência em projetos de extensão ou titulação mínima de mestre, currículo Lattes atualizado, e que apresentem parceria com organização externa (empresa pública ou privada, cooperativa ou organização sem fins lucrativos).</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>R$ 60.000,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Submissão de propostas (Até as 17h59 via Sigfapes)
 2026-06-27 a 2026-07-03: Prazo para submissão de recursos administrativos da habilitação (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
@@ -997,70 +792,70 @@
 ?: Contratação de suplentes (Período a ser definido, se aplicável. Até as 17h00.)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução do projeto será de 24 meses. As propostas devem ser submetidas para desenvolvimento em apenas uma das 10 microrregiões listadas no Quadro 2. Serão apoiados 4 projetos por microrregião e 10 projetos na ampla concorrência. É obrigatória a permanência de no mínimo 1 bolsista EXT-E ou EXT-F a partir do 3º mês de vigência do projeto, pelo prazo mínimo de 22 meses. A soma dos serviços de terceiros é limitada a 30% do valor total do projeto aprovado (incluído DOACI). As despesas operacionais e administrativas (DOACI) são limitadas a 10% do valor total do projeto, descontados os valores de bolsa. Os valores destinados a diárias não poderão superar 50% do valor máximo permitido para o projeto. A proposta deve apresentar, pelo menos, uma parceria com organização externa. Cada proponente poderá ser coordenador de somente uma proposta. Propostas com Nota Final inferior a 70 pontos serão desclassificadas.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Extensão%20Tecnológica%20-%2012-2026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_12_2026_-_EXTENSÃO_TECNOLÓGICA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Submissão de propostas (Até as 17h59 via SigFapes)</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do estado.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com titulação mínima de mestre, experiência comprovada em projetos de extensão nos últimos 3 anos, e vínculo empregatício, estatutário, temporário ou voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo. O proponente não deve ter sido contratado no Edital Fapes nº 04/2025 nem solicitado prorrogação de projeto do Edital FAPES nº 02/2024.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 5.000.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>R$ 80.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-06-23: Prazo para impugnação do edital (Até 5 dias úteis antes da data limite de submissão das propostas)
 2026-06-30: Submissão de propostas (Até as 17h59 via SigFapes)
@@ -1069,66 +864,66 @@
 2026-10-29 a 2026-11-05: Início da contratação e envio de documentos (Até 5 dias úteis da publicação do resultado homologado para o início do processo de contratação. Inclui assinatura do Termo de Outorga e envio do Registro da Lista de Checagem de Documentação (e-Flow) até as 17h00.)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução dos projetos é de 24 meses. É obrigatória a previsão de pelo menos um bolsista EXT-E ou EXT-F por um período mínimo de 22 meses. As propostas devem ser submetidas para apenas uma das 10 microrregiões listadas no edital. Proponentes que declararem pertencimento a grupos de ações afirmativas (PcD, negra, quilombola, indígena, trans ou travesti) podem receber pontuação adicional. Propostas com nota final inferior a 70 pontos serão desclassificadas. É exigida a elaboração de um vídeo apresentando os resultados do projeto. É indispensável a menção explícita e destacada ao apoio da Fapes em todas as divulgações do trabalho.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -1142,70 +937,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
 2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h (horário de Brasília) via SIGFAPES)
@@ -1228,70 +1023,70 @@
 2027-05-04: Período de contratação de suplentes (2ª chamada) (Se aplicável, até as 17h00min)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital, sendo responsabilidade do proponente acompanhar as atualizações no site da FAPES. O edital poderá ser suspenso, revogado ou anulado por interesse público ou exigência legal, sem direito a indenização. O proponente deve manter seus dados cadastrais atualizados no SIGFAPES. A FAPES não exigirá direitos de participação e propriedade intelectual sobre as pesquisas e projetos, mas deverá ser notificada em caso de registro de propriedade intelectual. Os participantes concordam em ceder direitos de imagem para divulgação das ações da FAPES.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana, no Espírito Santo. Ele oferece apoio técnico e financeiro para soluções inovadoras com potencial de se tornarem negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação para o desenvolvimento sustentável.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central-Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 30.000,00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)
 ?: Prazo para recurso administrativo (Fase 1) (Até 5 dias úteis após divulgação do resultado preliminar)
@@ -1301,199 +1096,199 @@
 ?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>O edital será executado em duas fases. Na Fase 1, serão selecionadas 80 propostas de cada microrregião. Na Fase 2, serão selecionadas 25 propostas ou mais por microrregião. O valor total do edital de R$ 4.500.000,00 será distribuído entre as 6 microrregiões, com até R$ 750.000,00 para cada, visando financiar 25 projetos ou mais por microrregião. A participação em no mínimo 80% das oficinas e mentorias é obrigatória para o proponente ou membros da equipe, sob pena de desclassificação. Proponentes podem submeter mais de uma proposta na Fase 1, mas apenas a de maior nota avançará para a Fase 2. Propostas com nota final inferior a 70,0 serão desclassificadas. A Fapes pode alterar as datas e prazos do cronograma.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-26 10:07
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1115,60 +1123,76 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Chamadas Internacionais</t>
+          <t>Inovação</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 26/06/2026</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+          <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+          <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que tenham como objetivo celebrar parcerias estratégicas com outras startups do Espírito Santo, nacionais ou internacionais. O edital busca fomentar a expansão do mercado, inovação e avanço tecnológico, aprimoramento de produtos ou serviços, acesso a novos canais ou redes de distribuição, atração de talentos e aprimoramento de competências, posicionamento de marca e mercado, acesso a oportunidades de financiamento ou investimento, e impacto socioambiental sustentável.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
+          <t>Startups (pessoas jurídicas) sediadas no Espírito Santo, com faturamento bruto anual de até R$ 16.000.000,00 e até 10 anos de inscrição no Cadastro Nacional da Pessoa Jurídica (CNPJ).</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>R$ 9.800.000,00</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Varia de R$ 120.000,00 a R$ 250.000,00, dependendo da modalidade de parceria (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, e R$ 250.000,00 para Modalidade III).</t>
+        </is>
+      </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+          <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)
+?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar da habilitação. O recurso administrativo deverá ser interposto por meio do formulário específico disponível no Sistema de Automação de Fluxos do Governo do Estado (E-Flow): https://fapes.es.gov.br/formularios.)
+?: Constituição de empresa e atualização documental no SIGFAPES (Para proponentes aprovados. Prazo até as 17h. Abertura da empresa/anexar os documentos no SIGFAPES. Datas são placeholders no edital.)
+?: Assinatura do Termo de Outorga e do Projeto Aprovado (Para proponentes aprovados. Prazo até as 17h. Necessário cadastro no portal 'Acesso Cidadão' e no 'E-DOCS' do Governo do Estado (www.acessocidadao.es.gov.br). Datas são placeholders no edital.)
+?: Constituição de empresa e atualização documental no SIGFAPES (Suplentes) (Para suplentes. Prazo até as 17h. Datas são placeholders no edital.)
+?: Assinatura do Termo de Outorga e do Projeto Aprovado (Suplentes) (Para suplentes. Prazo até as 17h. Datas são placeholders no edital.)
+?: Abertura de conta corrente para recebimento de recursos (O(a) outorgado(a) terá o prazo de 30 (trinta) dias a partir do início da vigência do Termo de Outorga para informar à Fapes os dados da conta bancária aberta, a contar da data da publicação da contratação do projeto no DIO-ES. A conta deve ser aberta no Banco Banestes.)
+?: Prestação de contas parcial (Até 30 dias após o 12º mês de vigência do Termo de Outorga de Subvenção Econômica.)
+?: Prestação de contas final (Até 30 dias após o prazo de vigência do Termo de Outorga de Subvenção Econômica.)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
+          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. É permitido a cada proponente submeter até 2 (duas) propostas de parceria, desde que em modalidades diferentes e com diferentes parceiros. É vedada a submissão de propostas com as mesmas startups alternando funções de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A FAPES não exigirá direitos decorrentes de participação e propriedade nas pesquisas e projetos incentivados. A primeira parcela dos recursos será liberada após a assinatura do Termo de Outorga e comprovação do aporte da contrapartida financeira. A segunda parcela será liberada 30 dias após o 12º mês de execução, mediante prestação de contas parcial, comprovação de 70% de recursos comprometidos/executados e aporte da segunda parcela da contrapartida financeira.</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1204,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1190,18 +1214,18 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
         </is>
       </c>
       <c r="H11" s="2" t="n"/>
@@ -1213,22 +1237,22 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1264,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1248,47 +1272,107 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
+          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-27 09:07
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -38,7 +38,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -972,25 +972,32 @@
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 27/06/2026</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
+          <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (até as 17:59h, via Sigfapes)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica." → "Fomentar o empreendedorismo inovador por meio de projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou de processos inovadores. O edital visa transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica. Destina-se a doutores em qualquer área de desenvolvimento."
+Público-alvo: "Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba." → "Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras."
+Submissão (removida): Abertura de empresa e atualização documental (1ª chamada) — 2026-10-27 a 2026-11-03
+Submissão (removida): Abertura de empresa e atualização documental (2ª chamada) — 2027-04-27 a 2027-05-03</t>
+        </is>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica.</t>
+          <t>Fomentar o empreendedorismo inovador por meio de projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou de processos inovadores. O edital visa transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica. Destina-se a doutores em qualquer área de desenvolvimento.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
+          <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1010,30 +1017,19 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
-2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h (horário de Brasília) via SIGFAPES)
-2026-07-31 a 2026-08-06: Prazo para recursos administrativos da habilitação (1ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
-2026-10-02 a 2026-10-08: Prazo para recursos administrativos da avaliação de mérito (1ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
-2026-10-14 a 2026-12-15: Período de submissão de propostas (2ª chamada) (Até as 17:59h (horário de Brasília) via SIGFAPES)
-2026-10-27 a 2026-11-03: Período de contratação (1ª chamada) (Até 5 dias úteis da publicação do resultado homologado)
-2026-10-27 a 2026-11-03: Abertura de empresa e atualização documental (1ª chamada) (Para propostas aprovadas sem empresas constituídas, até as 17h00min)
-2026-10-27 a 2026-11-03: Atualização documental no SIGFAPES (1ª chamada) (Envio de documentos pessoais, até as 17h00min)
-2026-10-27 a 2026-11-03: Assinatura do Termo de Outorga e Projeto Aprovado (1ª chamada) (Eletronicamente via E-docs, até as 17h00min)
-2026-11-03: Envio do e-Flow (Formulário nº 25) e disponibilização de documentos no SIGFAPES (1ª chamada) (Até as 17h00min)
-2026-11-04: Período de contratação de suplentes (1ª chamada) (Se aplicável, até as 17h00min)
-2027-01-08 a 2027-01-14: Prazo para recursos administrativos da habilitação (2ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
-2027-03-19 a 2027-03-25: Prazo para recursos administrativos da avaliação de mérito (2ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
-2027-04-27 a 2027-05-03: Período de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)
-2027-04-27 a 2027-05-03: Abertura de empresa e atualização documental (2ª chamada) (Para propostas aprovadas sem empresas constituídas, até as 17h00min)
-2027-04-27 a 2027-05-03: Atualização documental no SIGFAPES (2ª chamada) (Envio de documentos pessoais, até as 17h00min)
-2027-04-27 a 2027-05-03: Assinatura do Termo de Outorga e Projeto Aprovado (2ª chamada) (Eletronicamente via E-docs, até as 17h00min)
-2027-05-03: Envio do e-Flow (Formulário nº 25) e disponibilização de documentos no SIGFAPES (2ª chamada) (Até as 17h00min)
-2027-05-04: Período de contratação de suplentes (2ª chamada) (Se aplicável, até as 17h00min)</t>
+          <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (até as 17:59h, via Sigfapes)
+2026-07-31 a 2026-08-06: Prazo de submissão de recursos administrativos (habilitação - 1ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)
+2026-10-02 a 2026-10-08: Prazo de submissão de recursos administrativos (mérito e apresentação oral - 1ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)
+2026-10-14 a 2026-12-15: Período de submissão de propostas (2ª chamada) (até as 17:59h, via Sigfapes)
+2026-10-27 a 2026-10-31: Processo de contratação (1ª chamada) (Até 5 dias úteis da publicação do resultado homologado)
+2027-01-08 a 2027-01-14: Prazo de submissão de recursos administrativos (habilitação - 2ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)
+2027-03-19 a 2027-03-25: Prazo de submissão de recursos administrativos (mérito e apresentação oral - 2ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)
+2027-04-27 a 2027-05-03: Processo de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital, sendo responsabilidade do proponente acompanhar as atualizações no site da FAPES. O edital poderá ser suspenso, revogado ou anulado por interesse público ou exigência legal, sem direito a indenização. O proponente deve manter seus dados cadastrais atualizados no SIGFAPES. A FAPES não exigirá direitos de participação e propriedade intelectual sobre as pesquisas e projetos, mas deverá ser notificada em caso de registro de propriedade intelectual. Os participantes concordam em ceder direitos de imagem para divulgação das ações da FAPES.</t>
+          <t>O edital prevê duas chamadas para submissão de propostas. Os recursos financeiros remanescentes da primeira chamada poderão ser aplicados na segunda. O prazo de execução dos projetos será de 24 meses, prorrogável por até 12 meses. A subvenção econômica inclui R$ 50.000,00 para serviços de consultoria especializada de aceleradoras. A contrapartida financeira dos outorgados será de 5% do valor subvencionado. A verificação de vínculo empregatício do proponente será realizada no ato da contratação. Para propostas onde a instituição copartícipe é uma ICT ou IES/P vinculada ao Edital FAPES nº 12/2025, o NIT deverá ser formalmente comunicado sobre a parceria, conforme Anexo IX. No ato da contratação, será exigida a apresentação da Declaração de Ciência do NIT, quando aplicável. A definição de responsabilidades quanto ao registro ou depósito de pedido de proteção intelectual caberá ao outorgado e à instituição/empresa executora, conforme suas normativas internas e legislação. O Anexo III (Declaração de Apoio da Instituição Copartícipe) agora permite assinatura por autoridade com competência formalmente delegada. Foi incluído o Anexo IX (Modelo de Declaração de Ciência do Núcleo de Inovação Tecnológica – NIT).</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1131,9 +1127,9 @@
           <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 26/06/2026</t>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-28 09:14
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -972,9 +964,9 @@
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 27/06/2026</t>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -982,14 +974,7 @@
           <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (até as 17:59h, via Sigfapes)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica." → "Fomentar o empreendedorismo inovador por meio de projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou de processos inovadores. O edital visa transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica. Destina-se a doutores em qualquer área de desenvolvimento."
-Público-alvo: "Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba." → "Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras."
-Submissão (removida): Abertura de empresa e atualização documental (1ª chamada) — 2026-10-27 a 2026-11-03
-Submissão (removida): Abertura de empresa e atualização documental (2ª chamada) — 2027-04-27 a 2027-05-03</t>
-        </is>
-      </c>
+      <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Fomentar o empreendedorismo inovador por meio de projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou de processos inovadores. O edital visa transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica. Destina-se a doutores em qualquer área de desenvolvimento.</t>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-01 10:34
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -754,7 +754,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30: Submissão de propostas (Até as 17h59 via Sigfapes)</t>
+          <t>2026-06-27 a 2026-07-03: Prazo para submissão de recursos administrativos da habilitação (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -826,7 +826,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30: Submissão de propostas (Até as 17h59 via SigFapes)</t>
+          <t>2026-08-01 a 2026-08-07: Prazo para submissão de recursos administrativos (Habilitação) (05 dias úteis a partir da publicação do resultado preliminar da habilitação)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)</t>
+          <t>2026-09-14 a 2026-09-22: Envio da segunda proposta (Fase 2) (até as 17h59)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-03 09:56
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -531,7 +539,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28 a 2026-07-02: Prazo para dúvidas e informações (Até 2 dias úteis antecedentes ao término da submissão das propostas.)</t>
+          <t>2026-07-06: Submissão das propostas (Até as 17h59.)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
@@ -739,12 +747,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Extensão</t>
+          <t>Inovação</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 12/2026 - EXTENSÃO TECNOLÓGICA</t>
+          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -752,178 +760,34 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-27 a 2026-07-03: Prazo para submissão de recursos administrativos da habilitação (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)</t>
-        </is>
-      </c>
+      <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas. Os projetos devem ser coordenados por profissionais vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) no Espírito Santo, visando o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, com foco na inclusão social e produtiva nas microrregiões do estado.</t>
+          <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Profissionais (coordenadores de projeto) vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) públicas e privadas, localizadas no Espírito Santo, que possuam vínculo empregatício ou termo de adesão a trabalho voluntário, experiência em projetos de extensão ou titulação mínima de mestre, currículo Lattes atualizado, e que apresentem parceria com organização externa (empresa pública ou privada, cooperativa ou organização sem fins lucrativos).</t>
+          <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
+          <t>R$ 40.000.000,00</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>R$ 60.000,00</t>
-        </is>
-      </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>editais.extensao@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-30: Submissão de propostas (Até as 17h59 via Sigfapes)
-2026-06-27 a 2026-07-03: Prazo para submissão de recursos administrativos da habilitação (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
-2026-09-26 a 2026-10-01: Prazo para submissão de recursos administrativos da análise de mérito (05 (cinco) dias úteis a partir da publicação do resultado preliminar do mérito)
-2026-10-28: Assinatura do Termo de Outorga e Projeto Aprovado (Proponentes aprovados devem assinar eletronicamente via E-Docs. Prazo para assinatura será divulgado junto ao resultado final homologado.)
-?: Contratação de suplentes (Período a ser definido, se aplicável. Até as 17h00.)</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>O prazo de execução do projeto será de 24 meses. As propostas devem ser submetidas para desenvolvimento em apenas uma das 10 microrregiões listadas no Quadro 2. Serão apoiados 4 projetos por microrregião e 10 projetos na ampla concorrência. É obrigatória a permanência de no mínimo 1 bolsista EXT-E ou EXT-F a partir do 3º mês de vigência do projeto, pelo prazo mínimo de 22 meses. A soma dos serviços de terceiros é limitada a 30% do valor total do projeto aprovado (incluído DOACI). As despesas operacionais e administrativas (DOACI) são limitadas a 10% do valor total do projeto, descontados os valores de bolsa. Os valores destinados a diárias não poderão superar 50% do valor máximo permitido para o projeto. A proposta deve apresentar, pelo menos, uma parceria com organização externa. Cada proponente poderá ser coordenador de somente uma proposta. Propostas com Nota Final inferior a 70 pontos serão desclassificadas.</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Extensão%20Tecnológica%20-%2012-2026%20-%20Assinado.pdf</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>extensao/EDITAL_FAPES_No_12_2026_-_EXTENSÃO_TECNOLÓGICA.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Extensão</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-01 a 2026-08-07: Prazo para submissão de recursos administrativos (Habilitação) (05 dias úteis a partir da publicação do resultado preliminar da habilitação)</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do estado.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores com titulação mínima de mestre, experiência comprovada em projetos de extensão nos últimos 3 anos, e vínculo empregatício, estatutário, temporário ou voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo. O proponente não deve ter sido contratado no Edital Fapes nº 04/2025 nem solicitado prorrogação de projeto do Edital FAPES nº 02/2024.</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>R$ 5.000.000,00</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>R$ 80.000,00</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>editais.extensao@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-23: Prazo para impugnação do edital (Até 5 dias úteis antes da data limite de submissão das propostas)
-2026-06-30: Submissão de propostas (Até as 17h59 via SigFapes)
-2026-08-01 a 2026-08-07: Prazo para submissão de recursos administrativos (Habilitação) (05 dias úteis a partir da publicação do resultado preliminar da habilitação)
-2026-10-05 a 2026-10-09: Prazo para submissão de recursos administrativos (Análise de Mérito) (05 dias úteis a partir da publicação do resultado preliminar do mérito)
-2026-10-29 a 2026-11-05: Início da contratação e envio de documentos (Até 5 dias úteis da publicação do resultado homologado para o início do processo de contratação. Inclui assinatura do Termo de Outorga e envio do Registro da Lista de Checagem de Documentação (e-Flow) até as 17h00.)</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>O prazo de execução dos projetos é de 24 meses. É obrigatória a previsão de pelo menos um bolsista EXT-E ou EXT-F por um período mínimo de 22 meses. As propostas devem ser submetidas para apenas uma das 10 microrregiões listadas no edital. Proponentes que declararem pertencimento a grupos de ações afirmativas (PcD, negra, quilombola, indígena, trans ou travesti) podem receber pontuação adicional. Propostas com nota final inferior a 70 pontos serão desclassificadas. É exigida a elaboração de um vídeo apresentando os resultados do projeto. É indispensável a menção explícita e destacada ao apoio da Fapes em todas as divulgações do trabalho.</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Inovação</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>R$ 40.000.000,00</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>R$ 3.000.000,00</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>duvidas.inovacao@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -937,70 +801,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (até as 17:59h, via Sigfapes)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Fomentar o empreendedorismo inovador por meio de projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou de processos inovadores. O edital visa transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica. Destina-se a doutores em qualquer área de desenvolvimento.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (até as 17:59h, via Sigfapes)
 2026-07-31 a 2026-08-06: Prazo de submissão de recursos administrativos (habilitação - 1ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)
@@ -1012,143 +876,152 @@
 2027-04-27 a 2027-05-03: Processo de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>O edital prevê duas chamadas para submissão de propostas. Os recursos financeiros remanescentes da primeira chamada poderão ser aplicados na segunda. O prazo de execução dos projetos será de 24 meses, prorrogável por até 12 meses. A subvenção econômica inclui R$ 50.000,00 para serviços de consultoria especializada de aceleradoras. A contrapartida financeira dos outorgados será de 5% do valor subvencionado. A verificação de vínculo empregatício do proponente será realizada no ato da contratação. Para propostas onde a instituição copartícipe é uma ICT ou IES/P vinculada ao Edital FAPES nº 12/2025, o NIT deverá ser formalmente comunicado sobre a parceria, conforme Anexo IX. No ato da contratação, será exigida a apresentação da Declaração de Ciência do NIT, quando aplicável. A definição de responsabilidades quanto ao registro ou depósito de pedido de proteção intelectual caberá ao outorgado e à instituição/empresa executora, conforme suas normativas internas e legislação. O Anexo III (Declaração de Apoio da Instituição Copartícipe) agora permite assinatura por autoridade com competência formalmente delegada. Foi incluído o Anexo IX (Modelo de Declaração de Ciência do Núcleo de Inovação Tecnológica – NIT).</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14 a 2026-09-22: Envio da segunda proposta (Fase 2) (até as 17h59)</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana, no Espírito Santo. Ele oferece apoio técnico e financeiro para soluções inovadoras com potencial de se tornarem negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação para o desenvolvimento sustentável.</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central-Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 03/07/2026</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 a 2026-07-03: Envio da primeira proposta (até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana, no Espírito Santo. Ele oferece apoio técnico e financeiro para soluções inovadoras com potencial de se tornarem negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação para o desenvolvimento sustentável." → "O presente edital tem como objetivo geral estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. Isso será feito por meio de apoio técnico e financeiro a soluções inovadoras com potencial para se transformarem em negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação. O edital visa estimular a criação, formalização e fortalecimento de negócios, promovendo a inovação e o empreendedorismo como estratégias para o desenvolvimento sustentável."
+Público-alvo: "Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central-Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias." → "Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias."
+Contato: "duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br" → "duvidas.inovacao@fapes.es.gov.br, comunicacao@fapes.es.gov.br, (27) 3636-1850, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br"
+Submissão (nova): Envio da primeira proposta — 2026-05-21 a 2026-07-03
+Submissão (removida): Envio da primeira proposta (Fase 1) — 2026-05-21 a 2026-06-30</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>O presente edital tem como objetivo geral estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. Isso será feito por meio de apoio técnico e financeiro a soluções inovadoras com potencial para se transformarem em negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação. O edital visa estimular a criação, formalização e fortalecimento de negócios, promovendo a inovação e o empreendedorismo como estratégias para o desenvolvimento sustentável.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>R$ 30.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>duvidas.inovacao@fapes.es.gov.br, comunicacao@fapes.es.gov.br, (27) 3636-1850, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 a 2026-06-26: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)
+2026-05-21 a 2026-07-03: Envio da primeira proposta (até as 17h59)
 ?: Prazo para recurso administrativo (Fase 1) (Até 5 dias úteis após divulgação do resultado preliminar)
-2026-09-14 a 2026-09-22: Envio da segunda proposta (Fase 2) (até as 17h59)
-2026-09-21 a 2026-09-30: Apresentação do pitch (A partir de 21/09/2026)
+2026-09-14 a 2026-09-22: Envio da segunda proposta após a 1ª oficina e capacitação (até as 17h59)
+2026-09-21 a 2026-09-30: Apresentação do pitch
 ?: Prazo para recurso administrativo (Fase 2) (Até 5 dias úteis após divulgação do resultado preliminar)
 ?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>O edital será executado em duas fases. Na Fase 1, serão selecionadas 80 propostas de cada microrregião. Na Fase 2, serão selecionadas 25 propostas ou mais por microrregião. O valor total do edital de R$ 4.500.000,00 será distribuído entre as 6 microrregiões, com até R$ 750.000,00 para cada, visando financiar 25 projetos ou mais por microrregião. A participação em no mínimo 80% das oficinas e mentorias é obrigatória para o proponente ou membros da equipe, sob pena de desclassificação. Proponentes podem submeter mais de uma proposta na Fase 1, mas apenas a de maior nota avançará para a Fase 2. Propostas com nota final inferior a 70,0 serão desclassificadas. A Fapes pode alterar as datas e prazos do cronograma.</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Serão selecionadas 80 propostas de cada microrregião na Fase 1. Serão selecionadas 25 propostas ou mais por microrregião na Fase 2. A Fapes pode alterar as datas e os prazos definidos no cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas. O proponente poderá submeter mais de uma proposta na Fase 1, mas apenas a de maior nota será selecionada para a Fase 2, caso haja múltiplas propostas classificadas. Propostas com Nota Final inferior a 70,0 pontos serão desclassificadas em ambas as fases.</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que tenham como objetivo celebrar parcerias estratégicas com outras startups do Espírito Santo, nacionais ou internacionais. O edital busca fomentar a expansão do mercado, inovação e avanço tecnológico, aprimoramento de produtos ou serviços, acesso a novos canais ou redes de distribuição, atração de talentos e aprimoramento de competências, posicionamento de marca e mercado, acesso a oportunidades de financiamento ou investimento, e impacto socioambiental sustentável.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Startups (pessoas jurídicas) sediadas no Espírito Santo, com faturamento bruto anual de até R$ 16.000.000,00 e até 10 anos de inscrição no Cadastro Nacional da Pessoa Jurídica (CNPJ).</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 9.800.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Varia de R$ 120.000,00 a R$ 250.000,00, dependendo da modalidade de parceria (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, e R$ 250.000,00 para Modalidade III).</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)
 ?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar da habilitação. O recurso administrativo deverá ser interposto por meio do formulário específico disponível no Sistema de Automação de Fluxos do Governo do Estado (E-Flow): https://fapes.es.gov.br/formularios.)
@@ -1161,19 +1034,139 @@
 ?: Prestação de contas final (Até 30 dias após o prazo de vigência do Termo de Outorga de Subvenção Econômica.)</t>
         </is>
       </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. É permitido a cada proponente submeter até 2 (duas) propostas de parceria, desde que em modalidades diferentes e com diferentes parceiros. É vedada a submissão de propostas com as mesmas startups alternando funções de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A FAPES não exigirá direitos decorrentes de participação e propriedade nas pesquisas e projetos incentivados. A primeira parcela dos recursos será liberada após a assinatura do Termo de Outorga e comprovação do aporte da contrapartida financeira. A segunda parcela será liberada 30 dias após o 12º mês de execução, mediante prestação de contas parcial, comprovação de 70% de recursos comprometidos/executados e aporte da segunda parcela da contrapartida financeira.</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA ERC-CONFAP 2026</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. É permitido a cada proponente submeter até 2 (duas) propostas de parceria, desde que em modalidades diferentes e com diferentes parceiros. É vedada a submissão de propostas com as mesmas startups alternando funções de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A FAPES não exigirá direitos decorrentes de participação e propriedade nas pesquisas e projetos incentivados. A primeira parcela dos recursos será liberada após a assinatura do Termo de Outorga e comprovação do aporte da contrapartida financeira. A segunda parcela será liberada 30 dias após o 12º mês de execução, mediante prestação de contas parcial, comprovação de 70% de recursos comprometidos/executados e aporte da segunda parcela da contrapartida financeira.</t>
+          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1178,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1193,167 +1186,47 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
+      <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
       <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="n"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>€ 25.000,00 por ano de projeto</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA HORIZON EUROPE</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>€ 25.000,00 por ano de projeto</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-04 09:03
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -747,47 +747,121 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>Extensão</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 04/07/2026</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do estado." → "Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo, visando a redução de desigualdades ou vulnerabilidades sociais e a promoção do desenvolvimento socioambiental e econômico nas microrregiões do estado."
+Público-alvo: "Pesquisadores com titulação mínima de mestre, experiência comprovada em projetos de extensão nos últimos 3 anos, e vínculo empregatício, estatutário, temporário ou voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo. O proponente não deve ter sido contratado no Edital Fapes nº 04/2025 nem solicitado prorrogação de projeto do Edital FAPES nº 02/2024." → "Profissionais com graduação e experiência mínima de 3 anos em projetos de extensão ou titulação mínima de mestre, com vínculo empregatício, estatutário, por designação temporária ou termo de adesão a trabalho voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, e que residam no Espírito Santo ou municípios limítrofes."
+Submissão (nova): Data limite para submissão das propostas no Sigfapes — ? a 2026-07-02
+Submissão (removida): Submissão de propostas — ? a 2026-06-30</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo, visando a redução de desigualdades ou vulnerabilidades sociais e a promoção do desenvolvimento socioambiental e econômico nas microrregiões do estado.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Profissionais com graduação e experiência mínima de 3 anos em projetos de extensão ou titulação mínima de mestre, com vínculo empregatício, estatutário, por designação temporária ou termo de adesão a trabalho voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, e que residam no Espírito Santo ou municípios limítrofes.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>R$ 5.000.000,00</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>R$ 80.000,00</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>editais.extensao@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02: Data limite para submissão das propostas no Sigfapes (Até as 17h59)
+?: Prazo para submissão de recursos administrativos (habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
+?: Prazo para submissão de recursos administrativos (mérito) (05 (cinco) dias úteis a partir da publicação do resultado preliminar do mérito)
+?: Início da contratação (Até 5 (cinco) dias úteis da publicação do resultado homologado para o início do processo de contratação)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>O prazo de execução dos projetos é de 24 meses. É obrigatória a previsão de bolsas Ext-E ou Ext-F por um período mínimo de 22 meses. As propostas devem ser submetidas para desenvolvimento em apenas uma das 10 microrregiões listadas no Quadro 2 do edital. Será concedida pontuação adicional para propostas apresentadas por pessoas pertencentes a grupos de ações afirmativas (PcD, negra, quilombola, indígena, trans ou travesti). Propostas com nota final inferior a 70 pontos serão desclassificadas.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -801,70 +875,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (até as 17:59h, via Sigfapes)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Fomentar o empreendedorismo inovador por meio de projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou de processos inovadores. O edital visa transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica. Destina-se a doutores em qualquer área de desenvolvimento.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (até as 17:59h, via Sigfapes)
 2026-07-31 a 2026-08-06: Prazo de submissão de recursos administrativos (habilitação - 1ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)
@@ -876,78 +950,70 @@
 2027-04-27 a 2027-05-03: Processo de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>O edital prevê duas chamadas para submissão de propostas. Os recursos financeiros remanescentes da primeira chamada poderão ser aplicados na segunda. O prazo de execução dos projetos será de 24 meses, prorrogável por até 12 meses. A subvenção econômica inclui R$ 50.000,00 para serviços de consultoria especializada de aceleradoras. A contrapartida financeira dos outorgados será de 5% do valor subvencionado. A verificação de vínculo empregatício do proponente será realizada no ato da contratação. Para propostas onde a instituição copartícipe é uma ICT ou IES/P vinculada ao Edital FAPES nº 12/2025, o NIT deverá ser formalmente comunicado sobre a parceria, conforme Anexo IX. No ato da contratação, será exigida a apresentação da Declaração de Ciência do NIT, quando aplicável. A definição de responsabilidades quanto ao registro ou depósito de pedido de proteção intelectual caberá ao outorgado e à instituição/empresa executora, conforme suas normativas internas e legislação. O Anexo III (Declaração de Apoio da Instituição Copartícipe) agora permite assinatura por autoridade com competência formalmente delegada. Foi incluído o Anexo IX (Modelo de Declaração de Ciência do Núcleo de Inovação Tecnológica – NIT).</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 03/07/2026</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-21 a 2026-07-03: Envio da primeira proposta (até as 17h59)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana, no Espírito Santo. Ele oferece apoio técnico e financeiro para soluções inovadoras com potencial de se tornarem negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação para o desenvolvimento sustentável." → "O presente edital tem como objetivo geral estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. Isso será feito por meio de apoio técnico e financeiro a soluções inovadoras com potencial para se transformarem em negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação. O edital visa estimular a criação, formalização e fortalecimento de negócios, promovendo a inovação e o empreendedorismo como estratégias para o desenvolvimento sustentável."
-Público-alvo: "Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central-Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias." → "Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias."
-Contato: "duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br" → "duvidas.inovacao@fapes.es.gov.br, comunicacao@fapes.es.gov.br, (27) 3636-1850, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br"
-Submissão (nova): Envio da primeira proposta — 2026-05-21 a 2026-07-03
-Submissão (removida): Envio da primeira proposta (Fase 1) — 2026-05-21 a 2026-06-30</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14 a 2026-09-22: Envio da segunda proposta após a 1ª oficina e capacitação (até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>O presente edital tem como objetivo geral estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. Isso será feito por meio de apoio técnico e financeiro a soluções inovadoras com potencial para se transformarem em negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação. O edital visa estimular a criação, formalização e fortalecimento de negócios, promovendo a inovação e o empreendedorismo como estratégias para o desenvolvimento sustentável.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>R$ 30.000,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, comunicacao@fapes.es.gov.br, (27) 3636-1850, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-26: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)
 2026-05-21 a 2026-07-03: Envio da primeira proposta (até as 17h59)
@@ -958,70 +1024,70 @@
 ?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Serão selecionadas 80 propostas de cada microrregião na Fase 1. Serão selecionadas 25 propostas ou mais por microrregião na Fase 2. A Fapes pode alterar as datas e os prazos definidos no cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas. O proponente poderá submeter mais de uma proposta na Fase 1, mas apenas a de maior nota será selecionada para a Fase 2, caso haja múltiplas propostas classificadas. Propostas com Nota Final inferior a 70,0 pontos serão desclassificadas em ambas as fases.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que tenham como objetivo celebrar parcerias estratégicas com outras startups do Espírito Santo, nacionais ou internacionais. O edital busca fomentar a expansão do mercado, inovação e avanço tecnológico, aprimoramento de produtos ou serviços, acesso a novos canais ou redes de distribuição, atração de talentos e aprimoramento de competências, posicionamento de marca e mercado, acesso a oportunidades de financiamento ou investimento, e impacto socioambiental sustentável.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Startups (pessoas jurídicas) sediadas no Espírito Santo, com faturamento bruto anual de até R$ 16.000.000,00 e até 10 anos de inscrição no Cadastro Nacional da Pessoa Jurídica (CNPJ).</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 9.800.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Varia de R$ 120.000,00 a R$ 250.000,00, dependendo da modalidade de parceria (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, e R$ 250.000,00 para Modalidade III).</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)
 ?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar da habilitação. O recurso administrativo deverá ser interposto por meio do formulário específico disponível no Sistema de Automação de Fluxos do Governo do Estado (E-Flow): https://fapes.es.gov.br/formularios.)
@@ -1034,79 +1100,19 @@
 ?: Prestação de contas final (Até 30 dias após o prazo de vigência do Termo de Outorga de Subvenção Econômica.)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. É permitido a cada proponente submeter até 2 (duas) propostas de parceria, desde que em modalidades diferentes e com diferentes parceiros. É vedada a submissão de propostas com as mesmas startups alternando funções de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A FAPES não exigirá direitos decorrentes de participação e propriedade nas pesquisas e projetos incentivados. A primeira parcela dos recursos será liberada após a assinatura do Termo de Outorga e comprovação do aporte da contrapartida financeira. A segunda parcela será liberada 30 dias após o 12º mês de execução, mediante prestação de contas parcial, comprovação de 70% de recursos comprometidos/executados e aporte da segunda parcela da contrapartida financeira.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="n"/>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1118,7 +1124,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1128,18 +1134,18 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
         </is>
       </c>
       <c r="H10" s="2" t="n"/>
@@ -1151,22 +1157,22 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1184,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1186,47 +1192,107 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
+          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-05 09:11
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -755,20 +747,13 @@
           <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 04/07/2026</t>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do estado." → "Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo, visando a redução de desigualdades ou vulnerabilidades sociais e a promoção do desenvolvimento socioambiental e econômico nas microrregiões do estado."
-Público-alvo: "Pesquisadores com titulação mínima de mestre, experiência comprovada em projetos de extensão nos últimos 3 anos, e vínculo empregatício, estatutário, temporário ou voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo. O proponente não deve ter sido contratado no Edital Fapes nº 04/2025 nem solicitado prorrogação de projeto do Edital FAPES nº 02/2024." → "Profissionais com graduação e experiência mínima de 3 anos em projetos de extensão ou titulação mínima de mestre, com vínculo empregatício, estatutário, por designação temporária ou termo de adesão a trabalho voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, e que residam no Espírito Santo ou municípios limítrofes."
-Submissão (nova): Data limite para submissão das propostas no Sigfapes — ? a 2026-07-02
-Submissão (removida): Submissão de propostas — ? a 2026-06-30</t>
-        </is>
-      </c>
+      <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo, visando a redução de desigualdades ou vulnerabilidades sociais e a promoção do desenvolvimento socioambiental e econômico nas microrregiões do estado.</t>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-07 10:16
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,22 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +59,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -531,7 +547,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06: Submissão das propostas (Até as 17h59.)</t>
+          <t>2026-07-28 a 2026-08-03: Prazo para recurso (habilitação) (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação.)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
@@ -1109,55 +1125,47 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 07/07/2026</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+          <t>Apoiar a manutenção da bolsa de doutorado da FAPES para bolsistas aprovados na seleção do DAAD. O objetivo é permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, garantindo a continuidade do suporte financeiro durante o período de intercâmbio.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+          <t>Bolsistas de doutorado da FAPES que foram selecionados pelo DAAD, que estão adimplentes com a FAPES e que não estão no primeiro nem no último ano do doutorado.</t>
         </is>
       </c>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
+          <t>Para acesso ao conteúdo completo da chamada, consultar o site do CONFAP através do link: https://news.confap.org.br/daad-lanca-chamada-de-2026-do-programa-de-auxilio-para-doutorandos-brasileiros-com-bolsa-nacional/. As propostas devem ser submetidas na Plataforma do DAAD, e a FAPES realizará o controle de elegibilidade dos selecionados pelo DAAD.</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1177,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1179,18 +1187,18 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
         </is>
       </c>
       <c r="H11" s="2" t="n"/>
@@ -1202,22 +1210,22 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1229,55 +1237,134 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
+          <t>CHAMADA ERC-CONFAP 2026</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 07/07/2026</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos." → "Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo."
+Público-alvo: "Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros." → "Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes."
+Valor total: "-" → "US$ 18.000,00"
+Valor por proposta: "-" → "US$ 6.000,00"
+Contato: "internacional.confap@gmail.com" → "internacional.confap@gmail.com, global@fapes.es.gov.br"
+Submissão (nova): Submissão de propostas (CONFAP) — ? a 2026-08-10
+Submissão (removida): Submissao de propostas — ? a 2026-07-10</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
+2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
           <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-08 09:17
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -606,46 +606,359 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
+          <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Sem alteracoes</t>
+          <t>Removido (nao mais aberto)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 a 2026-07-24: Envio das inscrições - Categorias Projetos e Destaque (Até as 17h59, via SigFapes)</t>
+          <t>2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>O objetivo geral deste edital é selecionar e apoiar financeiramente pesquisadores e alunos para participação em eventos técnico-científicos de curta duração. Visa divulgar os resultados de projetos de pesquisa, desenvolvimento e inovação (P, D&amp;I) desenvolvidos em instituições de ensino superior e/ou pesquisa, públicas ou privadas, localizadas no Estado do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores e alunos de pós-graduação vinculados a Instituição de Ensino e/ou Pesquisa (IES/P), pública ou privada, localizada no estado do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>R$ 2.500.000,00</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>US$ 2.700,00</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-27: Prazo para solicitação de atendimento especializado (até 10 dias antes do prazo final de submissão da 1ª Chamada)
+2026-03-02: Prazo para impugnação do edital (até 5 dias úteis antes do prazo final de submissão da 1ª Chamada)
+2026-02-06 a 2026-03-09: Período de submissão (1ª Chamada) (eventos com início entre 01/05/2026 a 31/07/2026, até as 17h59)
+2026-03-07: Prazo para envio de dúvidas (1ª Chamada) (até 2 dias antes do prazo final de submissão da 1ª Chamada)
+2026-03-26: Prazo para interposição de recursos (1ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 1ª Chamada)
+2026-03-17 a 2026-04-24: Período de submissão (2ª Chamada) (eventos com início entre 01/08/2026 a 31/12/2026)
+2026-04-22: Prazo para envio de dúvidas (2ª Chamada) (até 2 dias antes do prazo final de submissão da 2ª Chamada)
+2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 2ª Chamada)
+2026-07-01 a 2026-08-20: Período de submissão (3ª Chamada) (eventos com início entre 04/01/2027 a 30/04/2027)
+2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)
+2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 3ª Chamada)</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>O valor total do edital será distribuído em três chamadas. O valor por proposta é fixo e varia conforme o local do evento: R$ 1.800,00 para eventos no Brasil (exceto Espírito Santo), US$ 1.400,00 para América Central ou América do Sul, US$ 2.300,00 para América do Norte e US$ 2.700,00 para outros continentes. A Fapes pode alterar as datas e prazos do cronograma. Cada proponente pode apresentar apenas uma proposta por chamada. O prazo para informar dados bancários é de até 30 dias corridos após o início da vigência do Termo de Outorga. O prazo para envio da prestação de contas é de até 30 dias após o término da vigência do Termo de Outorga. A contratação das propostas aprovadas ocorrerá em até 30 dias após a publicação do resultado final homologado. O envio do comprovante de aceite do trabalho é condicional para o repasse do recurso e deve ser feito até 15 dias antes do evento.</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_02-2026-Participação_Evento_Técnico_Científico.pdf</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_02_2026_-_PARTICIPAÇÃO_EM_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 03/2026 - ORGANIZAÇÃO DE EVENTOS TÉCNICO-CIENTÍFICOS</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Removido (nao mais aberto)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 3ª chamada)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Este edital visa selecionar propostas para conceder apoio financeiro a pesquisadores de nível superior. O objetivo é fomentar a organização de eventos técnico-científicos de curta duração, como congressos, simpósios e seminários, a serem realizados no Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores de nível superior vinculados a Instituição de Ensino Superior e/ou Pesquisa (IES/P), pública ou privada sem fins lucrativos, localizada no estado do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>R$ 2.500.000,00</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Varia de R$ 10.000,00 a R$ 35.000,00</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-02: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada)
+2026-02-06 a 2026-03-09: 1ª Chamada - Período de submissão de propostas (Eventos com início entre 01/05/2026 a 31/07/2026, até 17h59)
+2026-03-07: 1ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 1ª chamada)
+2026-03-20 a 2026-03-26: 1ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)
+2026-03-17 a 2026-04-24: 2ª Chamada - Período de submissão de propostas (Eventos com início entre 01/08/2026 a 31/12/2026)
+2026-04-22: 2ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 2ª chamada)
+2026-05-23 a 2026-05-29: 2ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)
+2026-07-01 a 2026-08-20: 3ª Chamada - Período de submissão de propostas (Eventos com início entre 04/01/2027 a 30/04/2027)
+2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 3ª chamada)
+2026-10-03 a 2026-10-09: 3ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)
+?: Contratação das propostas aprovadas (Até 30 dias após a publicação do resultado final homologado para cada chamada. As datas exatas serão publicadas posteriormente.)</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>O valor do auxílio financeiro é fixo e varia de acordo com o nível do evento: R$ 10.000,00 para Estadual/Regional, R$ 20.000,00 para Nacional e R$ 35.000,00 para Internacional. A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional. Cada proponente pode apresentar apenas uma proposta por chamada. Caso envie mais de uma, será considerada apenas a última enviada. O proponente que já tiver sido contratado neste edital não poderá submeter nova proposta. O evento deve ter duração máxima de 15 dias, consecutivos ou não, e ser chancelado por entidade/sociedade conforme o nível do evento (nacional ou internacional). Os recursos financeiros estão distribuídos por chamada e nível de evento, com possibilidade de remanejamento de saldos não utilizados entre níveis e chamadas subsequentes. É obrigatório mencionar o apoio da Fapes em todas as publicações e divulgações relacionadas ao projeto. A data de início do apoio poderá ser adiada, após a contratação, em até 12 meses, mediante justificativa.</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_03_2026_Organização_Eventos_Técnico-Científicos.pdf</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_03_2026_-_ORGANIZAÇÃO_DE_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO CIENTÍFICO</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Removido (nao mais aberto)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19 a 2026-07-19: Período de Contratação (2ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 01/08/2026 a 31/12/2026.)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Selecionar propostas para concessão de auxílio financeiro para a realização de estágio técnico-científico. O estágio pode ser em laboratório ou centro de pesquisa, desenvolvimento ou inovação (PD&amp;I), no país ou no exterior. O objetivo é aprimorar/desenvolver técnicas e processos, além de adquirir conhecimentos específicos vinculados a projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P), públicas ou privadas, localizadas no estado do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P pública ou privada, localizada no estado do Espírito Santo. Alunos regularmente matriculados em curso de Mestrado ou Doutorado de IES/P localizada no Espírito Santo e recomendado pela CAPES.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>R$ 2.000.000,00</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>R$ 10.000,00</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09 a 2026-03-12: Período de submissão de propostas (1ª Chamada) (Para estágios com início entre 01/05/2026 a 31/07/2026, até as 17h59.)
+2026-03-10: Prazo final para envio de dúvidas (1ª Chamada) (Até 2 dias antes do prazo final de submissão. Para estágios com início entre 01/05/2026 a 31/07/2026.)
+2026-03-17 a 2026-04-24: Período de submissão de propostas (2ª Chamada) (Para estágios com início entre 01/08/2026 a 31/12/2026.)
+2026-03-26: Prazo para interposição de recursos (1ª Chamada) (5 dias úteis após a publicação do resultado preliminar. Para estágios com início entre 01/05/2026 a 31/07/2026.)
+2026-03-31 a 2026-04-30: Período de Contratação (1ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 01/05/2026 a 31/07/2026.)
+2026-04-22: Prazo final para envio de dúvidas (2ª Chamada) (Até 2 dias antes do prazo final de submissão. Para estágios com início entre 01/08/2026 a 31/12/2026.)
+2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar. Para estágios com início entre 01/08/2026 a 31/12/2026.)
+2026-06-19 a 2026-07-19: Período de Contratação (2ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 01/08/2026 a 31/12/2026.)
+2026-07-01 a 2026-08-20: Período de submissão de propostas (3ª Chamada) (Para estágios com início entre 04/01/2027 a 30/04/2027.)
+2026-08-13: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas da última chamada.)
+2026-08-18: Prazo final para envio de dúvidas (3ª Chamada) (Até 2 dias antes do prazo final de submissão. Para estágios com início entre 04/01/2027 a 30/04/2027.)
+2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar. Para estágios com início entre 04/01/2027 a 30/04/2027.)
+2026-10-26 a 2026-11-25: Período de Contratação (3ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 04/01/2027 a 30/04/2027.)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas nas plataformas. Cada proponente pode apresentar apenas uma proposta por chamada. Não é permitida a contratação concomitante de projeto de estágio técnico-científico e visita técnico-científica para o mesmo período/chamada. O coordenador pode solicitar o adiamento da data de início do estágio por até 30 dias após a contratação, mediante justificativa. É obrigatório mencionar o apoio da Fapes em todas as publicações ou divulgações relacionadas ao projeto.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_04_2026_-_Estágio_Técnico_Cientifico.pdf</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_04_2026_-_ESTÁGIO_TÉCNICO_CIENTÍFICO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Removido (nao mais aberto)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Selecionar propostas para concessão de auxílio financeiro para a realização de visitas técnico-científicas em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, processos e adquirir conhecimentos específicos para projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas no Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>R$ 2.000.000,00</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>US$ 2.600,00</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09 a 2026-03-12: Submissão de propostas (1ª Chamada) (Até as 17h59. Para visitas com início entre 01/05/2026 a 31/07/2026.)
+2026-03-05: Prazo final para impugnação do edital (Até o quinto dia útil que anteceder o prazo final de submissão da 1ª Chamada.)
+2026-03-10: Prazo para envio de dúvidas sobre o edital (1ª Chamada) (Até 2 dias antes do prazo final de submissão.)
+2026-03-17 a 2026-04-24: Submissão de propostas (2ª Chamada) (Para visitas com início entre 01/08/2026 a 31/12/2026.)
+2026-03-26: Prazo para interposição de recursos (1ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)
+2026-04-22: Prazo para envio de dúvidas sobre o edital (2ª Chamada) (Até 2 dias antes do prazo final de submissão.)
+2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)
+2026-07-01 a 2026-08-20: Submissão de propostas (3ª Chamada) (Para visitas com início entre 04/01/2027 a 30/04/2027.)
+2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)
+2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade institucional, podendo reabrir prazos em casos de força maior ou falhas de sistema, com publicidade das alterações. Cada proponente pode submeter apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Proponentes já contratados neste edital não poderão submeter nova proposta. Após a contratação, o beneficiário pode solicitar adiamento da data de início da visita por até 30 dias, mediante justificativa e autorização. Não será permitida a alteração da instituição de destino da visita técnico-científica após a contratação.</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2005_2026%20-%20Visita%20Técnico%20Cientifica%20(1).pdf</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_05_2026_-_VISITA_TÉCNICO-CIENTÍFICA.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22 a 2026-07-24: Envio das inscrições - Categorias Projetos e Destaque (Até as 17h59, via SigFapes)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>Reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, além de matérias jornalísticas relacionadas à Fapes ou a projetos por ela fomentados, visando valorizar a ciência, tecnologia e inovação e ampliar sua divulgação no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos por ela fomentados.</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 308.000,00</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000,00</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-07-24: Envio das inscrições - Categorias Projetos e Destaque (Até as 17h59, via SigFapes)
 2026-06-22 a 2026-09-15: Envio das inscrições - Categoria Jornalismo (Até as 17h59, via SigFapes)
@@ -654,70 +967,70 @@
 ?: Solicitação de pagamento da premiação (Prazo máximo de 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES, mediante abertura de processo eletrônico no sistema E-Flow, via E-Docs)</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Não podem participar servidores da Fapes, membros do CCAF, cônjuges, companheiros e parentes até o segundo grau. É permitida apenas uma inscrição por pessoa. Os valores das premiações são brutos e sujeitos a IRRF, tendo caráter honorífico e não gerando vínculo empregatício. Solicitações de acessibilidade devem ser feitas com 10 dias de antecedência do prazo final de inscrição. O comparecimento à cerimônia de premiação é obrigatório, ou indicação de representante. Para a categoria Jornalismo, a matéria deve ter sido veiculada entre 01/09/2025 e 15/09/2026.</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-07-30: Contratação / Assinatura do TO e envio de documentos - 2ª Chamada (Até 30 dias após a publicação do resultado final homologado.)</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
 2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
@@ -736,66 +1049,66 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo, visando a redução de desigualdades ou vulnerabilidades sociais e a promoção do desenvolvimento socioambiental e econômico nas microrregiões do estado.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Profissionais com graduação e experiência mínima de 3 anos em projetos de extensão ou titulação mínima de mestre, com vínculo empregatício, estatutário, por designação temporária ou termo de adesão a trabalho voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, e que residam no Espírito Santo ou municípios limítrofes.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 5.000.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 80.000,00</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-07-02: Data limite para submissão das propostas no Sigfapes (Até as 17h59)
 ?: Prazo para submissão de recursos administrativos (habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
@@ -803,66 +1116,66 @@
 ?: Início da contratação (Até 5 (cinco) dias úteis da publicação do resultado homologado para o início do processo de contratação)</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução dos projetos é de 24 meses. É obrigatória a previsão de bolsas Ext-E ou Ext-F por um período mínimo de 22 meses. As propostas devem ser submetidas para desenvolvimento em apenas uma das 10 microrregiões listadas no Quadro 2 do edital. Será concedida pontuação adicional para propostas apresentadas por pessoas pertencentes a grupos de ações afirmativas (PcD, negra, quilombola, indígena, trans ou travesti). Propostas com nota final inferior a 70 pontos serão desclassificadas.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -876,70 +1189,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (até as 17:59h, via Sigfapes)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-31 a 2026-08-06: Prazo de submissão de recursos administrativos (habilitação - 1ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Fomentar o empreendedorismo inovador por meio de projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou de processos inovadores. O edital visa transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica. Destina-se a doutores em qualquer área de desenvolvimento.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (até as 17:59h, via Sigfapes)
 2026-07-31 a 2026-08-06: Prazo de submissão de recursos administrativos (habilitação - 1ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)
@@ -951,70 +1264,70 @@
 2027-04-27 a 2027-05-03: Processo de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>O edital prevê duas chamadas para submissão de propostas. Os recursos financeiros remanescentes da primeira chamada poderão ser aplicados na segunda. O prazo de execução dos projetos será de 24 meses, prorrogável por até 12 meses. A subvenção econômica inclui R$ 50.000,00 para serviços de consultoria especializada de aceleradoras. A contrapartida financeira dos outorgados será de 5% do valor subvencionado. A verificação de vínculo empregatício do proponente será realizada no ato da contratação. Para propostas onde a instituição copartícipe é uma ICT ou IES/P vinculada ao Edital FAPES nº 12/2025, o NIT deverá ser formalmente comunicado sobre a parceria, conforme Anexo IX. No ato da contratação, será exigida a apresentação da Declaração de Ciência do NIT, quando aplicável. A definição de responsabilidades quanto ao registro ou depósito de pedido de proteção intelectual caberá ao outorgado e à instituição/empresa executora, conforme suas normativas internas e legislação. O Anexo III (Declaração de Apoio da Instituição Copartícipe) agora permite assinatura por autoridade com competência formalmente delegada. Foi incluído o Anexo IX (Modelo de Declaração de Ciência do Núcleo de Inovação Tecnológica – NIT).</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-09-14 a 2026-09-22: Envio da segunda proposta após a 1ª oficina e capacitação (até as 17h59)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>O presente edital tem como objetivo geral estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. Isso será feito por meio de apoio técnico e financeiro a soluções inovadoras com potencial para se transformarem em negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação. O edital visa estimular a criação, formalização e fortalecimento de negócios, promovendo a inovação e o empreendedorismo como estratégias para o desenvolvimento sustentável.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>R$ 30.000,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, comunicacao@fapes.es.gov.br, (27) 3636-1850, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-26: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)
 2026-05-21 a 2026-07-03: Envio da primeira proposta (até as 17h59)
@@ -1025,70 +1338,70 @@
 ?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Serão selecionadas 80 propostas de cada microrregião na Fase 1. Serão selecionadas 25 propostas ou mais por microrregião na Fase 2. A Fapes pode alterar as datas e os prazos definidos no cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas. O proponente poderá submeter mais de uma proposta na Fase 1, mas apenas a de maior nota será selecionada para a Fase 2, caso haja múltiplas propostas classificadas. Propostas com Nota Final inferior a 70,0 pontos serão desclassificadas em ambas as fases.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que tenham como objetivo celebrar parcerias estratégicas com outras startups do Espírito Santo, nacionais ou internacionais. O edital busca fomentar a expansão do mercado, inovação e avanço tecnológico, aprimoramento de produtos ou serviços, acesso a novos canais ou redes de distribuição, atração de talentos e aprimoramento de competências, posicionamento de marca e mercado, acesso a oportunidades de financiamento ou investimento, e impacto socioambiental sustentável.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Startups (pessoas jurídicas) sediadas no Espírito Santo, com faturamento bruto anual de até R$ 16.000.000,00 e até 10 anos de inscrição no Cadastro Nacional da Pessoa Jurídica (CNPJ).</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>R$ 9.800.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Varia de R$ 120.000,00 a R$ 250.000,00, dependendo da modalidade de parceria (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, e R$ 250.000,00 para Modalidade III).</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)
 ?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar da habilitação. O recurso administrativo deverá ser interposto por meio do formulário específico disponível no Sistema de Automação de Fluxos do Governo do Estado (E-Flow): https://fapes.es.gov.br/formularios.)
@@ -1101,270 +1414,333 @@
 ?: Prestação de contas final (Até 30 dias após o prazo de vigência do Termo de Outorga de Subvenção Econômica.)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. É permitido a cada proponente submeter até 2 (duas) propostas de parceria, desde que em modalidades diferentes e com diferentes parceiros. É vedada a submissão de propostas com as mesmas startups alternando funções de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A FAPES não exigirá direitos decorrentes de participação e propriedade nas pesquisas e projetos incentivados. A primeira parcela dos recursos será liberada após a assinatura do Termo de Outorga e comprovação do aporte da contrapartida financeira. A segunda parcela será liberada 30 dias após o 12º mês de execução, mediante prestação de contas parcial, comprovação de 70% de recursos comprometidos/executados e aporte da segunda parcela da contrapartida financeira.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 08/07/2026</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 07/07/2026</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar a manutenção da bolsa de doutorado da FAPES para bolsistas aprovados na seleção do DAAD. O objetivo é permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, garantindo a continuidade do suporte financeiro durante o período de intercâmbio.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Bolsistas de doutorado da FAPES que foram selecionados pelo DAAD, que estão adimplentes com a FAPES e que não estão no primeiro nem no último ano do doutorado.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 08/07/2026</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Apoiar a manutenção da bolsa de doutorado da FAPES para bolsistas aprovados na seleção do DAAD. O objetivo é permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, garantindo a continuidade do suporte financeiro durante o período de intercâmbio." → "Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha."
+Público-alvo: "Bolsistas de doutorado da FAPES que foram selecionados pelo DAAD, que estão adimplentes com a FAPES e que não estão no primeiro nem no último ano do doutorado." → "Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, estejam adimplentes com a FAPES e não estejam no primeiro nem no último ano do doutorado."</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, estejam adimplentes com a FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>Para acesso ao conteúdo completo da chamada, consultar o site do CONFAP através do link: https://news.confap.org.br/daad-lanca-chamada-de-2026-do-programa-de-auxilio-para-doutorandos-brasileiros-com-bolsa-nacional/. As propostas devem ser submetidas na Plataforma do DAAD, e a FAPES realizará o controle de elegibilidade dos selecionados pelo DAAD.</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. As propostas devem ser submetidas na Plataforma do DAAD, e a FAPES realizará o controle de elegibilidade para os selecionados pelo DAAD. O conteúdo completo da chamada está disponível no site do CONFAP.</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="n"/>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 07/07/2026</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos." → "Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo."
-Público-alvo: "Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros." → "Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes."
-Valor total: "-" → "US$ 18.000,00"
-Valor por proposta: "-" → "US$ 6.000,00"
-Contato: "internacional.confap@gmail.com" → "internacional.confap@gmail.com, global@fapes.es.gov.br"
-Submissão (nova): Submissão de propostas (CONFAP) — ? a 2026-08-10
-Submissão (removida): Submissao de propostas — ? a 2026-07-10</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>US$ 18.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>US$ 6.000,00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
 2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-09 10:47
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,22 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -59,18 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -438,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -762,7 +746,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO CIENTÍFICO</t>
+          <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -772,18 +756,18 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 a 2026-07-19: Período de Contratação (2ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 01/08/2026 a 31/12/2026.)</t>
+          <t>2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Selecionar propostas para concessão de auxílio financeiro para a realização de estágio técnico-científico. O estágio pode ser em laboratório ou centro de pesquisa, desenvolvimento ou inovação (PD&amp;I), no país ou no exterior. O objetivo é aprimorar/desenvolver técnicas e processos, além de adquirir conhecimentos específicos vinculados a projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P), públicas ou privadas, localizadas no estado do Espírito Santo.</t>
+          <t>Selecionar propostas para concessão de auxílio financeiro para a realização de visitas técnico-científicas em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, processos e adquirir conhecimentos específicos para projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas no Espírito Santo.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P pública ou privada, localizada no estado do Espírito Santo. Alunos regularmente matriculados em curso de Mestrado ou Doutorado de IES/P localizada no Espírito Santo e recomendado pela CAPES.</t>
+          <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -793,7 +777,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>R$ 10.000,00</t>
+          <t>US$ 2.600,00</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -802,86 +786,6 @@
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 a 2026-03-12: Período de submissão de propostas (1ª Chamada) (Para estágios com início entre 01/05/2026 a 31/07/2026, até as 17h59.)
-2026-03-10: Prazo final para envio de dúvidas (1ª Chamada) (Até 2 dias antes do prazo final de submissão. Para estágios com início entre 01/05/2026 a 31/07/2026.)
-2026-03-17 a 2026-04-24: Período de submissão de propostas (2ª Chamada) (Para estágios com início entre 01/08/2026 a 31/12/2026.)
-2026-03-26: Prazo para interposição de recursos (1ª Chamada) (5 dias úteis após a publicação do resultado preliminar. Para estágios com início entre 01/05/2026 a 31/07/2026.)
-2026-03-31 a 2026-04-30: Período de Contratação (1ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 01/05/2026 a 31/07/2026.)
-2026-04-22: Prazo final para envio de dúvidas (2ª Chamada) (Até 2 dias antes do prazo final de submissão. Para estágios com início entre 01/08/2026 a 31/12/2026.)
-2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar. Para estágios com início entre 01/08/2026 a 31/12/2026.)
-2026-06-19 a 2026-07-19: Período de Contratação (2ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 01/08/2026 a 31/12/2026.)
-2026-07-01 a 2026-08-20: Período de submissão de propostas (3ª Chamada) (Para estágios com início entre 04/01/2027 a 30/04/2027.)
-2026-08-13: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas da última chamada.)
-2026-08-18: Prazo final para envio de dúvidas (3ª Chamada) (Até 2 dias antes do prazo final de submissão. Para estágios com início entre 04/01/2027 a 30/04/2027.)
-2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar. Para estágios com início entre 04/01/2027 a 30/04/2027.)
-2026-10-26 a 2026-11-25: Período de Contratação (3ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 04/01/2027 a 30/04/2027.)</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas nas plataformas. Cada proponente pode apresentar apenas uma proposta por chamada. Não é permitida a contratação concomitante de projeto de estágio técnico-científico e visita técnico-científica para o mesmo período/chamada. O coordenador pode solicitar o adiamento da data de início do estágio por até 30 dias após a contratação, mediante justificativa. É obrigatório mencionar o apoio da Fapes em todas as publicações ou divulgações relacionadas ao projeto.</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_04_2026_-_Estágio_Técnico_Cientifico.pdf</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_04_2026_-_ESTÁGIO_TÉCNICO_CIENTÍFICO.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Selecionar propostas para concessão de auxílio financeiro para a realização de visitas técnico-científicas em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, processos e adquirir conhecimentos específicos para projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas no Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>R$ 2.000.000,00</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>US$ 2.600,00</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-02-09 a 2026-03-12: Submissão de propostas (1ª Chamada) (Até as 17h59. Para visitas com início entre 01/05/2026 a 31/07/2026.)
 2026-03-05: Prazo final para impugnação do edital (Até o quinto dia útil que anteceder o prazo final de submissão da 1ª Chamada.)
@@ -895,70 +799,70 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade institucional, podendo reabrir prazos em casos de força maior ou falhas de sistema, com publicidade das alterações. Cada proponente pode submeter apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Proponentes já contratados neste edital não poderão submeter nova proposta. Após a contratação, o beneficiário pode solicitar adiamento da data de início da visita por até 30 dias, mediante justificativa e autorização. Não será permitida a alteração da instituição de destino da visita técnico-científica após a contratação.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2005_2026%20-%20Visita%20Técnico%20Cientifica%20(1).pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_05_2026_-_VISITA_TÉCNICO-CIENTÍFICA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-07-24: Envio das inscrições - Categorias Projetos e Destaque (Até as 17h59, via SigFapes)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, além de matérias jornalísticas relacionadas à Fapes ou a projetos por ela fomentados, visando valorizar a ciência, tecnologia e inovação e ampliar sua divulgação no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos por ela fomentados.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 308.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-07-24: Envio das inscrições - Categorias Projetos e Destaque (Até as 17h59, via SigFapes)
 2026-06-22 a 2026-09-15: Envio das inscrições - Categoria Jornalismo (Até as 17h59, via SigFapes)
@@ -967,70 +871,70 @@
 ?: Solicitação de pagamento da premiação (Prazo máximo de 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES, mediante abertura de processo eletrônico no sistema E-Flow, via E-Docs)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Não podem participar servidores da Fapes, membros do CCAF, cônjuges, companheiros e parentes até o segundo grau. É permitida apenas uma inscrição por pessoa. Os valores das premiações são brutos e sujeitos a IRRF, tendo caráter honorífico e não gerando vínculo empregatício. Solicitações de acessibilidade devem ser feitas com 10 dias de antecedência do prazo final de inscrição. O comparecimento à cerimônia de premiação é obrigatório, ou indicação de representante. Para a categoria Jornalismo, a matéria deve ter sido veiculada entre 01/09/2025 e 15/09/2026.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-07-30: Contratação / Assinatura do TO e envio de documentos - 2ª Chamada (Até 30 dias após a publicação do resultado final homologado.)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
 2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
@@ -1049,66 +953,66 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo, visando a redução de desigualdades ou vulnerabilidades sociais e a promoção do desenvolvimento socioambiental e econômico nas microrregiões do estado.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Profissionais com graduação e experiência mínima de 3 anos em projetos de extensão ou titulação mínima de mestre, com vínculo empregatício, estatutário, por designação temporária ou termo de adesão a trabalho voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, e que residam no Espírito Santo ou municípios limítrofes.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 5.000.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>R$ 80.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-07-02: Data limite para submissão das propostas no Sigfapes (Até as 17h59)
 ?: Prazo para submissão de recursos administrativos (habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
@@ -1116,66 +1020,66 @@
 ?: Início da contratação (Até 5 (cinco) dias úteis da publicação do resultado homologado para o início do processo de contratação)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução dos projetos é de 24 meses. É obrigatória a previsão de bolsas Ext-E ou Ext-F por um período mínimo de 22 meses. As propostas devem ser submetidas para desenvolvimento em apenas uma das 10 microrregiões listadas no Quadro 2 do edital. Será concedida pontuação adicional para propostas apresentadas por pessoas pertencentes a grupos de ações afirmativas (PcD, negra, quilombola, indígena, trans ou travesti). Propostas com nota final inferior a 70 pontos serão desclassificadas.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -1189,70 +1093,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>2026-07-31 a 2026-08-06: Prazo de submissão de recursos administrativos (habilitação - 1ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Fomentar o empreendedorismo inovador por meio de projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou de processos inovadores. O edital visa transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica. Destina-se a doutores em qualquer área de desenvolvimento.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (até as 17:59h, via Sigfapes)
 2026-07-31 a 2026-08-06: Prazo de submissão de recursos administrativos (habilitação - 1ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)
@@ -1264,70 +1168,70 @@
 2027-04-27 a 2027-05-03: Processo de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O edital prevê duas chamadas para submissão de propostas. Os recursos financeiros remanescentes da primeira chamada poderão ser aplicados na segunda. O prazo de execução dos projetos será de 24 meses, prorrogável por até 12 meses. A subvenção econômica inclui R$ 50.000,00 para serviços de consultoria especializada de aceleradoras. A contrapartida financeira dos outorgados será de 5% do valor subvencionado. A verificação de vínculo empregatício do proponente será realizada no ato da contratação. Para propostas onde a instituição copartícipe é uma ICT ou IES/P vinculada ao Edital FAPES nº 12/2025, o NIT deverá ser formalmente comunicado sobre a parceria, conforme Anexo IX. No ato da contratação, será exigida a apresentação da Declaração de Ciência do NIT, quando aplicável. A definição de responsabilidades quanto ao registro ou depósito de pedido de proteção intelectual caberá ao outorgado e à instituição/empresa executora, conforme suas normativas internas e legislação. O Anexo III (Declaração de Apoio da Instituição Copartícipe) agora permite assinatura por autoridade com competência formalmente delegada. Foi incluído o Anexo IX (Modelo de Declaração de Ciência do Núcleo de Inovação Tecnológica – NIT).</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-09-14 a 2026-09-22: Envio da segunda proposta após a 1ª oficina e capacitação (até as 17h59)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>O presente edital tem como objetivo geral estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. Isso será feito por meio de apoio técnico e financeiro a soluções inovadoras com potencial para se transformarem em negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação. O edital visa estimular a criação, formalização e fortalecimento de negócios, promovendo a inovação e o empreendedorismo como estratégias para o desenvolvimento sustentável.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 30.000,00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, comunicacao@fapes.es.gov.br, (27) 3636-1850, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-26: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)
 2026-05-21 a 2026-07-03: Envio da primeira proposta (até as 17h59)
@@ -1338,70 +1242,70 @@
 ?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>Serão selecionadas 80 propostas de cada microrregião na Fase 1. Serão selecionadas 25 propostas ou mais por microrregião na Fase 2. A Fapes pode alterar as datas e os prazos definidos no cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas. O proponente poderá submeter mais de uma proposta na Fase 1, mas apenas a de maior nota será selecionada para a Fase 2, caso haja múltiplas propostas classificadas. Propostas com Nota Final inferior a 70,0 pontos serão desclassificadas em ambas as fases.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que tenham como objetivo celebrar parcerias estratégicas com outras startups do Espírito Santo, nacionais ou internacionais. O edital busca fomentar a expansão do mercado, inovação e avanço tecnológico, aprimoramento de produtos ou serviços, acesso a novos canais ou redes de distribuição, atração de talentos e aprimoramento de competências, posicionamento de marca e mercado, acesso a oportunidades de financiamento ou investimento, e impacto socioambiental sustentável.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Startups (pessoas jurídicas) sediadas no Espírito Santo, com faturamento bruto anual de até R$ 16.000.000,00 e até 10 anos de inscrição no Cadastro Nacional da Pessoa Jurídica (CNPJ).</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 9.800.000,00</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Varia de R$ 120.000,00 a R$ 250.000,00, dependendo da modalidade de parceria (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, e R$ 250.000,00 para Modalidade III).</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)
 ?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar da habilitação. O recurso administrativo deverá ser interposto por meio do formulário específico disponível no Sistema de Automação de Fluxos do Governo do Estado (E-Flow): https://fapes.es.gov.br/formularios.)
@@ -1414,19 +1318,87 @@
 ?: Prestação de contas final (Até 30 dias após o prazo de vigência do Termo de Outorga de Subvenção Econômica.)</t>
         </is>
       </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. É permitido a cada proponente submeter até 2 (duas) propostas de parceria, desde que em modalidades diferentes e com diferentes parceiros. É vedada a submissão de propostas com as mesmas startups alternando funções de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A FAPES não exigirá direitos decorrentes de participação e propriedade nas pesquisas e projetos incentivados. A primeira parcela dos recursos será liberada após a assinatura do Termo de Outorga e comprovação do aporte da contrapartida financeira. A segunda parcela será liberada 30 dias após o 12º mês de execução, mediante prestação de contas parcial, comprovação de 70% de recursos comprometidos/executados e aporte da segunda parcela da contrapartida financeira.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. É permitido a cada proponente submeter até 2 (duas) propostas de parceria, desde que em modalidades diferentes e com diferentes parceiros. É vedada a submissão de propostas com as mesmas startups alternando funções de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A FAPES não exigirá direitos decorrentes de participação e propriedade nas pesquisas e projetos incentivados. A primeira parcela dos recursos será liberada após a assinatura do Termo de Outorga e comprovação do aporte da contrapartida financeira. A segunda parcela será liberada 30 dias após o 12º mês de execução, mediante prestação de contas parcial, comprovação de 70% de recursos comprometidos/executados e aporte da segunda parcela da contrapartida financeira.</t>
+          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1438,63 +1410,55 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 08/07/2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>R$ 150.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1506,52 +1470,64 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 08/07/2026</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "Apoiar a manutenção da bolsa de doutorado da FAPES para bolsistas aprovados na seleção do DAAD. O objetivo é permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, garantindo a continuidade do suporte financeiro durante o período de intercâmbio." → "Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha."
-Público-alvo: "Bolsistas de doutorado da FAPES que foram selecionados pelo DAAD, que estão adimplentes com a FAPES e que não estão no primeiro nem no último ano do doutorado." → "Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, estejam adimplentes com a FAPES e não estejam no primeiro nem no último ano do doutorado."</t>
-        </is>
-      </c>
+          <t>CHAMADA ERC-CONFAP 2026</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha.</t>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, estejam adimplentes com a FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
+          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr"/>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
+2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+        </is>
+      </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. As propostas devem ser submetidas na Plataforma do DAAD, e a FAPES realizará o controle de elegibilidade para os selecionados pelo DAAD. O conteúdo completo da chamada está disponível no site do CONFAP.</t>
+          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1563,7 +1539,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1571,176 +1547,47 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
+      <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>€ 25.000,00 por ano de projeto</t>
+        </is>
+      </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>US$ 6.000,00</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
-2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA HORIZON EUROPE</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>€ 25.000,00 por ano de projeto</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-10 10:07
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,22 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +59,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -746,46 +762,119 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
+          <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO-CIENTÍFICO</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 10/07/2026</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)</t>
+          <t>2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão.)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
+          <t>Selecionar propostas para concessão de auxílio financeiro para estágios técnico-científicos em laboratórios ou centros de PD&amp;I, no Brasil ou exterior. O objetivo é aprimorar técnicas, adquirir conhecimentos específicos para projetos de PD&amp;I no Espírito Santo, estimular o intercâmbio de conhecimentos, a formação de pós-graduandos e apoiar os Programas de Pós-graduação do estado.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas localizadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P localizadas no Espírito Santo, reconhecidos pela CAPES/CNE/MEC.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>R$ 2.000.000,00</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geped@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-05: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada.)
+2026-02-09 a 2026-03-12: 1ª Chamada - Período de submissão de propostas (Para estágios com início entre 01/05/2026 a 31/07/2026, até as 17h59.)
+2026-03-10: 1ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão.)
+2026-03-17 a 2026-04-24: 2ª Chamada - Período de submissão de propostas (Para estágios com início entre 01/08/2026 a 31/12/2026.)
+2026-03-20 a 2026-03-26: 1ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar.)
+2026-04-22: 2ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão.)
+2026-05-23 a 2026-05-29: 2ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar.)
+2026-07-01 a 2026-08-20: 3ª Chamada - Período de submissão de propostas (Para estágios com início entre 04/01/2027 a 30/04/2027.)
+2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão.)
+2026-10-03 a 2026-10-09: 3ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar.)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>O valor por proposta varia conforme o nível (duração do estágio) e a localização (Brasil - Região Sudeste, Brasil - Demais Estados, Exterior - América Central e do Sul, Exterior - América do Norte, Exterior - Demais Continentes), conforme tabela na seção 6.4 e 6.5 do edital. A Fapes pode alterar as datas e prazos do cronograma, reabrir prazos em casos de força maior ou falhas de sistema, e dará publicidade a essas alterações. Recursos financeiros não utilizados em uma chamada podem ser aplicados em chamadas subsequentes. O beneficiário não poderá utilizar outros recursos da Fapes para cobrir despesas do estágio se o auxílio concedido for insuficiente. Auxílios em moeda estrangeira serão convertidos com base no câmbio oficial na data de aprovação. Cada proponente pode apresentar apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Não é permitida a contratação concomitante de estágio técnico-científico e visita técnico-científica para o mesmo período/chamada. O edital pode ser revogado ou anulado sem direito a indenização. Casos omissos e dúvidas de interpretação serão dirimidos pela Diretoria Executiva da Fapes.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_04_2026_-_Estágio_Técnico_Cientifico.pdf</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_04_2026_-_ESTÁGIO_TÉCNICO-CIENTÍFICO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Removido (nao mais aberto)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
           <t>Selecionar propostas para concessão de auxílio financeiro para a realização de visitas técnico-científicas em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, processos e adquirir conhecimentos específicos para projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>US$ 2.600,00</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-02-09 a 2026-03-12: Submissão de propostas (1ª Chamada) (Até as 17h59. Para visitas com início entre 01/05/2026 a 31/07/2026.)
 2026-03-05: Prazo final para impugnação do edital (Até o quinto dia útil que anteceder o prazo final de submissão da 1ª Chamada.)
@@ -799,70 +888,70 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade institucional, podendo reabrir prazos em casos de força maior ou falhas de sistema, com publicidade das alterações. Cada proponente pode submeter apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Proponentes já contratados neste edital não poderão submeter nova proposta. Após a contratação, o beneficiário pode solicitar adiamento da data de início da visita por até 30 dias, mediante justificativa e autorização. Não será permitida a alteração da instituição de destino da visita técnico-científica após a contratação.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2005_2026%20-%20Visita%20Técnico%20Cientifica%20(1).pdf</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_05_2026_-_VISITA_TÉCNICO-CIENTÍFICA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-07-24: Envio das inscrições - Categorias Projetos e Destaque (Até as 17h59, via SigFapes)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, além de matérias jornalísticas relacionadas à Fapes ou a projetos por ela fomentados, visando valorizar a ciência, tecnologia e inovação e ampliar sua divulgação no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos por ela fomentados.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 308.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000,00</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-07-24: Envio das inscrições - Categorias Projetos e Destaque (Até as 17h59, via SigFapes)
 2026-06-22 a 2026-09-15: Envio das inscrições - Categoria Jornalismo (Até as 17h59, via SigFapes)
@@ -871,70 +960,70 @@
 ?: Solicitação de pagamento da premiação (Prazo máximo de 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES, mediante abertura de processo eletrônico no sistema E-Flow, via E-Docs)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Não podem participar servidores da Fapes, membros do CCAF, cônjuges, companheiros e parentes até o segundo grau. É permitida apenas uma inscrição por pessoa. Os valores das premiações são brutos e sujeitos a IRRF, tendo caráter honorífico e não gerando vínculo empregatício. Solicitações de acessibilidade devem ser feitas com 10 dias de antecedência do prazo final de inscrição. O comparecimento à cerimônia de premiação é obrigatório, ou indicação de representante. Para a categoria Jornalismo, a matéria deve ter sido veiculada entre 01/09/2025 e 15/09/2026.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-07-30: Contratação / Assinatura do TO e envio de documentos - 2ª Chamada (Até 30 dias após a publicação do resultado final homologado.)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
 2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
@@ -953,66 +1042,66 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo, visando a redução de desigualdades ou vulnerabilidades sociais e a promoção do desenvolvimento socioambiental e econômico nas microrregiões do estado.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Profissionais com graduação e experiência mínima de 3 anos em projetos de extensão ou titulação mínima de mestre, com vínculo empregatício, estatutário, por designação temporária ou termo de adesão a trabalho voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, e que residam no Espírito Santo ou municípios limítrofes.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 5.000.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 80.000,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-07-02: Data limite para submissão das propostas no Sigfapes (Até as 17h59)
 ?: Prazo para submissão de recursos administrativos (habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
@@ -1020,66 +1109,66 @@
 ?: Início da contratação (Até 5 (cinco) dias úteis da publicação do resultado homologado para o início do processo de contratação)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução dos projetos é de 24 meses. É obrigatória a previsão de bolsas Ext-E ou Ext-F por um período mínimo de 22 meses. As propostas devem ser submetidas para desenvolvimento em apenas uma das 10 microrregiões listadas no Quadro 2 do edital. Será concedida pontuação adicional para propostas apresentadas por pessoas pertencentes a grupos de ações afirmativas (PcD, negra, quilombola, indígena, trans ou travesti). Propostas com nota final inferior a 70 pontos serão desclassificadas.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -1093,70 +1182,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-07-31 a 2026-08-06: Prazo de submissão de recursos administrativos (habilitação - 1ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Fomentar o empreendedorismo inovador por meio de projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou de processos inovadores. O edital visa transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica. Destina-se a doutores em qualquer área de desenvolvimento.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (até as 17:59h, via Sigfapes)
 2026-07-31 a 2026-08-06: Prazo de submissão de recursos administrativos (habilitação - 1ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)
@@ -1168,70 +1257,70 @@
 2027-04-27 a 2027-05-03: Processo de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>O edital prevê duas chamadas para submissão de propostas. Os recursos financeiros remanescentes da primeira chamada poderão ser aplicados na segunda. O prazo de execução dos projetos será de 24 meses, prorrogável por até 12 meses. A subvenção econômica inclui R$ 50.000,00 para serviços de consultoria especializada de aceleradoras. A contrapartida financeira dos outorgados será de 5% do valor subvencionado. A verificação de vínculo empregatício do proponente será realizada no ato da contratação. Para propostas onde a instituição copartícipe é uma ICT ou IES/P vinculada ao Edital FAPES nº 12/2025, o NIT deverá ser formalmente comunicado sobre a parceria, conforme Anexo IX. No ato da contratação, será exigida a apresentação da Declaração de Ciência do NIT, quando aplicável. A definição de responsabilidades quanto ao registro ou depósito de pedido de proteção intelectual caberá ao outorgado e à instituição/empresa executora, conforme suas normativas internas e legislação. O Anexo III (Declaração de Apoio da Instituição Copartícipe) agora permite assinatura por autoridade com competência formalmente delegada. Foi incluído o Anexo IX (Modelo de Declaração de Ciência do Núcleo de Inovação Tecnológica – NIT).</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-09-14 a 2026-09-22: Envio da segunda proposta após a 1ª oficina e capacitação (até as 17h59)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>O presente edital tem como objetivo geral estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. Isso será feito por meio de apoio técnico e financeiro a soluções inovadoras com potencial para se transformarem em negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação. O edital visa estimular a criação, formalização e fortalecimento de negócios, promovendo a inovação e o empreendedorismo como estratégias para o desenvolvimento sustentável.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>R$ 30.000,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, comunicacao@fapes.es.gov.br, (27) 3636-1850, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-26: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)
 2026-05-21 a 2026-07-03: Envio da primeira proposta (até as 17h59)
@@ -1242,70 +1331,70 @@
 ?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Serão selecionadas 80 propostas de cada microrregião na Fase 1. Serão selecionadas 25 propostas ou mais por microrregião na Fase 2. A Fapes pode alterar as datas e os prazos definidos no cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas. O proponente poderá submeter mais de uma proposta na Fase 1, mas apenas a de maior nota será selecionada para a Fase 2, caso haja múltiplas propostas classificadas. Propostas com Nota Final inferior a 70,0 pontos serão desclassificadas em ambas as fases.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que tenham como objetivo celebrar parcerias estratégicas com outras startups do Espírito Santo, nacionais ou internacionais. O edital busca fomentar a expansão do mercado, inovação e avanço tecnológico, aprimoramento de produtos ou serviços, acesso a novos canais ou redes de distribuição, atração de talentos e aprimoramento de competências, posicionamento de marca e mercado, acesso a oportunidades de financiamento ou investimento, e impacto socioambiental sustentável.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Startups (pessoas jurídicas) sediadas no Espírito Santo, com faturamento bruto anual de até R$ 16.000.000,00 e até 10 anos de inscrição no Cadastro Nacional da Pessoa Jurídica (CNPJ).</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>R$ 9.800.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Varia de R$ 120.000,00 a R$ 250.000,00, dependendo da modalidade de parceria (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, e R$ 250.000,00 para Modalidade III).</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)
 ?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar da habilitação. O recurso administrativo deverá ser interposto por meio do formulário específico disponível no Sistema de Automação de Fluxos do Governo do Estado (E-Flow): https://fapes.es.gov.br/formularios.)
@@ -1318,87 +1407,19 @@
 ?: Prestação de contas final (Até 30 dias após o prazo de vigência do Termo de Outorga de Subvenção Econômica.)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. É permitido a cada proponente submeter até 2 (duas) propostas de parceria, desde que em modalidades diferentes e com diferentes parceiros. É vedada a submissão de propostas com as mesmas startups alternando funções de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A FAPES não exigirá direitos decorrentes de participação e propriedade nas pesquisas e projetos incentivados. A primeira parcela dos recursos será liberada após a assinatura do Termo de Outorga e comprovação do aporte da contrapartida financeira. A segunda parcela será liberada 30 dias após o 12º mês de execução, mediante prestação de contas parcial, comprovação de 70% de recursos comprometidos/executados e aporte da segunda parcela da contrapartida financeira.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>R$ 150.000,00</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1410,7 +1431,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1420,45 +1441,53 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
+          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1470,64 +1499,57 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 10/07/2026</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha." → "Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026."
+Público-alvo: "Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, estejam adimplentes com a FAPES e não estejam no primeiro nem no último ano do doutorado." → "Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado."
+Submissão (nova): Submissão de propostas — ? a ?</t>
+        </is>
+      </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>US$ 6.000,00</t>
-        </is>
-      </c>
+          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
-2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1561,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1547,47 +1569,176 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+        </is>
+      </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA ERC-CONFAP 2026</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
+2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-11 08:47
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,22 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -59,18 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -765,9 +749,9 @@
           <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO-CIENTÍFICO</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 10/07/2026</t>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1502,19 +1486,13 @@
           <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 10/07/2026</t>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha." → "Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026."
-Público-alvo: "Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, estejam adimplentes com a FAPES e não estejam no primeiro nem no último ano do doutorado." → "Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado."
-Submissão (nova): Submissão de propostas — ? a ?</t>
-        </is>
-      </c>
+      <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-14 09:09
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -516,120 +524,51 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Formação Científica</t>
+          <t>Difusão do Conhecimento</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 09/2026 - BOLSAS DE ESTÁGIO DOUTORADO SANDUÍCHE</t>
+          <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Sem alteracoes</t>
+          <t>Removido (nao mais aberto)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28 a 2026-08-03: Prazo para recurso (habilitação) (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação.)</t>
+          <t>2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Apoiar alunos de doutorado regularmente matriculados em programas de pós-graduação do Espírito Santo para a realização de estágio de pesquisa no exterior. O objetivo é proporcionar aprofundamento teórico, coleta e/ou tratamento de dados, ou desenvolvimento parcial da tese, visando ao intercâmbio científico e ao aprimoramento da qualificação acadêmica, com a concessão de bolsa na modalidade Doutorado Sanduíche.</t>
+          <t>O objetivo geral deste edital é selecionar e apoiar financeiramente pesquisadores e alunos para participação em eventos técnico-científicos de curta duração. Visa divulgar os resultados de projetos de pesquisa, desenvolvimento e inovação (P, D&amp;I) desenvolvidos em instituições de ensino superior e/ou pesquisa, públicas ou privadas, localizadas no Estado do Espírito Santo.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Alunos de doutorado regularmente matriculados em Programas de Pós-graduação stricto sensu, recomendados pela CAPES e vinculados a instituições de ensino superior e/ou pesquisa (IES/P) públicas ou privadas no Espírito Santo. Os proponentes devem ser brasileiros ou estrangeiros com autorização de residência, residentes no Espírito Santo, sem título de doutor, com currículo Lattes atualizado, cursando entre o 13º e o 42º mês do doutorado (com pelo menos seis meses restantes para a conclusão após o estágio no exterior), com proficiência na língua da instituição de destino, e com anuência do orientador, supervisor no exterior, e coordenador do PPG. Não devem ter realizado mobilidade acadêmica no exterior com auxílio da Fapes nos últimos 12 meses, nem ter sido contemplados com bolsa de Doutorado Sanduíche da Fapes, Capes ou CNPq anteriormente, e devem estar adimplentes junto à Fapes.</t>
+          <t>Pesquisadores e alunos de pós-graduação vinculados a Instituição de Ensino e/ou Pesquisa (IES/P), pública ou privada, localizada no estado do Espírito Santo.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>R$ 3.000.000,00</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="n"/>
+          <t>R$ 2.500.000,00</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>US$ 2.700,00</t>
+        </is>
+      </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>bolsas.duvidas@fapes.es.gov.br</t>
+          <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-28 a 2026-06-29: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de submissão das propostas.)
-2026-04-28 a 2026-07-02: Prazo para dúvidas e informações (Até 2 dias úteis antecedentes ao término da submissão das propostas.)
-2026-07-06: Submissão das propostas (Até as 17h59.)
-2026-07-28 a 2026-08-03: Prazo para recurso (habilitação) (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação.)
-2026-10-09 a 2026-10-16: Prazo para recurso (classificação) (Até 5 dias úteis após a divulgação do resultado preliminar de classificação.)
-2026-11-01: Contratação dos projetos (Inclui a assinatura eletrônica do Termo de Outorga e o envio de documentos pessoais, com datas a serem divulgadas no resultado homologado.)</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>A duração do estágio de doutorado sanduíche é de, no mínimo, 6 e, no máximo, 12 meses. Os valores das bolsas mensais variam de US$ 1.100,00 a US$ 1.800,00, dependendo do país de destino. O auxílio instalação é equivalente a uma mensalidade da bolsa. O auxílio seguro-saúde é limitado a US$ 90,00 por mês de bolsa, e o auxílio deslocamento é limitado a R$ 12.000,00. A conversão da moeda estrangeira (dólar) ocorre pelo câmbio oficial na data de aprovação do Resultado de Classificação. Taxas administrativas, acadêmicas (tuition &amp; fees), de bancada (bench fees) e adicional dependente não são cobertas. Não é permitida a alteração da instituição de destino ou do supervisor após a submissão da proposta. O prazo de vigência do instrumento de contratação é de 16 meses, improrrogáveis, e o proponente deve realizar o deslocamento dentro desse período. As atividades devem ser realizadas presencialmente na instituição de destino. Para o pagamento integral da mensalidade, o bolsista deve ter executado as atividades por no mínimo 16 dias no mês. O beneficiário tem 16 meses a partir do início da vigência do Termo de Outorga para iniciar e finalizar a bolsa. A existência de inadimplência do proponente com a Fapes ou com as Fazendas Federal, Estadual e Municipal e a Justiça Trabalhista constitui fator impeditivo para contratação. Para a assinatura eletrônica do Termo de Outorga, o proponente e o gestor institucional da IES/P devem ter cadastro ativo no portal 'Acesso Cidadão'.</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL%20FAPES%20N°%2009.2026%20-%20BDS.pdf</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>formacao_cientifica/EDITAL_FAPES_No_09_2026_-_BOLSAS_DE_ESTÁGIO_DOUTORADO_SANDUÍCHE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>O objetivo geral deste edital é selecionar e apoiar financeiramente pesquisadores e alunos para participação em eventos técnico-científicos de curta duração. Visa divulgar os resultados de projetos de pesquisa, desenvolvimento e inovação (P, D&amp;I) desenvolvidos em instituições de ensino superior e/ou pesquisa, públicas ou privadas, localizadas no Estado do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores e alunos de pós-graduação vinculados a Instituição de Ensino e/ou Pesquisa (IES/P), pública ou privada, localizada no estado do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>R$ 2.500.000,00</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>US$ 2.700,00</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>2026-02-27: Prazo para solicitação de atendimento especializado (até 10 dias antes do prazo final de submissão da 1ª Chamada)
 2026-03-02: Prazo para impugnação do edital (até 5 dias úteis antes do prazo final de submissão da 1ª Chamada)
@@ -644,70 +583,70 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 3ª Chamada)</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>O valor total do edital será distribuído em três chamadas. O valor por proposta é fixo e varia conforme o local do evento: R$ 1.800,00 para eventos no Brasil (exceto Espírito Santo), US$ 1.400,00 para América Central ou América do Sul, US$ 2.300,00 para América do Norte e US$ 2.700,00 para outros continentes. A Fapes pode alterar as datas e prazos do cronograma. Cada proponente pode apresentar apenas uma proposta por chamada. O prazo para informar dados bancários é de até 30 dias corridos após o início da vigência do Termo de Outorga. O prazo para envio da prestação de contas é de até 30 dias após o término da vigência do Termo de Outorga. A contratação das propostas aprovadas ocorrerá em até 30 dias após a publicação do resultado final homologado. O envio do comprovante de aceite do trabalho é condicional para o repasse do recurso e deve ser feito até 15 dias antes do evento.</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_02-2026-Participação_Evento_Técnico_Científico.pdf</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_02_2026_-_PARTICIPAÇÃO_EM_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 03/2026 - ORGANIZAÇÃO DE EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 3ª chamada)</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Este edital visa selecionar propostas para conceder apoio financeiro a pesquisadores de nível superior. O objetivo é fomentar a organização de eventos técnico-científicos de curta duração, como congressos, simpósios e seminários, a serem realizados no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores de nível superior vinculados a Instituição de Ensino Superior e/ou Pesquisa (IES/P), pública ou privada sem fins lucrativos, localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>R$ 2.500.000,00</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Varia de R$ 10.000,00 a R$ 35.000,00</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>2026-03-02: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada)
 2026-02-06 a 2026-03-09: 1ª Chamada - Período de submissão de propostas (Eventos com início entre 01/05/2026 a 31/07/2026, até 17h59)
@@ -722,66 +661,66 @@
 ?: Contratação das propostas aprovadas (Até 30 dias após a publicação do resultado final homologado para cada chamada. As datas exatas serão publicadas posteriormente.)</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>O valor do auxílio financeiro é fixo e varia de acordo com o nível do evento: R$ 10.000,00 para Estadual/Regional, R$ 20.000,00 para Nacional e R$ 35.000,00 para Internacional. A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional. Cada proponente pode apresentar apenas uma proposta por chamada. Caso envie mais de uma, será considerada apenas a última enviada. O proponente que já tiver sido contratado neste edital não poderá submeter nova proposta. O evento deve ter duração máxima de 15 dias, consecutivos ou não, e ser chancelado por entidade/sociedade conforme o nível do evento (nacional ou internacional). Os recursos financeiros estão distribuídos por chamada e nível de evento, com possibilidade de remanejamento de saldos não utilizados entre níveis e chamadas subsequentes. É obrigatório mencionar o apoio da Fapes em todas as publicações e divulgações relacionadas ao projeto. A data de início do apoio poderá ser adiada, após a contratação, em até 12 meses, mediante justificativa.</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_03_2026_Organização_Eventos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_03_2026_-_ORGANIZAÇÃO_DE_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO-CIENTÍFICO</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão.)</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Selecionar propostas para concessão de auxílio financeiro para estágios técnico-científicos em laboratórios ou centros de PD&amp;I, no Brasil ou exterior. O objetivo é aprimorar técnicas, adquirir conhecimentos específicos para projetos de PD&amp;I no Espírito Santo, estimular o intercâmbio de conhecimentos, a formação de pós-graduandos e apoiar os Programas de Pós-graduação do estado.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas localizadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P localizadas no Espírito Santo, reconhecidos pela CAPES/CNE/MEC.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="n"/>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geped@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>2026-03-05: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada.)
 2026-02-09 a 2026-03-12: 1ª Chamada - Período de submissão de propostas (Para estágios com início entre 01/05/2026 a 31/07/2026, até as 17h59.)
@@ -795,70 +734,70 @@
 2026-10-03 a 2026-10-09: 3ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>O valor por proposta varia conforme o nível (duração do estágio) e a localização (Brasil - Região Sudeste, Brasil - Demais Estados, Exterior - América Central e do Sul, Exterior - América do Norte, Exterior - Demais Continentes), conforme tabela na seção 6.4 e 6.5 do edital. A Fapes pode alterar as datas e prazos do cronograma, reabrir prazos em casos de força maior ou falhas de sistema, e dará publicidade a essas alterações. Recursos financeiros não utilizados em uma chamada podem ser aplicados em chamadas subsequentes. O beneficiário não poderá utilizar outros recursos da Fapes para cobrir despesas do estágio se o auxílio concedido for insuficiente. Auxílios em moeda estrangeira serão convertidos com base no câmbio oficial na data de aprovação. Cada proponente pode apresentar apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Não é permitida a contratação concomitante de estágio técnico-científico e visita técnico-científica para o mesmo período/chamada. O edital pode ser revogado ou anulado sem direito a indenização. Casos omissos e dúvidas de interpretação serão dirimidos pela Diretoria Executiva da Fapes.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_04_2026_-_Estágio_Técnico_Cientifico.pdf</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_04_2026_-_ESTÁGIO_TÉCNICO-CIENTÍFICO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Selecionar propostas para concessão de auxílio financeiro para a realização de visitas técnico-científicas em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, processos e adquirir conhecimentos específicos para projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>US$ 2.600,00</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>2026-02-09 a 2026-03-12: Submissão de propostas (1ª Chamada) (Até as 17h59. Para visitas com início entre 01/05/2026 a 31/07/2026.)
 2026-03-05: Prazo final para impugnação do edital (Até o quinto dia útil que anteceder o prazo final de submissão da 1ª Chamada.)
@@ -872,70 +811,70 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade institucional, podendo reabrir prazos em casos de força maior ou falhas de sistema, com publicidade das alterações. Cada proponente pode submeter apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Proponentes já contratados neste edital não poderão submeter nova proposta. Após a contratação, o beneficiário pode solicitar adiamento da data de início da visita por até 30 dias, mediante justificativa e autorização. Não será permitida a alteração da instituição de destino da visita técnico-científica após a contratação.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2005_2026%20-%20Visita%20Técnico%20Cientifica%20(1).pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_05_2026_-_VISITA_TÉCNICO-CIENTÍFICA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-07-24: Envio das inscrições - Categorias Projetos e Destaque (Até as 17h59, via SigFapes)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, além de matérias jornalísticas relacionadas à Fapes ou a projetos por ela fomentados, visando valorizar a ciência, tecnologia e inovação e ampliar sua divulgação no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos por ela fomentados.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 308.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-07-24: Envio das inscrições - Categorias Projetos e Destaque (Até as 17h59, via SigFapes)
 2026-06-22 a 2026-09-15: Envio das inscrições - Categoria Jornalismo (Até as 17h59, via SigFapes)
@@ -944,70 +883,70 @@
 ?: Solicitação de pagamento da premiação (Prazo máximo de 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES, mediante abertura de processo eletrônico no sistema E-Flow, via E-Docs)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Não podem participar servidores da Fapes, membros do CCAF, cônjuges, companheiros e parentes até o segundo grau. É permitida apenas uma inscrição por pessoa. Os valores das premiações são brutos e sujeitos a IRRF, tendo caráter honorífico e não gerando vínculo empregatício. Solicitações de acessibilidade devem ser feitas com 10 dias de antecedência do prazo final de inscrição. O comparecimento à cerimônia de premiação é obrigatório, ou indicação de representante. Para a categoria Jornalismo, a matéria deve ter sido veiculada entre 01/09/2025 e 15/09/2026.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-07-30: Contratação / Assinatura do TO e envio de documentos - 2ª Chamada (Até 30 dias após a publicação do resultado final homologado.)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
 2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
@@ -1026,66 +965,66 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo, visando a redução de desigualdades ou vulnerabilidades sociais e a promoção do desenvolvimento socioambiental e econômico nas microrregiões do estado.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Profissionais com graduação e experiência mínima de 3 anos em projetos de extensão ou titulação mínima de mestre, com vínculo empregatício, estatutário, por designação temporária ou termo de adesão a trabalho voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, e que residam no Espírito Santo ou municípios limítrofes.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 5.000.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>R$ 80.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-07-02: Data limite para submissão das propostas no Sigfapes (Até as 17h59)
 ?: Prazo para submissão de recursos administrativos (habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
@@ -1093,66 +1032,66 @@
 ?: Início da contratação (Até 5 (cinco) dias úteis da publicação do resultado homologado para o início do processo de contratação)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução dos projetos é de 24 meses. É obrigatória a previsão de bolsas Ext-E ou Ext-F por um período mínimo de 22 meses. As propostas devem ser submetidas para desenvolvimento em apenas uma das 10 microrregiões listadas no Quadro 2 do edital. Será concedida pontuação adicional para propostas apresentadas por pessoas pertencentes a grupos de ações afirmativas (PcD, negra, quilombola, indígena, trans ou travesti). Propostas com nota final inferior a 70 pontos serão desclassificadas.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -1166,70 +1105,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>2026-07-31 a 2026-08-06: Prazo de submissão de recursos administrativos (habilitação - 1ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Fomentar o empreendedorismo inovador por meio de projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou de processos inovadores. O edital visa transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica. Destina-se a doutores em qualquer área de desenvolvimento.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (até as 17:59h, via Sigfapes)
 2026-07-31 a 2026-08-06: Prazo de submissão de recursos administrativos (habilitação - 1ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)
@@ -1241,70 +1180,70 @@
 2027-04-27 a 2027-05-03: Processo de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O edital prevê duas chamadas para submissão de propostas. Os recursos financeiros remanescentes da primeira chamada poderão ser aplicados na segunda. O prazo de execução dos projetos será de 24 meses, prorrogável por até 12 meses. A subvenção econômica inclui R$ 50.000,00 para serviços de consultoria especializada de aceleradoras. A contrapartida financeira dos outorgados será de 5% do valor subvencionado. A verificação de vínculo empregatício do proponente será realizada no ato da contratação. Para propostas onde a instituição copartícipe é uma ICT ou IES/P vinculada ao Edital FAPES nº 12/2025, o NIT deverá ser formalmente comunicado sobre a parceria, conforme Anexo IX. No ato da contratação, será exigida a apresentação da Declaração de Ciência do NIT, quando aplicável. A definição de responsabilidades quanto ao registro ou depósito de pedido de proteção intelectual caberá ao outorgado e à instituição/empresa executora, conforme suas normativas internas e legislação. O Anexo III (Declaração de Apoio da Instituição Copartícipe) agora permite assinatura por autoridade com competência formalmente delegada. Foi incluído o Anexo IX (Modelo de Declaração de Ciência do Núcleo de Inovação Tecnológica – NIT).</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-09-14 a 2026-09-22: Envio da segunda proposta após a 1ª oficina e capacitação (até as 17h59)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>O presente edital tem como objetivo geral estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. Isso será feito por meio de apoio técnico e financeiro a soluções inovadoras com potencial para se transformarem em negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação. O edital visa estimular a criação, formalização e fortalecimento de negócios, promovendo a inovação e o empreendedorismo como estratégias para o desenvolvimento sustentável.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 30.000,00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, comunicacao@fapes.es.gov.br, (27) 3636-1850, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-26: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)
 2026-05-21 a 2026-07-03: Envio da primeira proposta (até as 17h59)
@@ -1315,70 +1254,70 @@
 ?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>Serão selecionadas 80 propostas de cada microrregião na Fase 1. Serão selecionadas 25 propostas ou mais por microrregião na Fase 2. A Fapes pode alterar as datas e os prazos definidos no cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas. O proponente poderá submeter mais de uma proposta na Fase 1, mas apenas a de maior nota será selecionada para a Fase 2, caso haja múltiplas propostas classificadas. Propostas com Nota Final inferior a 70,0 pontos serão desclassificadas em ambas as fases.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que tenham como objetivo celebrar parcerias estratégicas com outras startups do Espírito Santo, nacionais ou internacionais. O edital busca fomentar a expansão do mercado, inovação e avanço tecnológico, aprimoramento de produtos ou serviços, acesso a novos canais ou redes de distribuição, atração de talentos e aprimoramento de competências, posicionamento de marca e mercado, acesso a oportunidades de financiamento ou investimento, e impacto socioambiental sustentável.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Startups (pessoas jurídicas) sediadas no Espírito Santo, com faturamento bruto anual de até R$ 16.000.000,00 e até 10 anos de inscrição no Cadastro Nacional da Pessoa Jurídica (CNPJ).</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 9.800.000,00</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Varia de R$ 120.000,00 a R$ 250.000,00, dependendo da modalidade de parceria (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, e R$ 250.000,00 para Modalidade III).</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)
 ?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar da habilitação. O recurso administrativo deverá ser interposto por meio do formulário específico disponível no Sistema de Automação de Fluxos do Governo do Estado (E-Flow): https://fapes.es.gov.br/formularios.)
@@ -1391,19 +1330,87 @@
 ?: Prestação de contas final (Até 30 dias após o prazo de vigência do Termo de Outorga de Subvenção Econômica.)</t>
         </is>
       </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. É permitido a cada proponente submeter até 2 (duas) propostas de parceria, desde que em modalidades diferentes e com diferentes parceiros. É vedada a submissão de propostas com as mesmas startups alternando funções de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A FAPES não exigirá direitos decorrentes de participação e propriedade nas pesquisas e projetos incentivados. A primeira parcela dos recursos será liberada após a assinatura do Termo de Outorga e comprovação do aporte da contrapartida financeira. A segunda parcela será liberada 30 dias após o 12º mês de execução, mediante prestação de contas parcial, comprovação de 70% de recursos comprometidos/executados e aporte da segunda parcela da contrapartida financeira.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. É permitido a cada proponente submeter até 2 (duas) propostas de parceria, desde que em modalidades diferentes e com diferentes parceiros. É vedada a submissão de propostas com as mesmas startups alternando funções de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A FAPES não exigirá direitos decorrentes de participação e propriedade nas pesquisas e projetos incentivados. A primeira parcela dos recursos será liberada após a assinatura do Termo de Outorga e comprovação do aporte da contrapartida financeira. A segunda parcela será liberada 30 dias após o 12º mês de execução, mediante prestação de contas parcial, comprovação de 70% de recursos comprometidos/executados e aporte da segunda parcela da contrapartida financeira.</t>
+          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1422,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1423,32 +1430,20 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
-        </is>
-      </c>
+      <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>R$ 150.000,00</t>
-        </is>
-      </c>
+          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1456,22 +1451,22 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1483,7 +1478,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1491,43 +1486,47 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
         </is>
       </c>
       <c r="H15" s="2" t="n"/>
       <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1538,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1549,45 +1548,54 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
+          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
+2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
+          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1607,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1607,56 +1615,49 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)</t>
-        </is>
-      </c>
+      <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>US$ 6.000,00</t>
+          <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
-2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
+?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
+?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
+          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
@@ -1668,57 +1669,68 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
+          <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 14/07/2026</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)</t>
+        </is>
+      </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
+          <t>Este edital visa financiar projetos transnacionais de pesquisa e inovação em matérias-primas para a transição verde e digital. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
+          <t>Organizações de ensino superior e centros de pesquisa públicos. Os consórcios devem ser compostos por, no mínimo, três parceiros de três países diferentes (sendo pelo menos dois da UE ou países associados).</t>
         </is>
       </c>
       <c r="H18" s="2" t="n"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>€ 25.000,00 por ano de projeto</t>
+          <t>EUR 100.000,00</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
-?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
-?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
+          <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)
+2026-09-22: Submissão de propostas nacionais FAPES (Etapa 1) (Recomendado verificar requisitos da FAPES para submissão na plataforma nacional, prazo idêntico ao da submissão da pré-proposta internacional.)
+2026-10-06 a 2026-10-15: Período para interposição de recursos (elegibilidade Etapa 1) (Janela de 10 dias após a divulgação dos resultados de elegibilidade da Etapa 1)
+2026-12-16 a 2026-12-25: Período para interposição de recursos (resultados Etapa 1) (Janela de 10 dias após a divulgação dos resultados da Etapa 1)
+2027-01-31: Solicitações (e aprovação) de mudanças entre as etapas 1 e 2
+2027-02-15: Prazo final para submissão de propostas completas (Até as 15:00 CET)
+2027-02-15: Submissão de propostas nacionais FAPES (Etapa 2) (Recomendado verificar requisitos da FAPES para submissão na plataforma nacional, prazo idêntico ao da submissão da proposta completa internacional.)
+2027-03-06 a 2027-03-15: Período para interposição de recursos (elegibilidade Etapa 2) (Janela de 10 dias após a divulgação dos resultados de elegibilidade da Etapa 2)
+2027-05-16 a 2027-05-25: Período para interposição de recursos (resultados Etapa 2) (Janela de 10 dias após a divulgação dos resultados da Etapa 2)
+2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional / Início dos projetos (esperado)</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
+          <t>O edital é um Joint Transnational Call (JTC) 2026 da Parceria Europeia em Matérias-Primas para a Transição Verde e Digital (RAMP). A FAPES (Fundação de Amparo à Pesquisa e Inovação do Espírito Santo) participa sob o guarda-chuva do CONFAP. Cada parceiro de projeto é financiado diretamente por sua respectiva agência nacional/regional. A Comissão Europeia cofinancia os JTCs da RAMP, com o cofinanciamento sendo redistribuído pelas agências financiadoras aos seus beneficiários. A duração máxima dos projetos é de 36 meses. Propostas devem se enquadrar em um dos seis tópicos temáticos e adotar princípios de 'Safe and Sustainable by Design'. Conforme a tabela de elegibilidade de parceiros do CONFAP, empresas (SMEs e grandes) e entidades sem fins lucrativos (ONGs, associações, sociedades, fundações) não são elegíveis para financiamento pela FAPES.</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-15 09:12
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1672,9 +1664,9 @@
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 14/07/2026</t>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-23 09:22
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -830,25 +838,30 @@
           <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 23/07/2026</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 a 2026-07-24: Envio das inscrições - Categorias Projetos e Destaque (Até as 17h59, via SigFapes)</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
+          <t>2026-06-22 a 2026-07-24: Envio das inscrições – Categorias Projetos e Destaque (Até as 17h59, via SigFapes.)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, além de matérias jornalísticas relacionadas à Fapes ou a projetos por ela fomentados, visando valorizar a ciência, tecnologia e inovação e ampliar sua divulgação no Espírito Santo." → "O Prêmio Fapes visa reconhecer e premiar projetos e trajetórias profissionais de destaque nas áreas de pesquisa, extensão e inovação, além de matérias jornalísticas relacionadas à Fapes ou a projetos fomentados. O objetivo é valorizar a relevância, o impacto e a aplicabilidade da ciência para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados e ampliar a divulgação e popularização da CT&amp;I no estado."
+Público-alvo: "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos por ela fomentados." → "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas/projetos fomentados."</t>
+        </is>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, além de matérias jornalísticas relacionadas à Fapes ou a projetos por ela fomentados, visando valorizar a ciência, tecnologia e inovação e ampliar sua divulgação no Espírito Santo.</t>
+          <t>O Prêmio Fapes visa reconhecer e premiar projetos e trajetórias profissionais de destaque nas áreas de pesquisa, extensão e inovação, além de matérias jornalísticas relacionadas à Fapes ou a projetos fomentados. O objetivo é valorizar a relevância, o impacto e a aplicabilidade da ciência para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados e ampliar a divulgação e popularização da CT&amp;I no estado.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos por ela fomentados.</t>
+          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas/projetos fomentados.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -868,16 +881,14 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 a 2026-07-24: Envio das inscrições - Categorias Projetos e Destaque (Até as 17h59, via SigFapes)
-2026-06-22 a 2026-09-15: Envio das inscrições - Categoria Jornalismo (Até as 17h59, via SigFapes)
-?: Interposição de recursos administrativos (Até 5 (cinco) dias úteis após a publicação dos resultados preliminares no DIO-ES, via E-Flow)
-2026-11-03 a 2026-11-09: Votação popular - Categoria Jornalismo (No site da Fapes, uma única vez por subcategoria)
-?: Solicitação de pagamento da premiação (Prazo máximo de 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES, mediante abertura de processo eletrônico no sistema E-Flow, via E-Docs)</t>
+          <t>2026-06-22 a 2026-07-24: Envio das inscrições – Categorias Projetos e Destaque (Até as 17h59, via SigFapes.)
+2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (Até as 17h59, via SigFapes. Matéria veiculada entre 01/09/2025 e 15/09/2026.)
+?: Prazo para recurso administrativo (5 dias úteis após a divulgação do resultado preliminar, via E-Flow.)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Não podem participar servidores da Fapes, membros do CCAF, cônjuges, companheiros e parentes até o segundo grau. É permitida apenas uma inscrição por pessoa. Os valores das premiações são brutos e sujeitos a IRRF, tendo caráter honorífico e não gerando vínculo empregatício. Solicitações de acessibilidade devem ser feitas com 10 dias de antecedência do prazo final de inscrição. O comparecimento à cerimônia de premiação é obrigatório, ou indicação de representante. Para a categoria Jornalismo, a matéria deve ter sido veiculada entre 01/09/2025 e 15/09/2026.</t>
+          <t>Não podem participar: servidores da Fapes e membros do Conselho Científico-Administrativo da Fapes (CCAF), ativos ou que tenham atuado na Fundação no ano de publicação do edital e nos 3 (três) anos anteriores; cônjuges, companheiros e parentes, até o segundo grau, dessas pessoas. As inscrições devem ser realizadas exclusivamente pelo Sistema de Informação e Gestão de Projetos de Pesquisa da Fapes (SigFapes). É permitida apenas uma inscrição por pessoa neste edital; a última enviada dentro do prazo será considerada válida. Solicitações de atendimento especializado para pessoas com deficiência devem ser feitas com no mínimo 10 dias de antecedência do prazo final de inscrição. A etapa de habilitação é eliminatória. Em caso de empate, a maior pontuação nos critérios de avaliação (na ordem definida para cada subcategoria) será considerada; persistindo o empate, a inscrição enviada primeiro será selecionada. A premiação possui caráter exclusivamente honorífico, meritório e eventual, não configurando vínculo empregatício ou remuneração continuada. O pagamento da premiação financeira ocorrerá após a cerimônia de premiação e a publicação do resultado final no Diário Oficial do Estado do Espírito Santo – DIO-ES. Os contemplados deverão protocolar solicitação de pagamento no prazo máximo de até 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES, mediante abertura de processo eletrônico no sistema E-Flow, via E-Docs. Ao se inscrever, o participante autoriza o uso gratuito e por prazo indeterminado de seu nome, imagem, voz e informações para fins institucionais e de divulgação da Fapes e do prêmio. Qualquer pessoa pode solicitar a impugnação deste edital ou contestar seus termos, apresentando pedido fundamentado em até 5 (cinco) dias úteis antes do encerramento do prazo de envio das propostas, via E-Flow.</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-24 09:17
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -840,28 +840,28 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Atualizado - e-mail enviado em 23/07/2026</t>
+          <t>Atualizado - e-mail enviado em 24/07/2026</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 a 2026-07-24: Envio das inscrições – Categorias Projetos e Destaque (Até as 17h59, via SigFapes.)</t>
+          <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Objetivo: "Reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, além de matérias jornalísticas relacionadas à Fapes ou a projetos por ela fomentados, visando valorizar a ciência, tecnologia e inovação e ampliar sua divulgação no Espírito Santo." → "O Prêmio Fapes visa reconhecer e premiar projetos e trajetórias profissionais de destaque nas áreas de pesquisa, extensão e inovação, além de matérias jornalísticas relacionadas à Fapes ou a projetos fomentados. O objetivo é valorizar a relevância, o impacto e a aplicabilidade da ciência para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados e ampliar a divulgação e popularização da CT&amp;I no estado."
-Público-alvo: "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos por ela fomentados." → "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas/projetos fomentados."</t>
+          <t>Objetivo: "O Prêmio Fapes visa reconhecer e premiar projetos e trajetórias profissionais de destaque nas áreas de pesquisa, extensão e inovação, além de matérias jornalísticas relacionadas à Fapes ou a projetos fomentados. O objetivo é valorizar a relevância, o impacto e a aplicabilidade da ciência para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados e ampliar a divulgação e popularização da CT&amp;I no estado." → "O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação, valorizando a relevância e o impacto da ciência, tecnologia e inovação para o desenvolvimento do Espírito Santo."
+Público-alvo: "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas/projetos fomentados." → "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos fomentados."</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>O Prêmio Fapes visa reconhecer e premiar projetos e trajetórias profissionais de destaque nas áreas de pesquisa, extensão e inovação, além de matérias jornalísticas relacionadas à Fapes ou a projetos fomentados. O objetivo é valorizar a relevância, o impacto e a aplicabilidade da ciência para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados e ampliar a divulgação e popularização da CT&amp;I no estado.</t>
+          <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação, valorizando a relevância e o impacto da ciência, tecnologia e inovação para o desenvolvimento do Espírito Santo.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas/projetos fomentados.</t>
+          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos fomentados.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -881,14 +881,15 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 a 2026-07-24: Envio das inscrições – Categorias Projetos e Destaque (Até as 17h59, via SigFapes.)
-2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (Até as 17h59, via SigFapes. Matéria veiculada entre 01/09/2025 e 15/09/2026.)
-?: Prazo para recurso administrativo (5 dias úteis após a divulgação do resultado preliminar, via E-Flow.)</t>
+          <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)
+2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59. A matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.)
+?: Prazo para recurso administrativo (5 dias úteis após a divulgação do resultado preliminar)
+2026-11-03 a 2026-11-09: Votação popular – Categoria Jornalismo</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Não podem participar: servidores da Fapes e membros do Conselho Científico-Administrativo da Fapes (CCAF), ativos ou que tenham atuado na Fundação no ano de publicação do edital e nos 3 (três) anos anteriores; cônjuges, companheiros e parentes, até o segundo grau, dessas pessoas. As inscrições devem ser realizadas exclusivamente pelo Sistema de Informação e Gestão de Projetos de Pesquisa da Fapes (SigFapes). É permitida apenas uma inscrição por pessoa neste edital; a última enviada dentro do prazo será considerada válida. Solicitações de atendimento especializado para pessoas com deficiência devem ser feitas com no mínimo 10 dias de antecedência do prazo final de inscrição. A etapa de habilitação é eliminatória. Em caso de empate, a maior pontuação nos critérios de avaliação (na ordem definida para cada subcategoria) será considerada; persistindo o empate, a inscrição enviada primeiro será selecionada. A premiação possui caráter exclusivamente honorífico, meritório e eventual, não configurando vínculo empregatício ou remuneração continuada. O pagamento da premiação financeira ocorrerá após a cerimônia de premiação e a publicação do resultado final no Diário Oficial do Estado do Espírito Santo – DIO-ES. Os contemplados deverão protocolar solicitação de pagamento no prazo máximo de até 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES, mediante abertura de processo eletrônico no sistema E-Flow, via E-Docs. Ao se inscrever, o participante autoriza o uso gratuito e por prazo indeterminado de seu nome, imagem, voz e informações para fins institucionais e de divulgação da Fapes e do prêmio. Qualquer pessoa pode solicitar a impugnação deste edital ou contestar seus termos, apresentando pedido fundamentado em até 5 (cinco) dias úteis antes do encerramento do prazo de envio das propostas, via E-Flow.</t>
+          <t>Edição em homenagem à Professora Jurema José de Oliveira. Os valores das premiações possuem natureza bruta e estão sujeitos à incidência do Imposto de Renda Retido na Fonte – IRRF, na forma da legislação tributária vigente. A premiação prevista neste edital possui caráter exclusivamente honorífico, meritório e eventual, destinando-se ao reconhecimento institucional dos trabalhos classificados. A Fapes pode alterar datas e prazos do cronograma por necessidade administrativa ou decisão institucional. O comparecimento do premiado é obrigatório. Caso não possa comparecer, deve indicar formalmente um representante para o recebimento da premiação, com comunicação prévia à Fapes, pelo e-mail gabinete@fapes.es.gov.br. Para as categorias Projetos e Destaque, as 3 (três) propostas com as maiores notas seguem para votação pelo Comitê de Especialistas. Para a categoria Jornalismo, as 3 (três) matérias com maiores notas seguem para votação popular.</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-25 08:59
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -838,9 +830,9 @@
           <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 24/07/2026</t>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -848,12 +840,7 @@
           <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "O Prêmio Fapes visa reconhecer e premiar projetos e trajetórias profissionais de destaque nas áreas de pesquisa, extensão e inovação, além de matérias jornalísticas relacionadas à Fapes ou a projetos fomentados. O objetivo é valorizar a relevância, o impacto e a aplicabilidade da ciência para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados e ampliar a divulgação e popularização da CT&amp;I no estado." → "O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação, valorizando a relevância e o impacto da ciência, tecnologia e inovação para o desenvolvimento do Espírito Santo."
-Público-alvo: "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas/projetos fomentados." → "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos fomentados."</t>
-        </is>
-      </c>
+      <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação, valorizando a relevância e o impacto da ciência, tecnologia e inovação para o desenvolvimento do Espírito Santo.</t>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-01 09:01
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -516,51 +524,120 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Difusão do Conhecimento</t>
+          <t>Formação Científica</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
+          <t>EDITAL FAPES Nº 20/2026 - BOLSAS DE PÓS-DOUTORADO SÊNIOR</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 01/08/2026</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)</t>
+          <t>2026-09-14: Solicitação de recursos de acessibilidade (Até 10 dias do término de submissão das propostas, via e-mail bolsas.duvidas@fapes.es.gov.br.)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>Selecionar propostas para concessão de bolsas de pós-doutorado sênior, a serem realizadas em instituições de excelência no país ou no exterior. O objetivo é aprimorar a qualificação de pesquisadores, fortalecer as atividades de pesquisa científica e tecnológica, e ampliar a cooperação acadêmica nacional e internacional, contribuindo para o desenvolvimento científico e tecnológico no Espírito Santo e no Brasil.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores doutores vinculados a Instituições de Ensino e/ou Pesquisa (IES/P), públicas ou privadas, sediadas no estado do Espírito Santo, que tenham obtido o título de doutor há mais de 8 anos, conforme faixas de titulação especificadas no edital.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>R$ 6.000.000,00</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>bolsas.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao término da submissão das propostas, via Formulário de Impugnação de Edital no E-Flow.)
+2026-09-14: Solicitação de recursos de acessibilidade (Até 10 dias do término de submissão das propostas, via e-mail bolsas.duvidas@fapes.es.gov.br.)
+2026-09-24: Submissão de propostas (Até as 17h59, via Sistema de Informação e Gestão de Projetos da Fapes.)
+?: Prazo para recurso administrativo (habilitação) (5 dias úteis após a publicação do resultado preliminar de habilitação, via Formulário de Recurso Administrativo no E-Flow.)
+?: Prazo para recurso administrativo (classificação) (5 dias úteis após a publicação do resultado preliminar de classificação, via Formulário de Recurso Administrativo no E-Flow.)
+2027-01-18: Contratação das propostas (A partir desta data, com assinatura eletrônica do Termo de Outorga via E-Docs (Acesso Cidadão).)</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>O prazo de execução do projeto é de 16 meses, improrrogáveis, exceto em caso de Advento de Prole. Cada proponente pode apresentar apenas uma proposta; a última enviada será considerada. Os resultados são publicados no Diário Oficial do Estado do Espírito Santo (DIO-ES) e detalhados no site da Fapes. O beneficiário tem um interstício de 16 meses a partir do início da vigência do Termo de Outorga para iniciar e finalizar a bolsa. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. As atividades de pesquisa devem ser realizadas presencialmente na Instituição de Destino, sem modalidade à distância. Não é permitida a alteração da Instituição de Destino ou do Supervisor após a submissão da proposta. O proponente deve ser o bolsista POSDOC. A duração mínima do estágio pós-doutoral é de 6 meses e máxima de 10 meses. Casos omissos e dúvidas de interpretação serão dirimidos pela Direx.</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/POSDOC_Sênior%20-.pdf</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>formacao_cientifica/EDITAL_FAPES_No_20_2026_-_BOLSAS_DE_PÓS-DOUTORADO_SÊNIOR.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Removido (nao mais aberto)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>O objetivo geral deste edital é selecionar e apoiar financeiramente pesquisadores e alunos para participação em eventos técnico-científicos de curta duração. Visa divulgar os resultados de projetos de pesquisa, desenvolvimento e inovação (P, D&amp;I) desenvolvidos em instituições de ensino superior e/ou pesquisa, públicas ou privadas, localizadas no Estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores e alunos de pós-graduação vinculados a Instituição de Ensino e/ou Pesquisa (IES/P), pública ou privada, localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>R$ 2.500.000,00</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>US$ 2.700,00</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>2026-02-27: Prazo para solicitação de atendimento especializado (até 10 dias antes do prazo final de submissão da 1ª Chamada)
 2026-03-02: Prazo para impugnação do edital (até 5 dias úteis antes do prazo final de submissão da 1ª Chamada)
@@ -575,70 +652,70 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 3ª Chamada)</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>O valor total do edital será distribuído em três chamadas. O valor por proposta é fixo e varia conforme o local do evento: R$ 1.800,00 para eventos no Brasil (exceto Espírito Santo), US$ 1.400,00 para América Central ou América do Sul, US$ 2.300,00 para América do Norte e US$ 2.700,00 para outros continentes. A Fapes pode alterar as datas e prazos do cronograma. Cada proponente pode apresentar apenas uma proposta por chamada. O prazo para informar dados bancários é de até 30 dias corridos após o início da vigência do Termo de Outorga. O prazo para envio da prestação de contas é de até 30 dias após o término da vigência do Termo de Outorga. A contratação das propostas aprovadas ocorrerá em até 30 dias após a publicação do resultado final homologado. O envio do comprovante de aceite do trabalho é condicional para o repasse do recurso e deve ser feito até 15 dias antes do evento.</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_02-2026-Participação_Evento_Técnico_Científico.pdf</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_02_2026_-_PARTICIPAÇÃO_EM_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 03/2026 - ORGANIZAÇÃO DE EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 3ª chamada)</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Este edital visa selecionar propostas para conceder apoio financeiro a pesquisadores de nível superior. O objetivo é fomentar a organização de eventos técnico-científicos de curta duração, como congressos, simpósios e seminários, a serem realizados no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores de nível superior vinculados a Instituição de Ensino Superior e/ou Pesquisa (IES/P), pública ou privada sem fins lucrativos, localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>R$ 2.500.000,00</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Varia de R$ 10.000,00 a R$ 35.000,00</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>2026-03-02: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada)
 2026-02-06 a 2026-03-09: 1ª Chamada - Período de submissão de propostas (Eventos com início entre 01/05/2026 a 31/07/2026, até 17h59)
@@ -653,66 +730,66 @@
 ?: Contratação das propostas aprovadas (Até 30 dias após a publicação do resultado final homologado para cada chamada. As datas exatas serão publicadas posteriormente.)</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>O valor do auxílio financeiro é fixo e varia de acordo com o nível do evento: R$ 10.000,00 para Estadual/Regional, R$ 20.000,00 para Nacional e R$ 35.000,00 para Internacional. A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional. Cada proponente pode apresentar apenas uma proposta por chamada. Caso envie mais de uma, será considerada apenas a última enviada. O proponente que já tiver sido contratado neste edital não poderá submeter nova proposta. O evento deve ter duração máxima de 15 dias, consecutivos ou não, e ser chancelado por entidade/sociedade conforme o nível do evento (nacional ou internacional). Os recursos financeiros estão distribuídos por chamada e nível de evento, com possibilidade de remanejamento de saldos não utilizados entre níveis e chamadas subsequentes. É obrigatório mencionar o apoio da Fapes em todas as publicações e divulgações relacionadas ao projeto. A data de início do apoio poderá ser adiada, após a contratação, em até 12 meses, mediante justificativa.</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_03_2026_Organização_Eventos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_03_2026_-_ORGANIZAÇÃO_DE_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO-CIENTÍFICO</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão.)</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Selecionar propostas para concessão de auxílio financeiro para estágios técnico-científicos em laboratórios ou centros de PD&amp;I, no Brasil ou exterior. O objetivo é aprimorar técnicas, adquirir conhecimentos específicos para projetos de PD&amp;I no Espírito Santo, estimular o intercâmbio de conhecimentos, a formação de pós-graduandos e apoiar os Programas de Pós-graduação do estado.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas localizadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P localizadas no Espírito Santo, reconhecidos pela CAPES/CNE/MEC.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geped@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>2026-03-05: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada.)
 2026-02-09 a 2026-03-12: 1ª Chamada - Período de submissão de propostas (Para estágios com início entre 01/05/2026 a 31/07/2026, até as 17h59.)
@@ -726,70 +803,70 @@
 2026-10-03 a 2026-10-09: 3ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>O valor por proposta varia conforme o nível (duração do estágio) e a localização (Brasil - Região Sudeste, Brasil - Demais Estados, Exterior - América Central e do Sul, Exterior - América do Norte, Exterior - Demais Continentes), conforme tabela na seção 6.4 e 6.5 do edital. A Fapes pode alterar as datas e prazos do cronograma, reabrir prazos em casos de força maior ou falhas de sistema, e dará publicidade a essas alterações. Recursos financeiros não utilizados em uma chamada podem ser aplicados em chamadas subsequentes. O beneficiário não poderá utilizar outros recursos da Fapes para cobrir despesas do estágio se o auxílio concedido for insuficiente. Auxílios em moeda estrangeira serão convertidos com base no câmbio oficial na data de aprovação. Cada proponente pode apresentar apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Não é permitida a contratação concomitante de estágio técnico-científico e visita técnico-científica para o mesmo período/chamada. O edital pode ser revogado ou anulado sem direito a indenização. Casos omissos e dúvidas de interpretação serão dirimidos pela Diretoria Executiva da Fapes.</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_04_2026_-_Estágio_Técnico_Cientifico.pdf</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_04_2026_-_ESTÁGIO_TÉCNICO-CIENTÍFICO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Selecionar propostas para concessão de auxílio financeiro para a realização de visitas técnico-científicas em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, processos e adquirir conhecimentos específicos para projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>US$ 2.600,00</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-02-09 a 2026-03-12: Submissão de propostas (1ª Chamada) (Até as 17h59. Para visitas com início entre 01/05/2026 a 31/07/2026.)
 2026-03-05: Prazo final para impugnação do edital (Até o quinto dia útil que anteceder o prazo final de submissão da 1ª Chamada.)
@@ -803,70 +880,70 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade institucional, podendo reabrir prazos em casos de força maior ou falhas de sistema, com publicidade das alterações. Cada proponente pode submeter apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Proponentes já contratados neste edital não poderão submeter nova proposta. Após a contratação, o beneficiário pode solicitar adiamento da data de início da visita por até 30 dias, mediante justificativa e autorização. Não será permitida a alteração da instituição de destino da visita técnico-científica após a contratação.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2005_2026%20-%20Visita%20Técnico%20Cientifica%20(1).pdf</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_05_2026_-_VISITA_TÉCNICO-CIENTÍFICA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação, valorizando a relevância e o impacto da ciência, tecnologia e inovação para o desenvolvimento do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos fomentados.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 308.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000,00</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)
 2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59. A matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.)
@@ -874,70 +951,70 @@
 2026-11-03 a 2026-11-09: Votação popular – Categoria Jornalismo</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Edição em homenagem à Professora Jurema José de Oliveira. Os valores das premiações possuem natureza bruta e estão sujeitos à incidência do Imposto de Renda Retido na Fonte – IRRF, na forma da legislação tributária vigente. A premiação prevista neste edital possui caráter exclusivamente honorífico, meritório e eventual, destinando-se ao reconhecimento institucional dos trabalhos classificados. A Fapes pode alterar datas e prazos do cronograma por necessidade administrativa ou decisão institucional. O comparecimento do premiado é obrigatório. Caso não possa comparecer, deve indicar formalmente um representante para o recebimento da premiação, com comunicação prévia à Fapes, pelo e-mail gabinete@fapes.es.gov.br. Para as categorias Projetos e Destaque, as 3 (três) propostas com as maiores notas seguem para votação pelo Comitê de Especialistas. Para a categoria Jornalismo, as 3 (três) matérias com maiores notas seguem para votação popular.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-06-19 a 2026-08-25: Submissão de propostas - 3ª Chamada (Até as 17h59)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
 2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
@@ -956,66 +1033,66 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo, visando a redução de desigualdades ou vulnerabilidades sociais e a promoção do desenvolvimento socioambiental e econômico nas microrregiões do estado.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Profissionais com graduação e experiência mínima de 3 anos em projetos de extensão ou titulação mínima de mestre, com vínculo empregatício, estatutário, por designação temporária ou termo de adesão a trabalho voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, e que residam no Espírito Santo ou municípios limítrofes.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 5.000.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 80.000,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-07-02: Data limite para submissão das propostas no Sigfapes (Até as 17h59)
 ?: Prazo para submissão de recursos administrativos (habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
@@ -1023,92 +1100,19 @@
 ?: Início da contratação (Até 5 (cinco) dias úteis da publicação do resultado homologado para o início do processo de contratação)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução dos projetos é de 24 meses. É obrigatória a previsão de bolsas Ext-E ou Ext-F por um período mínimo de 22 meses. As propostas devem ser submetidas para desenvolvimento em apenas uma das 10 microrregiões listadas no Quadro 2 do edital. Será concedida pontuação adicional para propostas apresentadas por pessoas pertencentes a grupos de ações afirmativas (PcD, negra, quilombola, indígena, trans ou travesti). Propostas com nota final inferior a 70 pontos serão desclassificadas.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Inovação</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>R$ 40.000.000,00</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>R$ 3.000.000,00</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>duvidas.inovacao@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
-?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
-?: Interposição de recursos administrativos da habilitação (05 dias úteis a partir da publicação do resultado preliminar)
-?: Interposição de recursos administrativos da avaliação de TRL e mérito (05 dias úteis a partir da publicação do resultado preliminar)
-?: Interposição de recursos administrativos das visitas técnicas (05 dias úteis a partir da publicação do resultado preliminar da visita técnica)
-?: Submissão de documentação para contratação (Até 30 dias a partir da publicação do resultado homologado do julgamento de mérito)
-?: Informar dados da conta bancária (Até 30 dias após a publicação do Termo de Outorga)
-?: Prestação de contas parcial (1ª) (Até 30 dias após o 8º mês de vigência do Termo de Outorga)
-?: Prestação de contas parcial (2ª) (Até 30 dias após o 16º mês de vigência do Termo de Outorga)
-?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-02 08:58
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -532,9 +524,9 @@
           <t>EDITAL FAPES Nº 20/2026 - BOLSAS DE PÓS-DOUTORADO SÊNIOR</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 01/08/2026</t>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-03 10:38
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,22 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +59,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -521,42 +537,113 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 20/2026 - BOLSAS DE PÓS-DOUTORADO SÊNIOR</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>EDITAL FAPES Nº 19/2026 - PIC JR 2027</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 03/08/2026</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14: Solicitação de recursos de acessibilidade (Até 10 dias do término de submissão das propostas, via e-mail bolsas.duvidas@fapes.es.gov.br.)</t>
+          <t>2026-09-09: Submissão de propostas (Até as 17h59)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>O objetivo geral deste edital é selecionar projetos que despertem nos estudantes da Rede Pública de Educação Básica do Espírito Santo o interesse pela ciência, pelo desenvolvimento tecnológico e por ações de inovação. O programa apoia financeiramente projetos de pesquisa desenvolvidos em parceria entre escolas públicas de Educação Básica e Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo. Destina-se a pesquisadores, IES/P, professores e estudantes da Rede Pública de Educação Básica do Estado do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores (mínimo mestre) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo, em parceria com professores e estudantes da Rede Pública de Educação Básica do Estado do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>R$ 8.887.500,00</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>R$ 10.000,00</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>bolsas.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09: Submissão de propostas (Até as 17h59)
+?: Interposição de recursos (habilitação) (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação)
+?: Interposição de recursos (análise de mérito) (Até 5 dias úteis após a divulgação do resultado preliminar de análise de mérito)
+2027-02-09: Contratação dos projetos selecionados</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>O valor total do edital é distribuído por faixas (Educação Ambiental Formal, Práticas de Ciências da Natureza e Matemática, Bairros do Programa Estado Presente, Ampla Concorrência), com possibilidade de transferência de recursos entre elas. Além do auxílio financeiro de R$ 10.000,00 por projeto, são concedidas bolsas para coordenador (BCO), tutor (BTU), iniciação científica e tecnológica (ICT) e iniciação científica júnior (ICJr). Apenas as cinco bolsas de ICJr são obrigatórias. As bolsas BCO, BTU e ICT têm duração de até 10 meses, e as bolsas ICJr, até 9 meses. Os projetos devem ser inéditos para a Fapes. A Fapes abre mão dos direitos de participação e propriedade sobre pesquisas e projetos apoiados, mas os resultados econômicos da exploração comercial de criações protegidas serão partilhados.</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/PIC_JR_2027%20-.pdf</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>formacao_cientifica/EDITAL_FAPES_No_19_2026_-_PIC_JR_2027.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Formação Científica</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 20/2026 - BOLSAS DE PÓS-DOUTORADO SÊNIOR</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14: Solicitação de recursos de acessibilidade (Até 10 dias do término de submissão das propostas, via e-mail bolsas.duvidas@fapes.es.gov.br.)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>Selecionar propostas para concessão de bolsas de pós-doutorado sênior, a serem realizadas em instituições de excelência no país ou no exterior. O objetivo é aprimorar a qualificação de pesquisadores, fortalecer as atividades de pesquisa científica e tecnológica, e ampliar a cooperação acadêmica nacional e internacional, contribuindo para o desenvolvimento científico e tecnológico no Espírito Santo e no Brasil.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores doutores vinculados a Instituições de Ensino e/ou Pesquisa (IES/P), públicas ou privadas, sediadas no estado do Espírito Santo, que tenham obtido o título de doutor há mais de 8 anos, conforme faixas de titulação especificadas no edital.</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>R$ 6.000.000,00</t>
         </is>
       </c>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>bolsas.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao término da submissão das propostas, via Formulário de Impugnação de Edital no E-Flow.)
 2026-09-14: Solicitação de recursos de acessibilidade (Até 10 dias do término de submissão das propostas, via e-mail bolsas.duvidas@fapes.es.gov.br.)
@@ -566,70 +653,70 @@
 2027-01-18: Contratação das propostas (A partir desta data, com assinatura eletrônica do Termo de Outorga via E-Docs (Acesso Cidadão).)</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução do projeto é de 16 meses, improrrogáveis, exceto em caso de Advento de Prole. Cada proponente pode apresentar apenas uma proposta; a última enviada será considerada. Os resultados são publicados no Diário Oficial do Estado do Espírito Santo (DIO-ES) e detalhados no site da Fapes. O beneficiário tem um interstício de 16 meses a partir do início da vigência do Termo de Outorga para iniciar e finalizar a bolsa. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. As atividades de pesquisa devem ser realizadas presencialmente na Instituição de Destino, sem modalidade à distância. Não é permitida a alteração da Instituição de Destino ou do Supervisor após a submissão da proposta. O proponente deve ser o bolsista POSDOC. A duração mínima do estágio pós-doutoral é de 6 meses e máxima de 10 meses. Casos omissos e dúvidas de interpretação serão dirimidos pela Direx.</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/POSDOC_Sênior%20-.pdf</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>formacao_cientifica/EDITAL_FAPES_No_20_2026_-_BOLSAS_DE_PÓS-DOUTORADO_SÊNIOR.pdf</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>O objetivo geral deste edital é selecionar e apoiar financeiramente pesquisadores e alunos para participação em eventos técnico-científicos de curta duração. Visa divulgar os resultados de projetos de pesquisa, desenvolvimento e inovação (P, D&amp;I) desenvolvidos em instituições de ensino superior e/ou pesquisa, públicas ou privadas, localizadas no Estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores e alunos de pós-graduação vinculados a Instituição de Ensino e/ou Pesquisa (IES/P), pública ou privada, localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>R$ 2.500.000,00</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>US$ 2.700,00</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>2026-02-27: Prazo para solicitação de atendimento especializado (até 10 dias antes do prazo final de submissão da 1ª Chamada)
 2026-03-02: Prazo para impugnação do edital (até 5 dias úteis antes do prazo final de submissão da 1ª Chamada)
@@ -644,70 +731,70 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 3ª Chamada)</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>O valor total do edital será distribuído em três chamadas. O valor por proposta é fixo e varia conforme o local do evento: R$ 1.800,00 para eventos no Brasil (exceto Espírito Santo), US$ 1.400,00 para América Central ou América do Sul, US$ 2.300,00 para América do Norte e US$ 2.700,00 para outros continentes. A Fapes pode alterar as datas e prazos do cronograma. Cada proponente pode apresentar apenas uma proposta por chamada. O prazo para informar dados bancários é de até 30 dias corridos após o início da vigência do Termo de Outorga. O prazo para envio da prestação de contas é de até 30 dias após o término da vigência do Termo de Outorga. A contratação das propostas aprovadas ocorrerá em até 30 dias após a publicação do resultado final homologado. O envio do comprovante de aceite do trabalho é condicional para o repasse do recurso e deve ser feito até 15 dias antes do evento.</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_02-2026-Participação_Evento_Técnico_Científico.pdf</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_02_2026_-_PARTICIPAÇÃO_EM_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 03/2026 - ORGANIZAÇÃO DE EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 3ª chamada)</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Este edital visa selecionar propostas para conceder apoio financeiro a pesquisadores de nível superior. O objetivo é fomentar a organização de eventos técnico-científicos de curta duração, como congressos, simpósios e seminários, a serem realizados no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores de nível superior vinculados a Instituição de Ensino Superior e/ou Pesquisa (IES/P), pública ou privada sem fins lucrativos, localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>R$ 2.500.000,00</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Varia de R$ 10.000,00 a R$ 35.000,00</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>2026-03-02: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada)
 2026-02-06 a 2026-03-09: 1ª Chamada - Período de submissão de propostas (Eventos com início entre 01/05/2026 a 31/07/2026, até 17h59)
@@ -722,66 +809,66 @@
 ?: Contratação das propostas aprovadas (Até 30 dias após a publicação do resultado final homologado para cada chamada. As datas exatas serão publicadas posteriormente.)</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>O valor do auxílio financeiro é fixo e varia de acordo com o nível do evento: R$ 10.000,00 para Estadual/Regional, R$ 20.000,00 para Nacional e R$ 35.000,00 para Internacional. A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional. Cada proponente pode apresentar apenas uma proposta por chamada. Caso envie mais de uma, será considerada apenas a última enviada. O proponente que já tiver sido contratado neste edital não poderá submeter nova proposta. O evento deve ter duração máxima de 15 dias, consecutivos ou não, e ser chancelado por entidade/sociedade conforme o nível do evento (nacional ou internacional). Os recursos financeiros estão distribuídos por chamada e nível de evento, com possibilidade de remanejamento de saldos não utilizados entre níveis e chamadas subsequentes. É obrigatório mencionar o apoio da Fapes em todas as publicações e divulgações relacionadas ao projeto. A data de início do apoio poderá ser adiada, após a contratação, em até 12 meses, mediante justificativa.</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_03_2026_Organização_Eventos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_03_2026_-_ORGANIZAÇÃO_DE_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO-CIENTÍFICO</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão.)</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Selecionar propostas para concessão de auxílio financeiro para estágios técnico-científicos em laboratórios ou centros de PD&amp;I, no Brasil ou exterior. O objetivo é aprimorar técnicas, adquirir conhecimentos específicos para projetos de PD&amp;I no Espírito Santo, estimular o intercâmbio de conhecimentos, a formação de pós-graduandos e apoiar os Programas de Pós-graduação do estado.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas localizadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P localizadas no Espírito Santo, reconhecidos pela CAPES/CNE/MEC.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="n"/>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geped@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-03-05: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada.)
 2026-02-09 a 2026-03-12: 1ª Chamada - Período de submissão de propostas (Para estágios com início entre 01/05/2026 a 31/07/2026, até as 17h59.)
@@ -795,70 +882,70 @@
 2026-10-03 a 2026-10-09: 3ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>O valor por proposta varia conforme o nível (duração do estágio) e a localização (Brasil - Região Sudeste, Brasil - Demais Estados, Exterior - América Central e do Sul, Exterior - América do Norte, Exterior - Demais Continentes), conforme tabela na seção 6.4 e 6.5 do edital. A Fapes pode alterar as datas e prazos do cronograma, reabrir prazos em casos de força maior ou falhas de sistema, e dará publicidade a essas alterações. Recursos financeiros não utilizados em uma chamada podem ser aplicados em chamadas subsequentes. O beneficiário não poderá utilizar outros recursos da Fapes para cobrir despesas do estágio se o auxílio concedido for insuficiente. Auxílios em moeda estrangeira serão convertidos com base no câmbio oficial na data de aprovação. Cada proponente pode apresentar apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Não é permitida a contratação concomitante de estágio técnico-científico e visita técnico-científica para o mesmo período/chamada. O edital pode ser revogado ou anulado sem direito a indenização. Casos omissos e dúvidas de interpretação serão dirimidos pela Diretoria Executiva da Fapes.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_04_2026_-_Estágio_Técnico_Cientifico.pdf</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_04_2026_-_ESTÁGIO_TÉCNICO-CIENTÍFICO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Selecionar propostas para concessão de auxílio financeiro para a realização de visitas técnico-científicas em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, processos e adquirir conhecimentos específicos para projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>US$ 2.600,00</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-02-09 a 2026-03-12: Submissão de propostas (1ª Chamada) (Até as 17h59. Para visitas com início entre 01/05/2026 a 31/07/2026.)
 2026-03-05: Prazo final para impugnação do edital (Até o quinto dia útil que anteceder o prazo final de submissão da 1ª Chamada.)
@@ -872,70 +959,70 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade institucional, podendo reabrir prazos em casos de força maior ou falhas de sistema, com publicidade das alterações. Cada proponente pode submeter apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Proponentes já contratados neste edital não poderão submeter nova proposta. Após a contratação, o beneficiário pode solicitar adiamento da data de início da visita por até 30 dias, mediante justificativa e autorização. Não será permitida a alteração da instituição de destino da visita técnico-científica após a contratação.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2005_2026%20-%20Visita%20Técnico%20Cientifica%20(1).pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_05_2026_-_VISITA_TÉCNICO-CIENTÍFICA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação, valorizando a relevância e o impacto da ciência, tecnologia e inovação para o desenvolvimento do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos fomentados.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 308.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)
 2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59. A matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.)
@@ -943,70 +1030,70 @@
 2026-11-03 a 2026-11-09: Votação popular – Categoria Jornalismo</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Edição em homenagem à Professora Jurema José de Oliveira. Os valores das premiações possuem natureza bruta e estão sujeitos à incidência do Imposto de Renda Retido na Fonte – IRRF, na forma da legislação tributária vigente. A premiação prevista neste edital possui caráter exclusivamente honorífico, meritório e eventual, destinando-se ao reconhecimento institucional dos trabalhos classificados. A Fapes pode alterar datas e prazos do cronograma por necessidade administrativa ou decisão institucional. O comparecimento do premiado é obrigatório. Caso não possa comparecer, deve indicar formalmente um representante para o recebimento da premiação, com comunicação prévia à Fapes, pelo e-mail gabinete@fapes.es.gov.br. Para as categorias Projetos e Destaque, as 3 (três) propostas com as maiores notas seguem para votação pelo Comitê de Especialistas. Para a categoria Jornalismo, as 3 (três) matérias com maiores notas seguem para votação popular.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>2026-06-19 a 2026-08-25: Submissão de propostas - 3ª Chamada (Até as 17h59)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
 2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
@@ -1025,66 +1112,66 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo, visando a redução de desigualdades ou vulnerabilidades sociais e a promoção do desenvolvimento socioambiental e econômico nas microrregiões do estado.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Profissionais com graduação e experiência mínima de 3 anos em projetos de extensão ou titulação mínima de mestre, com vínculo empregatício, estatutário, por designação temporária ou termo de adesão a trabalho voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, e que residam no Espírito Santo ou municípios limítrofes.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 5.000.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 80.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-07-02: Data limite para submissão das propostas no Sigfapes (Até as 17h59)
 ?: Prazo para submissão de recursos administrativos (habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
@@ -1092,70 +1179,146 @@
 ?: Início da contratação (Até 5 (cinco) dias úteis da publicação do resultado homologado para o início do processo de contratação)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução dos projetos é de 24 meses. É obrigatória a previsão de bolsas Ext-E ou Ext-F por um período mínimo de 22 meses. As propostas devem ser submetidas para desenvolvimento em apenas uma das 10 microrregiões listadas no Quadro 2 do edital. Será concedida pontuação adicional para propostas apresentadas por pessoas pertencentes a grupos de ações afirmativas (PcD, negra, quilombola, indígena, trans ou travesti). Propostas com nota final inferior a 70 pontos serão desclassificadas.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 03/08/2026</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES)." → "Promover o aumento da competitividade dos setores econômicos capixabas por meio de projetos de inovação, desenvolvidos por empresas (incluindo cooperativas de trabalho) em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas. O apoio se dará por meio de um modelo de coinvestimento tripartite (FAPES, empresa/cooperativa, ICT/IES), com projetos alinhados ao Plano ES 500 Anos e ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES)."
+Público-alvo: "Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas." → "Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas ou cooperativas de trabalho capixabas."
+Valor por proposta: "R$ 3.000.000,00" → "R$ 500.000,00 a R$ 3.000.000,00"
+Contato: "duvidas.inovacao@fapes.es.gov.br" → "duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br"
+Submissão (nova): Submissão das propostas no SIGFAPES — 2026-03-30 a ?</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Promover o aumento da competitividade dos setores econômicos capixabas por meio de projetos de inovação, desenvolvidos por empresas (incluindo cooperativas de trabalho) em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas. O apoio se dará por meio de um modelo de coinvestimento tripartite (FAPES, empresa/cooperativa, ICT/IES), com projetos alinhados ao Plano ES 500 Anos e ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas ou cooperativas de trabalho capixabas.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>R$ 40.000.000,00</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>R$ 500.000,00 a R$ 3.000.000,00</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-30: Submissão das propostas no SIGFAPES (Fluxo contínuo)
+?: Prazo de submissão dos recursos administrativos (Habilitação) (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)
+?: Prazo de submissão dos recursos administrativos (TRL/Mérito) (5 dias úteis a partir da publicação do resultado preliminar do TRL/Mérito.)
+?: Prazo de submissão dos recursos administrativos (Visita Técnica) (5 dias úteis a partir da publicação do resultado preliminar da visita técnica.)
+?: Submissão das documentações para contratação (Até 30 dias a partir da publicação do resultado homologado do julgamento de mérito.)</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>O prazo de execução do projeto é de 24 meses, com possibilidade de prorrogação por até 12 meses. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais; cooperativas de trabalho devem apresentar Demonstração de Sobras ou Perdas (DSP). As empresas devem estar ativas há pelo menos 6 meses e não podem ter sido contratadas em editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026, a menos que o projeto, coordenador e equipe executora sejam distintos. É permitida apenas uma proposta por empresa. Em caso de inabilitação ou desclassificação, a empresa poderá realizar uma nova submissão, exceto se reprovada pelo Comitê de Conformidade, o que impede nova submissão nesta chamada. A aprovação da proposta não garante a contratação, que está sujeita à disponibilidade financeira da FAPES, ordem de submissão e visita técnica. O critério de desempate é a data de submissão da proposta no SIGFAPES. Propostas com Nota Final inferior a 80 pontos ou notas individuais inferiores a 4 em critérios específicos serão desclassificadas. A impugnação dos termos do edital deve ser feita em até 5 dias úteis antes do encerramento do prazo de submissão das propostas do primeiro ciclo (considerando o fluxo contínuo, esta observação se refere a um prazo inicial para impugnação do edital em si).</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Inovação</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-07-31 a 2026-08-06: Prazo de submissão de recursos administrativos (habilitação - 1ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Fomentar o empreendedorismo inovador por meio de projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou de processos inovadores. O edital visa transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica. Destina-se a doutores em qualquer área de desenvolvimento.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (até as 17:59h, via Sigfapes)
 2026-07-31 a 2026-08-06: Prazo de submissão de recursos administrativos (habilitação - 1ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)
@@ -1167,70 +1330,70 @@
 2027-04-27 a 2027-05-03: Processo de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>O edital prevê duas chamadas para submissão de propostas. Os recursos financeiros remanescentes da primeira chamada poderão ser aplicados na segunda. O prazo de execução dos projetos será de 24 meses, prorrogável por até 12 meses. A subvenção econômica inclui R$ 50.000,00 para serviços de consultoria especializada de aceleradoras. A contrapartida financeira dos outorgados será de 5% do valor subvencionado. A verificação de vínculo empregatício do proponente será realizada no ato da contratação. Para propostas onde a instituição copartícipe é uma ICT ou IES/P vinculada ao Edital FAPES nº 12/2025, o NIT deverá ser formalmente comunicado sobre a parceria, conforme Anexo IX. No ato da contratação, será exigida a apresentação da Declaração de Ciência do NIT, quando aplicável. A definição de responsabilidades quanto ao registro ou depósito de pedido de proteção intelectual caberá ao outorgado e à instituição/empresa executora, conforme suas normativas internas e legislação. O Anexo III (Declaração de Apoio da Instituição Copartícipe) agora permite assinatura por autoridade com competência formalmente delegada. Foi incluído o Anexo IX (Modelo de Declaração de Ciência do Núcleo de Inovação Tecnológica – NIT).</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>2026-09-14 a 2026-09-22: Envio da segunda proposta após a 1ª oficina e capacitação (até as 17h59)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>O presente edital tem como objetivo geral estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. Isso será feito por meio de apoio técnico e financeiro a soluções inovadoras com potencial para se transformarem em negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação. O edital visa estimular a criação, formalização e fortalecimento de negócios, promovendo a inovação e o empreendedorismo como estratégias para o desenvolvimento sustentável.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>R$ 30.000,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, comunicacao@fapes.es.gov.br, (27) 3636-1850, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-26: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)
 2026-05-21 a 2026-07-03: Envio da primeira proposta (até as 17h59)
@@ -1241,70 +1404,70 @@
 ?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Serão selecionadas 80 propostas de cada microrregião na Fase 1. Serão selecionadas 25 propostas ou mais por microrregião na Fase 2. A Fapes pode alterar as datas e os prazos definidos no cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas. O proponente poderá submeter mais de uma proposta na Fase 1, mas apenas a de maior nota será selecionada para a Fase 2, caso haja múltiplas propostas classificadas. Propostas com Nota Final inferior a 70,0 pontos serão desclassificadas em ambas as fases.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que tenham como objetivo celebrar parcerias estratégicas com outras startups do Espírito Santo, nacionais ou internacionais. O edital busca fomentar a expansão do mercado, inovação e avanço tecnológico, aprimoramento de produtos ou serviços, acesso a novos canais ou redes de distribuição, atração de talentos e aprimoramento de competências, posicionamento de marca e mercado, acesso a oportunidades de financiamento ou investimento, e impacto socioambiental sustentável.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Startups (pessoas jurídicas) sediadas no Espírito Santo, com faturamento bruto anual de até R$ 16.000.000,00 e até 10 anos de inscrição no Cadastro Nacional da Pessoa Jurídica (CNPJ).</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>R$ 9.800.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Varia de R$ 120.000,00 a R$ 250.000,00, dependendo da modalidade de parceria (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, e R$ 250.000,00 para Modalidade III).</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)
 ?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar da habilitação. O recurso administrativo deverá ser interposto por meio do formulário específico disponível no Sistema de Automação de Fluxos do Governo do Estado (E-Flow): https://fapes.es.gov.br/formularios.)
@@ -1317,143 +1480,19 @@
 ?: Prestação de contas final (Até 30 dias após o prazo de vigência do Termo de Outorga de Subvenção Econômica.)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. É permitido a cada proponente submeter até 2 (duas) propostas de parceria, desde que em modalidades diferentes e com diferentes parceiros. É vedada a submissão de propostas com as mesmas startups alternando funções de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A FAPES não exigirá direitos decorrentes de participação e propriedade nas pesquisas e projetos incentivados. A primeira parcela dos recursos será liberada após a assinatura do Termo de Outorga e comprovação do aporte da contrapartida financeira. A segunda parcela será liberada 30 dias após o 12º mês de execução, mediante prestação de contas parcial, comprovação de 70% de recursos comprometidos/executados e aporte da segunda parcela da contrapartida financeira.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>R$ 150.000,00</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
-        </is>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1465,7 +1504,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1475,45 +1514,53 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
+          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1572,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1533,165 +1580,281 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)</t>
-        </is>
-      </c>
+      <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
+          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA ERC-CONFAP 2026</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
           <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>US$ 18.000,00</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>US$ 6.000,00</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
 2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Este edital visa financiar projetos transnacionais de pesquisa e inovação em matérias-primas para a transição verde e digital. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Organizações de ensino superior e centros de pesquisa públicos. Os consórcios devem ser compostos por, no mínimo, três parceiros de três países diferentes (sendo pelo menos dois da UE ou países associados).</t>
         </is>
       </c>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)
 2026-09-22: Submissão de propostas nacionais FAPES (Etapa 1) (Recomendado verificar requisitos da FAPES para submissão na plataforma nacional, prazo idêntico ao da submissão da pré-proposta internacional.)
@@ -1705,17 +1868,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional / Início dos projetos (esperado)</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>O edital é um Joint Transnational Call (JTC) 2026 da Parceria Europeia em Matérias-Primas para a Transição Verde e Digital (RAMP). A FAPES (Fundação de Amparo à Pesquisa e Inovação do Espírito Santo) participa sob o guarda-chuva do CONFAP. Cada parceiro de projeto é financiado diretamente por sua respectiva agência nacional/regional. A Comissão Europeia cofinancia os JTCs da RAMP, com o cofinanciamento sendo redistribuído pelas agências financiadoras aos seus beneficiários. A duração máxima dos projetos é de 36 meses. Propostas devem se enquadrar em um dos seis tópicos temáticos e adotar princípios de 'Safe and Sustainable by Design'. Conforme a tabela de elegibilidade de parceiros do CONFAP, empresas (SMEs e grandes) e entidades sem fins lucrativos (ONGs, associações, sociedades, fundações) não são elegíveis para financiamento pela FAPES.</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-04 09:56
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,22 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -59,18 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -438,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -540,9 +524,9 @@
           <t>EDITAL FAPES Nº 19/2026 - PIC JR 2027</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 03/08/2026</t>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1131,12 +1115,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Extensão</t>
+          <t>Inovação</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
+          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1148,105 +1132,30 @@
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo, visando a redução de desigualdades ou vulnerabilidades sociais e a promoção do desenvolvimento socioambiental e econômico nas microrregiões do estado.</t>
+          <t>Promover o aumento da competitividade dos setores econômicos capixabas por meio de projetos de inovação, desenvolvidos por empresas (incluindo cooperativas de trabalho) em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas. O apoio se dará por meio de um modelo de coinvestimento tripartite (FAPES, empresa/cooperativa, ICT/IES), com projetos alinhados ao Plano ES 500 Anos e ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Profissionais com graduação e experiência mínima de 3 anos em projetos de extensão ou titulação mínima de mestre, com vínculo empregatício, estatutário, por designação temporária ou termo de adesão a trabalho voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, e que residam no Espírito Santo ou municípios limítrofes.</t>
+          <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas ou cooperativas de trabalho capixabas.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>R$ 5.000.000,00</t>
+          <t>R$ 40.000.000,00</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>R$ 80.000,00</t>
+          <t>R$ 500.000,00 a R$ 3.000.000,00</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>editais.extensao@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-02: Data limite para submissão das propostas no Sigfapes (Até as 17h59)
-?: Prazo para submissão de recursos administrativos (habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
-?: Prazo para submissão de recursos administrativos (mérito) (05 (cinco) dias úteis a partir da publicação do resultado preliminar do mérito)
-?: Início da contratação (Até 5 (cinco) dias úteis da publicação do resultado homologado para o início do processo de contratação)</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>O prazo de execução dos projetos é de 24 meses. É obrigatória a previsão de bolsas Ext-E ou Ext-F por um período mínimo de 22 meses. As propostas devem ser submetidas para desenvolvimento em apenas uma das 10 microrregiões listadas no Quadro 2 do edital. Será concedida pontuação adicional para propostas apresentadas por pessoas pertencentes a grupos de ações afirmativas (PcD, negra, quilombola, indígena, trans ou travesti). Propostas com nota final inferior a 70 pontos serão desclassificadas.</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Inovação</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 03/08/2026</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES)." → "Promover o aumento da competitividade dos setores econômicos capixabas por meio de projetos de inovação, desenvolvidos por empresas (incluindo cooperativas de trabalho) em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas. O apoio se dará por meio de um modelo de coinvestimento tripartite (FAPES, empresa/cooperativa, ICT/IES), com projetos alinhados ao Plano ES 500 Anos e ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES)."
-Público-alvo: "Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas." → "Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas ou cooperativas de trabalho capixabas."
-Valor por proposta: "R$ 3.000.000,00" → "R$ 500.000,00 a R$ 3.000.000,00"
-Contato: "duvidas.inovacao@fapes.es.gov.br" → "duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br"
-Submissão (nova): Submissão das propostas no SIGFAPES — 2026-03-30 a ?</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Promover o aumento da competitividade dos setores econômicos capixabas por meio de projetos de inovação, desenvolvidos por empresas (incluindo cooperativas de trabalho) em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas. O apoio se dará por meio de um modelo de coinvestimento tripartite (FAPES, empresa/cooperativa, ICT/IES), com projetos alinhados ao Plano ES 500 Anos e ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas ou cooperativas de trabalho capixabas.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>R$ 40.000.000,00</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>R$ 500.000,00 a R$ 3.000.000,00</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-03-30: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 ?: Prazo de submissão dos recursos administrativos (Habilitação) (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)
@@ -1255,70 +1164,70 @@
 ?: Submissão das documentações para contratação (Até 30 dias a partir da publicação do resultado homologado do julgamento de mérito.)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução do projeto é de 24 meses, com possibilidade de prorrogação por até 12 meses. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais; cooperativas de trabalho devem apresentar Demonstração de Sobras ou Perdas (DSP). As empresas devem estar ativas há pelo menos 6 meses e não podem ter sido contratadas em editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026, a menos que o projeto, coordenador e equipe executora sejam distintos. É permitida apenas uma proposta por empresa. Em caso de inabilitação ou desclassificação, a empresa poderá realizar uma nova submissão, exceto se reprovada pelo Comitê de Conformidade, o que impede nova submissão nesta chamada. A aprovação da proposta não garante a contratação, que está sujeita à disponibilidade financeira da FAPES, ordem de submissão e visita técnica. O critério de desempate é a data de submissão da proposta no SIGFAPES. Propostas com Nota Final inferior a 80 pontos ou notas individuais inferiores a 4 em critérios específicos serão desclassificadas. A impugnação dos termos do edital deve ser feita em até 5 dias úteis antes do encerramento do prazo de submissão das propostas do primeiro ciclo (considerando o fluxo contínuo, esta observação se refere a um prazo inicial para impugnação do edital em si).</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-07-31 a 2026-08-06: Prazo de submissão de recursos administrativos (habilitação - 1ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Fomentar o empreendedorismo inovador por meio de projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou de processos inovadores. O edital visa transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica. Destina-se a doutores em qualquer área de desenvolvimento.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (até as 17:59h, via Sigfapes)
 2026-07-31 a 2026-08-06: Prazo de submissão de recursos administrativos (habilitação - 1ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)
@@ -1330,70 +1239,70 @@
 2027-04-27 a 2027-05-03: Processo de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>O edital prevê duas chamadas para submissão de propostas. Os recursos financeiros remanescentes da primeira chamada poderão ser aplicados na segunda. O prazo de execução dos projetos será de 24 meses, prorrogável por até 12 meses. A subvenção econômica inclui R$ 50.000,00 para serviços de consultoria especializada de aceleradoras. A contrapartida financeira dos outorgados será de 5% do valor subvencionado. A verificação de vínculo empregatício do proponente será realizada no ato da contratação. Para propostas onde a instituição copartícipe é uma ICT ou IES/P vinculada ao Edital FAPES nº 12/2025, o NIT deverá ser formalmente comunicado sobre a parceria, conforme Anexo IX. No ato da contratação, será exigida a apresentação da Declaração de Ciência do NIT, quando aplicável. A definição de responsabilidades quanto ao registro ou depósito de pedido de proteção intelectual caberá ao outorgado e à instituição/empresa executora, conforme suas normativas internas e legislação. O Anexo III (Declaração de Apoio da Instituição Copartícipe) agora permite assinatura por autoridade com competência formalmente delegada. Foi incluído o Anexo IX (Modelo de Declaração de Ciência do Núcleo de Inovação Tecnológica – NIT).</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-09-14 a 2026-09-22: Envio da segunda proposta após a 1ª oficina e capacitação (até as 17h59)</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>O presente edital tem como objetivo geral estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. Isso será feito por meio de apoio técnico e financeiro a soluções inovadoras com potencial para se transformarem em negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação. O edital visa estimular a criação, formalização e fortalecimento de negócios, promovendo a inovação e o empreendedorismo como estratégias para o desenvolvimento sustentável.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>R$ 30.000,00</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, comunicacao@fapes.es.gov.br, (27) 3636-1850, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-26: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)
 2026-05-21 a 2026-07-03: Envio da primeira proposta (até as 17h59)
@@ -1404,70 +1313,70 @@
 ?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Serão selecionadas 80 propostas de cada microrregião na Fase 1. Serão selecionadas 25 propostas ou mais por microrregião na Fase 2. A Fapes pode alterar as datas e os prazos definidos no cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas. O proponente poderá submeter mais de uma proposta na Fase 1, mas apenas a de maior nota será selecionada para a Fase 2, caso haja múltiplas propostas classificadas. Propostas com Nota Final inferior a 70,0 pontos serão desclassificadas em ambas as fases.</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que tenham como objetivo celebrar parcerias estratégicas com outras startups do Espírito Santo, nacionais ou internacionais. O edital busca fomentar a expansão do mercado, inovação e avanço tecnológico, aprimoramento de produtos ou serviços, acesso a novos canais ou redes de distribuição, atração de talentos e aprimoramento de competências, posicionamento de marca e mercado, acesso a oportunidades de financiamento ou investimento, e impacto socioambiental sustentável.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Startups (pessoas jurídicas) sediadas no Espírito Santo, com faturamento bruto anual de até R$ 16.000.000,00 e até 10 anos de inscrição no Cadastro Nacional da Pessoa Jurídica (CNPJ).</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>R$ 9.800.000,00</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Varia de R$ 120.000,00 a R$ 250.000,00, dependendo da modalidade de parceria (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, e R$ 250.000,00 para Modalidade III).</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)
 ?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar da habilitação. O recurso administrativo deverá ser interposto por meio do formulário específico disponível no Sistema de Automação de Fluxos do Governo do Estado (E-Flow): https://fapes.es.gov.br/formularios.)
@@ -1480,19 +1389,87 @@
 ?: Prestação de contas final (Até 30 dias após o prazo de vigência do Termo de Outorga de Subvenção Econômica.)</t>
         </is>
       </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. É permitido a cada proponente submeter até 2 (duas) propostas de parceria, desde que em modalidades diferentes e com diferentes parceiros. É vedada a submissão de propostas com as mesmas startups alternando funções de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A FAPES não exigirá direitos decorrentes de participação e propriedade nas pesquisas e projetos incentivados. A primeira parcela dos recursos será liberada após a assinatura do Termo de Outorga e comprovação do aporte da contrapartida financeira. A segunda parcela será liberada 30 dias após o 12º mês de execução, mediante prestação de contas parcial, comprovação de 70% de recursos comprometidos/executados e aporte da segunda parcela da contrapartida financeira.</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. É permitido a cada proponente submeter até 2 (duas) propostas de parceria, desde que em modalidades diferentes e com diferentes parceiros. É vedada a submissão de propostas com as mesmas startups alternando funções de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A FAPES não exigirá direitos decorrentes de participação e propriedade nas pesquisas e projetos incentivados. A primeira parcela dos recursos será liberada após a assinatura do Termo de Outorga e comprovação do aporte da contrapartida financeira. A segunda parcela será liberada 30 dias após o 12º mês de execução, mediante prestação de contas parcial, comprovação de 70% de recursos comprometidos/executados e aporte da segunda parcela da contrapartida financeira.</t>
+          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1481,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1512,32 +1489,20 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
-        </is>
-      </c>
+      <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>R$ 150.000,00</t>
-        </is>
-      </c>
+          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1545,22 +1510,22 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1572,7 +1537,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1580,43 +1545,47 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+        </is>
+      </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1628,7 +1597,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1638,45 +1607,54 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
+          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
+2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
+          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1688,7 +1666,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1696,165 +1674,96 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)</t>
-        </is>
-      </c>
+      <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>US$ 6.000,00</t>
+          <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
-2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA HORIZON EUROPE</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>€ 25.000,00 por ano de projeto</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Este edital visa financiar projetos transnacionais de pesquisa e inovação em matérias-primas para a transição verde e digital. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Organizações de ensino superior e centros de pesquisa públicos. Os consórcios devem ser compostos por, no mínimo, três parceiros de três países diferentes (sendo pelo menos dois da UE ou países associados).</t>
         </is>
       </c>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)
 2026-09-22: Submissão de propostas nacionais FAPES (Etapa 1) (Recomendado verificar requisitos da FAPES para submissão na plataforma nacional, prazo idêntico ao da submissão da pré-proposta internacional.)
@@ -1868,17 +1777,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional / Início dos projetos (esperado)</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>O edital é um Joint Transnational Call (JTC) 2026 da Parceria Europeia em Matérias-Primas para a Transição Verde e Digital (RAMP). A FAPES (Fundação de Amparo à Pesquisa e Inovação do Espírito Santo) participa sob o guarda-chuva do CONFAP. Cada parceiro de projeto é financiado diretamente por sua respectiva agência nacional/regional. A Comissão Europeia cofinancia os JTCs da RAMP, com o cofinanciamento sendo redistribuído pelas agências financiadoras aos seus beneficiários. A duração máxima dos projetos é de 36 meses. Propostas devem se enquadrar em um dos seis tópicos temáticos e adotar princípios de 'Safe and Sustainable by Design'. Conforme a tabela de elegibilidade de parceiros do CONFAP, empresas (SMEs e grandes) e entidades sem fins lucrativos (ONGs, associações, sociedades, fundações) não são elegíveis para financiamento pela FAPES.</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-05 09:51
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1038,46 +1046,123 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
+          <t>EDITAL FAPES N° 25/2025 - PARTICIPAÇÃO DE EQUIPES DE ESTUDANTES EM MOSTRAS E COMPETIÇÕES TÉCNICO-CIENTÍFICAS</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Sem alteracoes</t>
+          <t>Removido (nao mais aberto)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 a 2026-08-25: Submissão de propostas - 3ª Chamada (Até as 17h59)</t>
+          <t>2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
+          <t>Conceder apoio financeiro a equipes formadas por estudantes de nível médio, de graduação e pós-graduação, coordenadas por um professor orientador. O objetivo é permitir a participação dessas equipes em mostras e competições técnico-científicas de âmbito regional, nacional ou internacional, visando a divulgação e difusão de resultados obtidos por instituições de ensino do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Professores(as) coordenadores(as) de equipes de 3 a 5 estudantes, vinculados(as) a instituições de ensino médio públicas ou instituições de ensino superior públicas ou privadas localizadas no estado do Espírito Santo. O proponente deve ter formação mínima de nível superior, vínculo ativo com a instituição, atuar em sala de aula na mesma instituição dos estudantes, ter Lattes atualizado há menos de 6 meses, estar regularizado junto à Fapes e morar no Espírito Santo ou municípios limítrofes. Estudantes de instituições privadas devem ser bolsistas integrais financiados por programas governamentais estaduais ou federais.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 500.000,00</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>US$ 1.500,00</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>?: Prazo para impugnação do edital (5 dias úteis antes do encerramento do prazo de submissão da 1ª Chamada)
+2025-11-10 a 2025-12-16: Submissão de propostas (Até as 17h:59. Para 1ª Chamada (eventos com início entre 01/03/2026 a 30/06/2026))
+?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar. Para 1ª Chamada (eventos com início entre 01/03/2026 a 30/06/2026))
+2026-03-04 a 2026-04-09: Submissão de propostas (Até as 17:59h. Para 2ª Chamada (eventos com início entre 01/07/2026 a 31/12/2026))
+?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar. Para 2ª Chamada (eventos com início entre 01/07/2026 a 31/12/2026))
+2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))
+?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))
+?: Contratação e assinatura do Termo de Outorga (Até 30 dias após a publicação do resultado final homologado. Período específico de assinatura será definido após a homologação.)
+?: Prazo para informar dados bancários (Até 30 dias após a assinatura e publicação do Termo de Outorga)
+?: Prazo para prestação de contas (Até 30 dias após o término da vigência do Termo de Outorga)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>O valor por proposta varia conforme a categoria do evento: R$ 500,00 para eventos regionais, R$ 1.200,00 para eventos nacionais e US$ 1.500,00 para eventos internacionais. O edital prevê três chamadas com períodos de submissão e eventos distintos. O início do evento proposto deve corresponder ao período da chamada selecionada. A Fapes pode alterar as datas e prazos definidos no cronograma. Cada coordenador pode apresentar apenas uma proposta. Não são contempladas propostas para participação em concursos ou premiações sem natureza acadêmica, técnico-científica ou tecnológica, ou competições esportivas.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_N_25_2025_Participação_Equipe_em_Mostras_e_Competições-2.pdf</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_N°_25_2025_-_PARTICIPAÇÃO_DE_EQUIPES_DE_ESTUDANTES_EM_MOSTRAS_E_COMPETIÇÕES_TÉCNICO-CIENTÍFICAS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19 a 2026-08-25: Submissão de propostas - 3ª Chamada (Até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
 2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
@@ -1096,66 +1181,66 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Promover o aumento da competitividade dos setores econômicos capixabas por meio de projetos de inovação, desenvolvidos por empresas (incluindo cooperativas de trabalho) em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas. O apoio se dará por meio de um modelo de coinvestimento tripartite (FAPES, empresa/cooperativa, ICT/IES), com projetos alinhados ao Plano ES 500 Anos e ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas ou cooperativas de trabalho capixabas.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 500.000,00 a R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-03-30: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 ?: Prazo de submissão dos recursos administrativos (Habilitação) (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)
@@ -1164,94 +1249,19 @@
 ?: Submissão das documentações para contratação (Até 30 dias a partir da publicação do resultado homologado do julgamento de mérito.)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução do projeto é de 24 meses, com possibilidade de prorrogação por até 12 meses. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais; cooperativas de trabalho devem apresentar Demonstração de Sobras ou Perdas (DSP). As empresas devem estar ativas há pelo menos 6 meses e não podem ter sido contratadas em editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026, a menos que o projeto, coordenador e equipe executora sejam distintos. É permitida apenas uma proposta por empresa. Em caso de inabilitação ou desclassificação, a empresa poderá realizar uma nova submissão, exceto se reprovada pelo Comitê de Conformidade, o que impede nova submissão nesta chamada. A aprovação da proposta não garante a contratação, que está sujeita à disponibilidade financeira da FAPES, ordem de submissão e visita técnica. O critério de desempate é a data de submissão da proposta no SIGFAPES. Propostas com Nota Final inferior a 80 pontos ou notas individuais inferiores a 4 em critérios específicos serão desclassificadas. A impugnação dos termos do edital deve ser feita em até 5 dias úteis antes do encerramento do prazo de submissão das propostas do primeiro ciclo (considerando o fluxo contínuo, esta observação se refere a um prazo inicial para impugnação do edital em si).</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Inovação</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-31 a 2026-08-06: Prazo de submissão de recursos administrativos (habilitação - 1ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Fomentar o empreendedorismo inovador por meio de projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou de processos inovadores. O edital visa transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica. Destina-se a doutores em qualquer área de desenvolvimento.</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>R$ 10.662.000,00</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>R$ 355.400,00</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (até as 17:59h, via Sigfapes)
-2026-07-31 a 2026-08-06: Prazo de submissão de recursos administrativos (habilitação - 1ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)
-2026-10-02 a 2026-10-08: Prazo de submissão de recursos administrativos (mérito e apresentação oral - 1ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)
-2026-10-14 a 2026-12-15: Período de submissão de propostas (2ª chamada) (até as 17:59h, via Sigfapes)
-2026-10-27 a 2026-10-31: Processo de contratação (1ª chamada) (Até 5 dias úteis da publicação do resultado homologado)
-2027-01-08 a 2027-01-14: Prazo de submissão de recursos administrativos (habilitação - 2ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)
-2027-03-19 a 2027-03-25: Prazo de submissão de recursos administrativos (mérito e apresentação oral - 2ª chamada) (5 dias úteis a partir do 1º dia de publicação do resultado preliminar)
-2027-04-27 a 2027-05-03: Processo de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>O edital prevê duas chamadas para submissão de propostas. Os recursos financeiros remanescentes da primeira chamada poderão ser aplicados na segunda. O prazo de execução dos projetos será de 24 meses, prorrogável por até 12 meses. A subvenção econômica inclui R$ 50.000,00 para serviços de consultoria especializada de aceleradoras. A contrapartida financeira dos outorgados será de 5% do valor subvencionado. A verificação de vínculo empregatício do proponente será realizada no ato da contratação. Para propostas onde a instituição copartícipe é uma ICT ou IES/P vinculada ao Edital FAPES nº 12/2025, o NIT deverá ser formalmente comunicado sobre a parceria, conforme Anexo IX. No ato da contratação, será exigida a apresentação da Declaração de Ciência do NIT, quando aplicável. A definição de responsabilidades quanto ao registro ou depósito de pedido de proteção intelectual caberá ao outorgado e à instituição/empresa executora, conforme suas normativas internas e legislação. O Anexo III (Declaração de Apoio da Instituição Copartícipe) agora permite assinatura por autoridade com competência formalmente delegada. Foi incluído o Anexo IX (Modelo de Declaração de Ciência do Núcleo de Inovação Tecnológica – NIT).</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1273,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
+          <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1271,112 +1281,34 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14 a 2026-09-22: Envio da segunda proposta após a 1ª oficina e capacitação (até as 17h59)</t>
-        </is>
-      </c>
+      <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>O presente edital tem como objetivo geral estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. Isso será feito por meio de apoio técnico e financeiro a soluções inovadoras com potencial para se transformarem em negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação. O edital visa estimular a criação, formalização e fortalecimento de negócios, promovendo a inovação e o empreendedorismo como estratégias para o desenvolvimento sustentável.</t>
+          <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que tenham como objetivo celebrar parcerias estratégicas com outras startups do Espírito Santo, nacionais ou internacionais. O edital busca fomentar a expansão do mercado, inovação e avanço tecnológico, aprimoramento de produtos ou serviços, acesso a novos canais ou redes de distribuição, atração de talentos e aprimoramento de competências, posicionamento de marca e mercado, acesso a oportunidades de financiamento ou investimento, e impacto socioambiental sustentável.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
+          <t>Startups (pessoas jurídicas) sediadas no Espírito Santo, com faturamento bruto anual de até R$ 16.000.000,00 e até 10 anos de inscrição no Cadastro Nacional da Pessoa Jurídica (CNPJ).</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>R$ 4.500.000,00</t>
+          <t>R$ 9.800.000,00</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>R$ 30.000,00</t>
+          <t>Varia de R$ 120.000,00 a R$ 250.000,00, dependendo da modalidade de parceria (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, e R$ 250.000,00 para Modalidade III).</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>duvidas.inovacao@fapes.es.gov.br, comunicacao@fapes.es.gov.br, (27) 3636-1850, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-21 a 2026-06-26: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)
-2026-05-21 a 2026-07-03: Envio da primeira proposta (até as 17h59)
-?: Prazo para recurso administrativo (Fase 1) (Até 5 dias úteis após divulgação do resultado preliminar)
-2026-09-14 a 2026-09-22: Envio da segunda proposta após a 1ª oficina e capacitação (até as 17h59)
-2026-09-21 a 2026-09-30: Apresentação do pitch
-?: Prazo para recurso administrativo (Fase 2) (Até 5 dias úteis após divulgação do resultado preliminar)
-?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>Serão selecionadas 80 propostas de cada microrregião na Fase 1. Serão selecionadas 25 propostas ou mais por microrregião na Fase 2. A Fapes pode alterar as datas e os prazos definidos no cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas. O proponente poderá submeter mais de uma proposta na Fase 1, mas apenas a de maior nota será selecionada para a Fase 2, caso haja múltiplas propostas classificadas. Propostas com Nota Final inferior a 70,0 pontos serão desclassificadas em ambas as fases.</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Inovação</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que tenham como objetivo celebrar parcerias estratégicas com outras startups do Espírito Santo, nacionais ou internacionais. O edital busca fomentar a expansão do mercado, inovação e avanço tecnológico, aprimoramento de produtos ou serviços, acesso a novos canais ou redes de distribuição, atração de talentos e aprimoramento de competências, posicionamento de marca e mercado, acesso a oportunidades de financiamento ou investimento, e impacto socioambiental sustentável.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Startups (pessoas jurídicas) sediadas no Espírito Santo, com faturamento bruto anual de até R$ 16.000.000,00 e até 10 anos de inscrição no Cadastro Nacional da Pessoa Jurídica (CNPJ).</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>R$ 9.800.000,00</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>Varia de R$ 120.000,00 a R$ 250.000,00, dependendo da modalidade de parceria (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, e R$ 250.000,00 para Modalidade III).</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)
 ?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar da habilitação. O recurso administrativo deverá ser interposto por meio do formulário específico disponível no Sistema de Automação de Fluxos do Governo do Estado (E-Flow): https://fapes.es.gov.br/formularios.)
@@ -1389,19 +1321,83 @@
 ?: Prestação de contas final (Até 30 dias após o prazo de vigência do Termo de Outorga de Subvenção Econômica.)</t>
         </is>
       </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. É permitido a cada proponente submeter até 2 (duas) propostas de parceria, desde que em modalidades diferentes e com diferentes parceiros. É vedada a submissão de propostas com as mesmas startups alternando funções de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A FAPES não exigirá direitos decorrentes de participação e propriedade nas pesquisas e projetos incentivados. A primeira parcela dos recursos será liberada após a assinatura do Termo de Outorga e comprovação do aporte da contrapartida financeira. A segunda parcela será liberada 30 dias após o 12º mês de execução, mediante prestação de contas parcial, comprovação de 70% de recursos comprometidos/executados e aporte da segunda parcela da contrapartida financeira.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP CDTI 2026</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 05/08/2026</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>€ 75.000,00</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
+        </is>
+      </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. É permitido a cada proponente submeter até 2 (duas) propostas de parceria, desde que em modalidades diferentes e com diferentes parceiros. É vedada a submissão de propostas com as mesmas startups alternando funções de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A FAPES não exigirá direitos decorrentes de participação e propriedade nas pesquisas e projetos incentivados. A primeira parcela dos recursos será liberada após a assinatura do Termo de Outorga e comprovação do aporte da contrapartida financeira. A segunda parcela será liberada 30 dias após o 12º mês de execução, mediante prestação de contas parcial, comprovação de 70% de recursos comprometidos/executados e aporte da segunda parcela da contrapartida financeira.</t>
+          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-06 09:55
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -38,7 +38,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -1276,13 +1276,23 @@
           <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 06/08/2026</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18: Prazo de submissão de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Público-alvo: "Startups (pessoas jurídicas) sediadas no Espírito Santo, com faturamento bruto anual de até R$ 16.000.000,00 e até 10 anos de inscrição no Cadastro Nacional da Pessoa Jurídica (CNPJ)." → "Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo, e com CNPJ constituído há no mínimo 1 ano e no máximo 10 anos, que atendam aos requisitos do edital."
+Valor por proposta: "Varia de R$ 120.000,00 a R$ 250.000,00, dependendo da modalidade de parceria (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, e R$ 250.000,00 para Modalidade III)." → "Varia por modalidade: R$ 120.000,00 (Modalidade I), R$ 150.000,00 (Modalidade II), R$ 250.000,00 (Modalidade III)."
+Contato: "duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br" → "duvidas.inovacao@fapes.es.gov.br"</t>
+        </is>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que tenham como objetivo celebrar parcerias estratégicas com outras startups do Espírito Santo, nacionais ou internacionais. O edital busca fomentar a expansão do mercado, inovação e avanço tecnológico, aprimoramento de produtos ou serviços, acesso a novos canais ou redes de distribuição, atração de talentos e aprimoramento de competências, posicionamento de marca e mercado, acesso a oportunidades de financiamento ou investimento, e impacto socioambiental sustentável.</t>
@@ -1290,7 +1300,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Startups (pessoas jurídicas) sediadas no Espírito Santo, com faturamento bruto anual de até R$ 16.000.000,00 e até 10 anos de inscrição no Cadastro Nacional da Pessoa Jurídica (CNPJ).</t>
+          <t>Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo, e com CNPJ constituído há no mínimo 1 ano e no máximo 10 anos, que atendam aos requisitos do edital.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1300,30 +1310,25 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Varia de R$ 120.000,00 a R$ 250.000,00, dependendo da modalidade de parceria (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, e R$ 250.000,00 para Modalidade III).</t>
+          <t>Varia por modalidade: R$ 120.000,00 (Modalidade I), R$ 150.000,00 (Modalidade II), R$ 250.000,00 (Modalidade III).</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)
-?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar da habilitação. O recurso administrativo deverá ser interposto por meio do formulário específico disponível no Sistema de Automação de Fluxos do Governo do Estado (E-Flow): https://fapes.es.gov.br/formularios.)
-?: Constituição de empresa e atualização documental no SIGFAPES (Para proponentes aprovados. Prazo até as 17h. Abertura da empresa/anexar os documentos no SIGFAPES. Datas são placeholders no edital.)
-?: Assinatura do Termo de Outorga e do Projeto Aprovado (Para proponentes aprovados. Prazo até as 17h. Necessário cadastro no portal 'Acesso Cidadão' e no 'E-DOCS' do Governo do Estado (www.acessocidadao.es.gov.br). Datas são placeholders no edital.)
-?: Constituição de empresa e atualização documental no SIGFAPES (Suplentes) (Para suplentes. Prazo até as 17h. Datas são placeholders no edital.)
-?: Assinatura do Termo de Outorga e do Projeto Aprovado (Suplentes) (Para suplentes. Prazo até as 17h. Datas são placeholders no edital.)
-?: Abertura de conta corrente para recebimento de recursos (O(a) outorgado(a) terá o prazo de 30 (trinta) dias a partir do início da vigência do Termo de Outorga para informar à Fapes os dados da conta bancária aberta, a contar da data da publicação da contratação do projeto no DIO-ES. A conta deve ser aberta no Banco Banestes.)
-?: Prestação de contas parcial (Até 30 dias após o 12º mês de vigência do Termo de Outorga de Subvenção Econômica.)
-?: Prestação de contas final (Até 30 dias após o prazo de vigência do Termo de Outorga de Subvenção Econômica.)</t>
+          <t>2026-07-28: Prazo para impugnação do edital (Até 5 dias úteis antes da data final de submissão das propostas.)
+2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)
+2026-08-18: Prazo de submissão de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)
+2026-12-01 a 2026-12-30: Prazo para informar dados da conta bancária (30 dias a partir do início da vigência do Termo de Outorga para informar dados da conta bancária aberta no Banco Banestes.)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. É permitido a cada proponente submeter até 2 (duas) propostas de parceria, desde que em modalidades diferentes e com diferentes parceiros. É vedada a submissão de propostas com as mesmas startups alternando funções de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A FAPES não exigirá direitos decorrentes de participação e propriedade nas pesquisas e projetos incentivados. A primeira parcela dos recursos será liberada após a assinatura do Termo de Outorga e comprovação do aporte da contrapartida financeira. A segunda parcela será liberada 30 dias após o 12º mês de execução, mediante prestação de contas parcial, comprovação de 70% de recursos comprometidos/executados e aporte da segunda parcela da contrapartida financeira.</t>
+          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital no site da FAPES. Cada proponente pode submeter até 2 propostas de parceria, em modalidades diferentes e com parceiros distintos. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A contratação exige adimplência do coordenador e da empresa com FAPES, Fazendas Públicas (Federal, Estadual, Municipal), Justiça Trabalhista, INSS e FGTS. A primeira parcela será liberada após assinatura e publicação do Termo de Outorga e comprovação do aporte da contrapartida financeira. A segunda parcela será liberada 30 dias após o 12º mês de execução, mediante prestação de contas parcial e comprovação de execução mínima de 70% dos recursos. É obrigatória a referência ao apoio da FAPES em divulgações, exceto em período eleitoral. A FAPES não exigirá direitos de propriedade intelectual decorrentes dos projetos incentivados. Erros de menor relevância na proposta ou documentação podem ser saneados a critério da FAPES, desde que não prejudiquem a avaliação de mérito. Não serão admitidas alterações nos documentos enviados após a submissão da proposta.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -1348,9 +1353,9 @@
           <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 05/08/2026</t>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-07 08:41
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -38,7 +38,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -664,51 +664,122 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Difusão do Conhecimento</t>
+          <t>Pesquisa</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
+          <t>EDITAL FAPES Nº 21/2026 - REDES DE PESQUISA, DESENVOLVIMENTO E INOVAÇÃO EM SETORES ESTRATÉGICOS</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 07/08/2026</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)</t>
+          <t>2026-09-10: Envio de dúvidas sobre o edital (Até as 17h59)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
+          <t>O edital Redes de Pesquisa, Desenvolvimento e Inovação (PD&amp;I) em Setores Estratégicos da Fapes tem como finalidade apoiar financeiramente a criação e o fortalecimento de redes que promovam ações coletivas de PD&amp;I. O objetivo geral é selecionar projetos para criar e fortalecer redes estruturantes de PD&amp;I em setores estratégicos e de interesse do Espírito Santo, consolidando grupos de referência em áreas do conhecimento.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores doutores vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo, que atuem como coordenadores de propostas.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>R$ 12.000.000,00</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>R$ 1.200.000,00</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10: Envio de dúvidas sobre o edital (Até as 17h59)
+2026-08-07 a 2026-09-14: Submissão de propostas (Até as 17h59, via SigFapes)
+?: Interposição de recursos (habilitação) (Até 5 dias úteis após a divulgação do resultado preliminar da habilitação)
+?: Interposição de recursos (análise de mérito) (Até 5 dias úteis após a divulgação do resultado preliminar da análise de mérito)</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>As propostas devem ter prazo de execução de até 36 meses e prever no orçamento 1 bolsista pós-doutorado (POSDOC) e 1 estudante de graduação (ICT). As linhas temáticas incluem: Saúde Única, Saúde de Precisão, Imunobiológicos e Biofármacos, Preservação e Restauração ecológica do bioma da Mata Atlântica, Transformação digital e rastreabilidade ambiental, Economia Circular e Soberania digital e cibersegurança. A equipe executora deve ser exclusiva e composta por no mínimo 7 pesquisadores além do coordenador, com distribuição específica de doutores de diferentes IES/P e um pesquisador de órgão público estadual. Os recursos serão distribuídos garantindo ao menos uma proposta contemplada por linha temática, e as demais por ordem decrescente de nota final. Somente propostas com nota final igual ou superior a 70,0 pontos serão classificadas. Despesas de custeio com serviços de terceiros são limitadas a 30% do valor máximo por proposta. Despesas de capital financiáveis devem ter vida útil superior a dois anos e valor superior a 80 VRTEs. Não são financiáveis mobiliário (exceto se indispensável à pesquisa) e veículos motorizados (exceto se objeto da pesquisa).</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_21-2026_-_Redes_de_PDI_em_Setores_Estratégicos.pdf</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>pesquisa/EDITAL_FAPES_No_21_2026_-_REDES_DE_PESQUISA,_DESENVOLVIMENTO_E_INOVAÇÃO_EM_SETORES_ESTRATÉGICOS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Removido (nao mais aberto)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>O objetivo geral deste edital é selecionar e apoiar financeiramente pesquisadores e alunos para participação em eventos técnico-científicos de curta duração. Visa divulgar os resultados de projetos de pesquisa, desenvolvimento e inovação (P, D&amp;I) desenvolvidos em instituições de ensino superior e/ou pesquisa, públicas ou privadas, localizadas no Estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores e alunos de pós-graduação vinculados a Instituição de Ensino e/ou Pesquisa (IES/P), pública ou privada, localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>R$ 2.500.000,00</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>US$ 2.700,00</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>2026-02-27: Prazo para solicitação de atendimento especializado (até 10 dias antes do prazo final de submissão da 1ª Chamada)
 2026-03-02: Prazo para impugnação do edital (até 5 dias úteis antes do prazo final de submissão da 1ª Chamada)
@@ -723,70 +794,70 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 3ª Chamada)</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>O valor total do edital será distribuído em três chamadas. O valor por proposta é fixo e varia conforme o local do evento: R$ 1.800,00 para eventos no Brasil (exceto Espírito Santo), US$ 1.400,00 para América Central ou América do Sul, US$ 2.300,00 para América do Norte e US$ 2.700,00 para outros continentes. A Fapes pode alterar as datas e prazos do cronograma. Cada proponente pode apresentar apenas uma proposta por chamada. O prazo para informar dados bancários é de até 30 dias corridos após o início da vigência do Termo de Outorga. O prazo para envio da prestação de contas é de até 30 dias após o término da vigência do Termo de Outorga. A contratação das propostas aprovadas ocorrerá em até 30 dias após a publicação do resultado final homologado. O envio do comprovante de aceite do trabalho é condicional para o repasse do recurso e deve ser feito até 15 dias antes do evento.</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_02-2026-Participação_Evento_Técnico_Científico.pdf</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_02_2026_-_PARTICIPAÇÃO_EM_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 03/2026 - ORGANIZAÇÃO DE EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 3ª chamada)</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Este edital visa selecionar propostas para conceder apoio financeiro a pesquisadores de nível superior. O objetivo é fomentar a organização de eventos técnico-científicos de curta duração, como congressos, simpósios e seminários, a serem realizados no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores de nível superior vinculados a Instituição de Ensino Superior e/ou Pesquisa (IES/P), pública ou privada sem fins lucrativos, localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 2.500.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Varia de R$ 10.000,00 a R$ 35.000,00</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-03-02: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada)
 2026-02-06 a 2026-03-09: 1ª Chamada - Período de submissão de propostas (Eventos com início entre 01/05/2026 a 31/07/2026, até 17h59)
@@ -801,66 +872,66 @@
 ?: Contratação das propostas aprovadas (Até 30 dias após a publicação do resultado final homologado para cada chamada. As datas exatas serão publicadas posteriormente.)</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>O valor do auxílio financeiro é fixo e varia de acordo com o nível do evento: R$ 10.000,00 para Estadual/Regional, R$ 20.000,00 para Nacional e R$ 35.000,00 para Internacional. A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional. Cada proponente pode apresentar apenas uma proposta por chamada. Caso envie mais de uma, será considerada apenas a última enviada. O proponente que já tiver sido contratado neste edital não poderá submeter nova proposta. O evento deve ter duração máxima de 15 dias, consecutivos ou não, e ser chancelado por entidade/sociedade conforme o nível do evento (nacional ou internacional). Os recursos financeiros estão distribuídos por chamada e nível de evento, com possibilidade de remanejamento de saldos não utilizados entre níveis e chamadas subsequentes. É obrigatório mencionar o apoio da Fapes em todas as publicações e divulgações relacionadas ao projeto. A data de início do apoio poderá ser adiada, após a contratação, em até 12 meses, mediante justificativa.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_03_2026_Organização_Eventos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_03_2026_-_ORGANIZAÇÃO_DE_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO-CIENTÍFICO</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão.)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Selecionar propostas para concessão de auxílio financeiro para estágios técnico-científicos em laboratórios ou centros de PD&amp;I, no Brasil ou exterior. O objetivo é aprimorar técnicas, adquirir conhecimentos específicos para projetos de PD&amp;I no Espírito Santo, estimular o intercâmbio de conhecimentos, a formação de pós-graduandos e apoiar os Programas de Pós-graduação do estado.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas localizadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P localizadas no Espírito Santo, reconhecidos pela CAPES/CNE/MEC.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geped@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-03-05: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada.)
 2026-02-09 a 2026-03-12: 1ª Chamada - Período de submissão de propostas (Para estágios com início entre 01/05/2026 a 31/07/2026, até as 17h59.)
@@ -874,70 +945,70 @@
 2026-10-03 a 2026-10-09: 3ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>O valor por proposta varia conforme o nível (duração do estágio) e a localização (Brasil - Região Sudeste, Brasil - Demais Estados, Exterior - América Central e do Sul, Exterior - América do Norte, Exterior - Demais Continentes), conforme tabela na seção 6.4 e 6.5 do edital. A Fapes pode alterar as datas e prazos do cronograma, reabrir prazos em casos de força maior ou falhas de sistema, e dará publicidade a essas alterações. Recursos financeiros não utilizados em uma chamada podem ser aplicados em chamadas subsequentes. O beneficiário não poderá utilizar outros recursos da Fapes para cobrir despesas do estágio se o auxílio concedido for insuficiente. Auxílios em moeda estrangeira serão convertidos com base no câmbio oficial na data de aprovação. Cada proponente pode apresentar apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Não é permitida a contratação concomitante de estágio técnico-científico e visita técnico-científica para o mesmo período/chamada. O edital pode ser revogado ou anulado sem direito a indenização. Casos omissos e dúvidas de interpretação serão dirimidos pela Diretoria Executiva da Fapes.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_04_2026_-_Estágio_Técnico_Cientifico.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_04_2026_-_ESTÁGIO_TÉCNICO-CIENTÍFICO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Selecionar propostas para concessão de auxílio financeiro para a realização de visitas técnico-científicas em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, processos e adquirir conhecimentos específicos para projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>US$ 2.600,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-02-09 a 2026-03-12: Submissão de propostas (1ª Chamada) (Até as 17h59. Para visitas com início entre 01/05/2026 a 31/07/2026.)
 2026-03-05: Prazo final para impugnação do edital (Até o quinto dia útil que anteceder o prazo final de submissão da 1ª Chamada.)
@@ -951,70 +1022,70 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade institucional, podendo reabrir prazos em casos de força maior ou falhas de sistema, com publicidade das alterações. Cada proponente pode submeter apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Proponentes já contratados neste edital não poderão submeter nova proposta. Após a contratação, o beneficiário pode solicitar adiamento da data de início da visita por até 30 dias, mediante justificativa e autorização. Não será permitida a alteração da instituição de destino da visita técnico-científica após a contratação.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2005_2026%20-%20Visita%20Técnico%20Cientifica%20(1).pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_05_2026_-_VISITA_TÉCNICO-CIENTÍFICA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59. A matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação, valorizando a relevância e o impacto da ciência, tecnologia e inovação para o desenvolvimento do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos fomentados.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 308.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)
 2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59. A matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.)
@@ -1022,70 +1093,70 @@
 2026-11-03 a 2026-11-09: Votação popular – Categoria Jornalismo</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>Edição em homenagem à Professora Jurema José de Oliveira. Os valores das premiações possuem natureza bruta e estão sujeitos à incidência do Imposto de Renda Retido na Fonte – IRRF, na forma da legislação tributária vigente. A premiação prevista neste edital possui caráter exclusivamente honorífico, meritório e eventual, destinando-se ao reconhecimento institucional dos trabalhos classificados. A Fapes pode alterar datas e prazos do cronograma por necessidade administrativa ou decisão institucional. O comparecimento do premiado é obrigatório. Caso não possa comparecer, deve indicar formalmente um representante para o recebimento da premiação, com comunicação prévia à Fapes, pelo e-mail gabinete@fapes.es.gov.br. Para as categorias Projetos e Destaque, as 3 (três) propostas com as maiores notas seguem para votação pelo Comitê de Especialistas. Para a categoria Jornalismo, as 3 (três) matérias com maiores notas seguem para votação popular.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 25/2025 - PARTICIPAÇÃO DE EQUIPES DE ESTUDANTES EM MOSTRAS E COMPETIÇÕES TÉCNICO-CIENTÍFICAS</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Conceder apoio financeiro a equipes formadas por estudantes de nível médio, de graduação e pós-graduação, coordenadas por um professor orientador. O objetivo é permitir a participação dessas equipes em mostras e competições técnico-científicas de âmbito regional, nacional ou internacional, visando a divulgação e difusão de resultados obtidos por instituições de ensino do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Professores(as) coordenadores(as) de equipes de 3 a 5 estudantes, vinculados(as) a instituições de ensino médio públicas ou instituições de ensino superior públicas ou privadas localizadas no estado do Espírito Santo. O proponente deve ter formação mínima de nível superior, vínculo ativo com a instituição, atuar em sala de aula na mesma instituição dos estudantes, ter Lattes atualizado há menos de 6 meses, estar regularizado junto à Fapes e morar no Espírito Santo ou municípios limítrofes. Estudantes de instituições privadas devem ser bolsistas integrais financiados por programas governamentais estaduais ou federais.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 500.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>?: Prazo para impugnação do edital (5 dias úteis antes do encerramento do prazo de submissão da 1ª Chamada)
 2025-11-10 a 2025-12-16: Submissão de propostas (Até as 17h:59. Para 1ª Chamada (eventos com início entre 01/03/2026 a 30/06/2026))
@@ -1099,70 +1170,70 @@
 ?: Prazo para prestação de contas (Até 30 dias após o término da vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O valor por proposta varia conforme a categoria do evento: R$ 500,00 para eventos regionais, R$ 1.200,00 para eventos nacionais e US$ 1.500,00 para eventos internacionais. O edital prevê três chamadas com períodos de submissão e eventos distintos. O início do evento proposto deve corresponder ao período da chamada selecionada. A Fapes pode alterar as datas e prazos definidos no cronograma. Cada coordenador pode apresentar apenas uma proposta. Não são contempladas propostas para participação em concursos ou premiações sem natureza acadêmica, técnico-científica ou tecnológica, ou competições esportivas.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_N_25_2025_Participação_Equipe_em_Mostras_e_Competições-2.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_N°_25_2025_-_PARTICIPAÇÃO_DE_EQUIPES_DE_ESTUDANTES_EM_MOSTRAS_E_COMPETIÇÕES_TÉCNICO-CIENTÍFICAS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-06-19 a 2026-08-25: Submissão de propostas - 3ª Chamada (Até as 17h59)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
 2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
@@ -1181,66 +1252,66 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Promover o aumento da competitividade dos setores econômicos capixabas por meio de projetos de inovação, desenvolvidos por empresas (incluindo cooperativas de trabalho) em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas. O apoio se dará por meio de um modelo de coinvestimento tripartite (FAPES, empresa/cooperativa, ICT/IES), com projetos alinhados ao Plano ES 500 Anos e ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas ou cooperativas de trabalho capixabas.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>R$ 500.000,00 a R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-03-30: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 ?: Prazo de submissão dos recursos administrativos (Habilitação) (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)
@@ -1249,76 +1320,70 @@
 ?: Submissão das documentações para contratação (Até 30 dias a partir da publicação do resultado homologado do julgamento de mérito.)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução do projeto é de 24 meses, com possibilidade de prorrogação por até 12 meses. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais; cooperativas de trabalho devem apresentar Demonstração de Sobras ou Perdas (DSP). As empresas devem estar ativas há pelo menos 6 meses e não podem ter sido contratadas em editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026, a menos que o projeto, coordenador e equipe executora sejam distintos. É permitida apenas uma proposta por empresa. Em caso de inabilitação ou desclassificação, a empresa poderá realizar uma nova submissão, exceto se reprovada pelo Comitê de Conformidade, o que impede nova submissão nesta chamada. A aprovação da proposta não garante a contratação, que está sujeita à disponibilidade financeira da FAPES, ordem de submissão e visita técnica. O critério de desempate é a data de submissão da proposta no SIGFAPES. Propostas com Nota Final inferior a 80 pontos ou notas individuais inferiores a 4 em critérios específicos serão desclassificadas. A impugnação dos termos do edital deve ser feita em até 5 dias úteis antes do encerramento do prazo de submissão das propostas do primeiro ciclo (considerando o fluxo contínuo, esta observação se refere a um prazo inicial para impugnação do edital em si).</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 06/08/2026</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: Prazo de submissão de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Público-alvo: "Startups (pessoas jurídicas) sediadas no Espírito Santo, com faturamento bruto anual de até R$ 16.000.000,00 e até 10 anos de inscrição no Cadastro Nacional da Pessoa Jurídica (CNPJ)." → "Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo, e com CNPJ constituído há no mínimo 1 ano e no máximo 10 anos, que atendam aos requisitos do edital."
-Valor por proposta: "Varia de R$ 120.000,00 a R$ 250.000,00, dependendo da modalidade de parceria (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, e R$ 250.000,00 para Modalidade III)." → "Varia por modalidade: R$ 120.000,00 (Modalidade I), R$ 150.000,00 (Modalidade II), R$ 250.000,00 (Modalidade III)."
-Contato: "duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br" → "duvidas.inovacao@fapes.es.gov.br"</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que tenham como objetivo celebrar parcerias estratégicas com outras startups do Espírito Santo, nacionais ou internacionais. O edital busca fomentar a expansão do mercado, inovação e avanço tecnológico, aprimoramento de produtos ou serviços, acesso a novos canais ou redes de distribuição, atração de talentos e aprimoramento de competências, posicionamento de marca e mercado, acesso a oportunidades de financiamento ou investimento, e impacto socioambiental sustentável.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo, e com CNPJ constituído há no mínimo 1 ano e no máximo 10 anos, que atendam aos requisitos do edital.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>R$ 9.800.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Varia por modalidade: R$ 120.000,00 (Modalidade I), R$ 150.000,00 (Modalidade II), R$ 250.000,00 (Modalidade III).</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2026-07-28: Prazo para impugnação do edital (Até 5 dias úteis antes da data final de submissão das propostas.)
 2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)
@@ -1326,83 +1391,19 @@
 2026-12-01 a 2026-12-30: Prazo para informar dados da conta bancária (30 dias a partir do início da vigência do Termo de Outorga para informar dados da conta bancária aberta no Banco Banestes.)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital no site da FAPES. Cada proponente pode submeter até 2 propostas de parceria, em modalidades diferentes e com parceiros distintos. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A contratação exige adimplência do coordenador e da empresa com FAPES, Fazendas Públicas (Federal, Estadual, Municipal), Justiça Trabalhista, INSS e FGTS. A primeira parcela será liberada após assinatura e publicação do Termo de Outorga e comprovação do aporte da contrapartida financeira. A segunda parcela será liberada 30 dias após o 12º mês de execução, mediante prestação de contas parcial e comprovação de execução mínima de 70% dos recursos. É obrigatória a referência ao apoio da FAPES em divulgações, exceto em período eleitoral. A FAPES não exigirá direitos de propriedade intelectual decorrentes dos projetos incentivados. Erros de menor relevância na proposta ou documentação podem ser saneados a critério da FAPES, desde que não prejudiquem a avaliação de mérito. Não serão admitidas alterações nos documentos enviados após a submissão da proposta.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>€ 75.000,00</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1415,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1424,53 +1425,49 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
+          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1482,7 +1479,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1490,20 +1487,32 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1511,22 +1520,22 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
+          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1538,7 +1547,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1546,47 +1555,43 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
+      <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1598,7 +1603,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1608,163 +1613,223 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA ERC-CONFAP 2026</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
           <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>US$ 18.000,00</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>US$ 6.000,00</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
 2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Este edital visa financiar projetos transnacionais de pesquisa e inovação em matérias-primas para a transição verde e digital. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Organizações de ensino superior e centros de pesquisa públicos. Os consórcios devem ser compostos por, no mínimo, três parceiros de três países diferentes (sendo pelo menos dois da UE ou países associados).</t>
         </is>
       </c>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)
 2026-09-22: Submissão de propostas nacionais FAPES (Etapa 1) (Recomendado verificar requisitos da FAPES para submissão na plataforma nacional, prazo idêntico ao da submissão da pré-proposta internacional.)
@@ -1778,17 +1843,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional / Início dos projetos (esperado)</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>O edital é um Joint Transnational Call (JTC) 2026 da Parceria Europeia em Matérias-Primas para a Transição Verde e Digital (RAMP). A FAPES (Fundação de Amparo à Pesquisa e Inovação do Espírito Santo) participa sob o guarda-chuva do CONFAP. Cada parceiro de projeto é financiado diretamente por sua respectiva agência nacional/regional. A Comissão Europeia cofinancia os JTCs da RAMP, com o cofinanciamento sendo redistribuído pelas agências financiadoras aos seus beneficiários. A duração máxima dos projetos é de 36 meses. Propostas devem se enquadrar em um dos seis tópicos temáticos e adotar princípios de 'Safe and Sustainable by Design'. Conforme a tabela de elegibilidade de parceiros do CONFAP, empresas (SMEs e grandes) e entidades sem fins lucrativos (ONGs, associações, sociedades, fundações) não são elegíveis para financiamento pela FAPES.</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-08 08:22
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -672,9 +664,9 @@
           <t>EDITAL FAPES Nº 21/2026 - REDES DE PESQUISA, DESENVOLVIMENTO E INOVAÇÃO EM SETORES ESTRATÉGICOS</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 07/08/2026</t>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-11 08:39
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -1663,11 +1663,7 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)</t>
-        </is>
-      </c>
+      <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-12 08:41
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1331,12 +1331,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Inovação</t>
+          <t>Chamadas Internacionais</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
+          <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1346,56 +1346,49 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18: Prazo de submissão de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que tenham como objetivo celebrar parcerias estratégicas com outras startups do Espírito Santo, nacionais ou internacionais. O edital busca fomentar a expansão do mercado, inovação e avanço tecnológico, aprimoramento de produtos ou serviços, acesso a novos canais ou redes de distribuição, atração de talentos e aprimoramento de competências, posicionamento de marca e mercado, acesso a oportunidades de financiamento ou investimento, e impacto socioambiental sustentável.</t>
+          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo, e com CNPJ constituído há no mínimo 1 ano e no máximo 10 anos, que atendam aos requisitos do edital.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>R$ 9.800.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Varia por modalidade: R$ 120.000,00 (Modalidade I), R$ 150.000,00 (Modalidade II), R$ 250.000,00 (Modalidade III).</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>duvidas.inovacao@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28: Prazo para impugnação do edital (Até 5 dias úteis antes da data final de submissão das propostas.)
-2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES, até as 17h59.)
-2026-08-18: Prazo de submissão de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)
-2026-12-01 a 2026-12-30: Prazo para informar dados da conta bancária (30 dias a partir do início da vigência do Termo de Outorga para informar dados da conta bancária aberta no Banco Banestes.)</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital no site da FAPES. Cada proponente pode submeter até 2 propostas de parceria, em modalidades diferentes e com parceiros distintos. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A contratação exige adimplência do coordenador e da empresa com FAPES, Fazendas Públicas (Federal, Estadual, Municipal), Justiça Trabalhista, INSS e FGTS. A primeira parcela será liberada após assinatura e publicação do Termo de Outorga e comprovação do aporte da contrapartida financeira. A segunda parcela será liberada 30 dias após o 12º mês de execução, mediante prestação de contas parcial e comprovação de execução mínima de 70% dos recursos. É obrigatória a referência ao apoio da FAPES em divulgações, exceto em período eleitoral. A FAPES não exigirá direitos de propriedade intelectual decorrentes dos projetos incentivados. Erros de menor relevância na proposta ou documentação podem ser saneados a critério da FAPES, desde que não prejudiquem a avaliação de mérito. Não serão admitidas alterações nos documentos enviados após a submissão da proposta.</t>
+          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1400,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1417,49 +1410,53 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="n"/>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>R$ 150.000,00</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
+          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1468,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1479,32 +1476,20 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
-        </is>
-      </c>
+      <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>R$ 150.000,00</t>
-        </is>
-      </c>
+          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1512,22 +1497,22 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1524,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1547,43 +1532,47 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+        </is>
+      </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1584,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1603,47 +1592,52 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
+      <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
+          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
+2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
+          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1655,7 +1649,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1667,157 +1661,92 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>US$ 6.000,00</t>
+          <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
-2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA HORIZON EUROPE</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>€ 25.000,00 por ano de projeto</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Este edital visa financiar projetos transnacionais de pesquisa e inovação em matérias-primas para a transição verde e digital. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Organizações de ensino superior e centros de pesquisa públicos. Os consórcios devem ser compostos por, no mínimo, três parceiros de três países diferentes (sendo pelo menos dois da UE ou países associados).</t>
         </is>
       </c>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)
 2026-09-22: Submissão de propostas nacionais FAPES (Etapa 1) (Recomendado verificar requisitos da FAPES para submissão na plataforma nacional, prazo idêntico ao da submissão da pré-proposta internacional.)
@@ -1831,17 +1760,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional / Início dos projetos (esperado)</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>O edital é um Joint Transnational Call (JTC) 2026 da Parceria Europeia em Matérias-Primas para a Transição Verde e Digital (RAMP). A FAPES (Fundação de Amparo à Pesquisa e Inovação do Espírito Santo) participa sob o guarda-chuva do CONFAP. Cada parceiro de projeto é financiado diretamente por sua respectiva agência nacional/regional. A Comissão Europeia cofinancia os JTCs da RAMP, com o cofinanciamento sendo redistribuído pelas agências financiadoras aos seus beneficiários. A duração máxima dos projetos é de 36 meses. Propostas devem se enquadrar em um dos seis tópicos temáticos e adotar princípios de 'Safe and Sustainable by Design'. Conforme a tabela de elegibilidade de parceiros do CONFAP, empresas (SMEs e grandes) e entidades sem fins lucrativos (ONGs, associações, sociedades, fundações) não são elegíveis para financiamento pela FAPES.</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-19 08:19
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)</t>
+          <t>2026-07-01 a 2026-08-20: Período de submissão (3ª Chamada) (eventos com início entre 04/01/2027 a 30/04/2027)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -820,7 +820,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 3ª chamada)</t>
+          <t>2026-07-01 a 2026-08-20: 3ª Chamada - Período de submissão de propostas (Eventos com início entre 04/01/2027 a 30/04/2027)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -898,7 +898,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão.)</t>
+          <t>2026-07-01 a 2026-08-20: 3ª Chamada - Período de submissão de propostas (Para estágios com início entre 04/01/2027 a 30/04/2027.)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
@@ -971,7 +971,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)</t>
+          <t>2026-07-01 a 2026-08-20: Submissão de propostas (3ª Chamada) (Para visitas com início entre 04/01/2027 a 30/04/2027.)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-20 08:21
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1189,20 +1197,25 @@
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 20/08/2026</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 a 2026-08-25: Submissão de propostas - 3ª Chamada (Até as 17h59)</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
+          <t>2026-06-19 a 2026-08-25: Submissão de propostas (3ª Chamada, até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade." → "O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. A chamada pública visa selecionar propostas para concessão de auxílio financeiro para tal finalidade, valorizando a produção técnico-científica e ampliando a visibilidade das atividades de pesquisa e inovação."
+Contato: "editais.duvidas@fapes.es.gov.br" → "editais.duvidas@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br"</t>
+        </is>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
+          <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. A chamada pública visa selecionar propostas para concessão de auxílio financeiro para tal finalidade, valorizando a produção técnico-científica e ampliando a visibilidade das atividades de pesquisa e inovação.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1222,31 +1235,28 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
+          <t>editais.duvidas@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
-2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
-?: Interposição de recursos - 1ª Chamada (5 dias úteis após a publicação do resultado preliminar)
-2026-04-30: Contratação / Assinatura do TO e envio de documentos - 1ª Chamada (Até 30 dias após a publicação do resultado final homologado.)
-2026-03-19 a 2026-05-25: Submissão de propostas - 2ª Chamada (Até as 17h59)
-?: Interposição de recursos - 2ª Chamada (5 dias úteis após a publicação do resultado preliminar)
-2026-07-30: Contratação / Assinatura do TO e envio de documentos - 2ª Chamada (Até 30 dias após a publicação do resultado final homologado.)
-2026-06-19 a 2026-08-25: Submissão de propostas - 3ª Chamada (Até as 17h59)
-?: Interposição de recursos - 3ª Chamada (5 dias úteis após a publicação do resultado preliminar)
-2026-10-30: Contratação / Assinatura do TO e envio de documentos - 3ª Chamada (Até 30 dias após a publicação do resultado final homologado.)
-2026-09-06 a 2026-10-26: Submissão de propostas - 4ª Chamada (Até as 17h59)
-?: Interposição de recursos - 4ª Chamada (5 dias úteis após a publicação do resultado preliminar)
-2026-12-30: Contratação / Assinatura do TO e envio de documentos - 4ª Chamada (Até 30 dias após a publicação do resultado final homologado.)
-?: Informar dados da conta bancária (Até 30 dias a partir do início da vigência do TO (publicação no DIO-ES).)
-?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
+          <t>2025-12-22 a 2026-02-25: Submissão de propostas (1ª Chamada, até as 17h59)
+2026-02-17: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada)
+?: Interposição de recursos (1ª Chamada, 5 dias úteis após a publicação do resultado preliminar)
+2026-03-19 a 2026-05-25: Submissão de propostas (2ª Chamada, até as 17h59)
+?: Interposição de recursos (2ª Chamada, 5 dias úteis após a publicação do resultado preliminar)
+2026-06-19 a 2026-08-25: Submissão de propostas (3ª Chamada, até as 17h59)
+?: Interposição de recursos (3ª Chamada, 5 dias úteis após a publicação do resultado preliminar)
+2026-09-06 a 2026-10-26: Submissão de propostas (4ª Chamada, até as 17h59)
+?: Interposição de recursos (4ª Chamada, 5 dias úteis após a publicação do resultado preliminar)
+?: Contratação das propostas aprovadas (Até 30 dias após a publicação do resultado final homologado de cada chamada)
+?: Informar dados bancários (Até 30 dias após a assinatura e publicação do Termo de Outorga de cada projeto)
+?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga (prazo máximo de execução do projeto é de 12 meses))</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
+          <t>O artigo deve ter sido aceito em periódico classificado entre A1 e A4 no Qualis-Capes (2021-2024) ou com percentil igual ou superior a 50% nas plataformas Scopus ou ISI Web of Science. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta por chamada; caso envie mais de uma, apenas a última será considerada. O prazo máximo para execução de cada projeto é de 12 meses.</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-21 08:19
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -750,7 +742,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01 a 2026-08-20: Período de submissão (3ª Chamada) (eventos com início entre 04/01/2027 a 30/04/2027)</t>
+          <t>2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 3ª Chamada)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -828,7 +820,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01 a 2026-08-20: 3ª Chamada - Período de submissão de propostas (Eventos com início entre 04/01/2027 a 30/04/2027)</t>
+          <t>2026-10-03 a 2026-10-09: 3ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -906,7 +898,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01 a 2026-08-20: 3ª Chamada - Período de submissão de propostas (Para estágios com início entre 04/01/2027 a 30/04/2027.)</t>
+          <t>2026-10-03 a 2026-10-09: 3ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
@@ -979,7 +971,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01 a 2026-08-20: Submissão de propostas (3ª Chamada) (Para visitas com início entre 04/01/2027 a 30/04/2027.)</t>
+          <t>2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
@@ -1197,9 +1189,9 @@
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 20/08/2026</t>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1207,12 +1199,7 @@
           <t>2026-06-19 a 2026-08-25: Submissão de propostas (3ª Chamada, até as 17h59)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade." → "O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. A chamada pública visa selecionar propostas para concessão de auxílio financeiro para tal finalidade, valorizando a produção técnico-científica e ampliando a visibilidade das atividades de pesquisa e inovação."
-Contato: "editais.duvidas@fapes.es.gov.br" → "editais.duvidas@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br"</t>
-        </is>
-      </c>
+      <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. A chamada pública visa selecionar propostas para concessão de auxílio financeiro para tal finalidade, valorizando a produção técnico-científica e ampliando a visibilidade das atividades de pesquisa e inovação.</t>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-22 08:13
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -732,38 +732,38 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
+          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Removido (nao mais aberto)</t>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 3ª Chamada)</t>
+          <t>2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59. A matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>O objetivo geral deste edital é selecionar e apoiar financeiramente pesquisadores e alunos para participação em eventos técnico-científicos de curta duração. Visa divulgar os resultados de projetos de pesquisa, desenvolvimento e inovação (P, D&amp;I) desenvolvidos em instituições de ensino superior e/ou pesquisa, públicas ou privadas, localizadas no Estado do Espírito Santo.</t>
+          <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação, valorizando a relevância e o impacto da ciência, tecnologia e inovação para o desenvolvimento do Espírito Santo.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores e alunos de pós-graduação vinculados a Instituição de Ensino e/ou Pesquisa (IES/P), pública ou privada, localizada no estado do Espírito Santo.</t>
+          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos fomentados.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>R$ 2.500.000,00</t>
+          <t>R$ 308.000,00</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>US$ 2.700,00</t>
+          <t>R$ 12.000,00</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -772,312 +772,6 @@
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-27: Prazo para solicitação de atendimento especializado (até 10 dias antes do prazo final de submissão da 1ª Chamada)
-2026-03-02: Prazo para impugnação do edital (até 5 dias úteis antes do prazo final de submissão da 1ª Chamada)
-2026-02-06 a 2026-03-09: Período de submissão (1ª Chamada) (eventos com início entre 01/05/2026 a 31/07/2026, até as 17h59)
-2026-03-07: Prazo para envio de dúvidas (1ª Chamada) (até 2 dias antes do prazo final de submissão da 1ª Chamada)
-2026-03-26: Prazo para interposição de recursos (1ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 1ª Chamada)
-2026-03-17 a 2026-04-24: Período de submissão (2ª Chamada) (eventos com início entre 01/08/2026 a 31/12/2026)
-2026-04-22: Prazo para envio de dúvidas (2ª Chamada) (até 2 dias antes do prazo final de submissão da 2ª Chamada)
-2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 2ª Chamada)
-2026-07-01 a 2026-08-20: Período de submissão (3ª Chamada) (eventos com início entre 04/01/2027 a 30/04/2027)
-2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)
-2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 3ª Chamada)</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>O valor total do edital será distribuído em três chamadas. O valor por proposta é fixo e varia conforme o local do evento: R$ 1.800,00 para eventos no Brasil (exceto Espírito Santo), US$ 1.400,00 para América Central ou América do Sul, US$ 2.300,00 para América do Norte e US$ 2.700,00 para outros continentes. A Fapes pode alterar as datas e prazos do cronograma. Cada proponente pode apresentar apenas uma proposta por chamada. O prazo para informar dados bancários é de até 30 dias corridos após o início da vigência do Termo de Outorga. O prazo para envio da prestação de contas é de até 30 dias após o término da vigência do Termo de Outorga. A contratação das propostas aprovadas ocorrerá em até 30 dias após a publicação do resultado final homologado. O envio do comprovante de aceite do trabalho é condicional para o repasse do recurso e deve ser feito até 15 dias antes do evento.</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_02-2026-Participação_Evento_Técnico_Científico.pdf</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_02_2026_-_PARTICIPAÇÃO_EM_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 03/2026 - ORGANIZAÇÃO DE EVENTOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-03 a 2026-10-09: 3ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Este edital visa selecionar propostas para conceder apoio financeiro a pesquisadores de nível superior. O objetivo é fomentar a organização de eventos técnico-científicos de curta duração, como congressos, simpósios e seminários, a serem realizados no Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores de nível superior vinculados a Instituição de Ensino Superior e/ou Pesquisa (IES/P), pública ou privada sem fins lucrativos, localizada no estado do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>R$ 2.500.000,00</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Varia de R$ 10.000,00 a R$ 35.000,00</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-02: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada)
-2026-02-06 a 2026-03-09: 1ª Chamada - Período de submissão de propostas (Eventos com início entre 01/05/2026 a 31/07/2026, até 17h59)
-2026-03-07: 1ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 1ª chamada)
-2026-03-20 a 2026-03-26: 1ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)
-2026-03-17 a 2026-04-24: 2ª Chamada - Período de submissão de propostas (Eventos com início entre 01/08/2026 a 31/12/2026)
-2026-04-22: 2ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 2ª chamada)
-2026-05-23 a 2026-05-29: 2ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)
-2026-07-01 a 2026-08-20: 3ª Chamada - Período de submissão de propostas (Eventos com início entre 04/01/2027 a 30/04/2027)
-2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 3ª chamada)
-2026-10-03 a 2026-10-09: 3ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)
-?: Contratação das propostas aprovadas (Até 30 dias após a publicação do resultado final homologado para cada chamada. As datas exatas serão publicadas posteriormente.)</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>O valor do auxílio financeiro é fixo e varia de acordo com o nível do evento: R$ 10.000,00 para Estadual/Regional, R$ 20.000,00 para Nacional e R$ 35.000,00 para Internacional. A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional. Cada proponente pode apresentar apenas uma proposta por chamada. Caso envie mais de uma, será considerada apenas a última enviada. O proponente que já tiver sido contratado neste edital não poderá submeter nova proposta. O evento deve ter duração máxima de 15 dias, consecutivos ou não, e ser chancelado por entidade/sociedade conforme o nível do evento (nacional ou internacional). Os recursos financeiros estão distribuídos por chamada e nível de evento, com possibilidade de remanejamento de saldos não utilizados entre níveis e chamadas subsequentes. É obrigatório mencionar o apoio da Fapes em todas as publicações e divulgações relacionadas ao projeto. A data de início do apoio poderá ser adiada, após a contratação, em até 12 meses, mediante justificativa.</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_03_2026_Organização_Eventos_Técnico-Científicos.pdf</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_03_2026_-_ORGANIZAÇÃO_DE_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO-CIENTÍFICO</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-03 a 2026-10-09: 3ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar.)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Selecionar propostas para concessão de auxílio financeiro para estágios técnico-científicos em laboratórios ou centros de PD&amp;I, no Brasil ou exterior. O objetivo é aprimorar técnicas, adquirir conhecimentos específicos para projetos de PD&amp;I no Espírito Santo, estimular o intercâmbio de conhecimentos, a formação de pós-graduandos e apoiar os Programas de Pós-graduação do estado.</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas localizadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P localizadas no Espírito Santo, reconhecidos pela CAPES/CNE/MEC.</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>R$ 2.000.000,00</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geped@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-05: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada.)
-2026-02-09 a 2026-03-12: 1ª Chamada - Período de submissão de propostas (Para estágios com início entre 01/05/2026 a 31/07/2026, até as 17h59.)
-2026-03-10: 1ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão.)
-2026-03-17 a 2026-04-24: 2ª Chamada - Período de submissão de propostas (Para estágios com início entre 01/08/2026 a 31/12/2026.)
-2026-03-20 a 2026-03-26: 1ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar.)
-2026-04-22: 2ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão.)
-2026-05-23 a 2026-05-29: 2ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar.)
-2026-07-01 a 2026-08-20: 3ª Chamada - Período de submissão de propostas (Para estágios com início entre 04/01/2027 a 30/04/2027.)
-2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão.)
-2026-10-03 a 2026-10-09: 3ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar.)</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>O valor por proposta varia conforme o nível (duração do estágio) e a localização (Brasil - Região Sudeste, Brasil - Demais Estados, Exterior - América Central e do Sul, Exterior - América do Norte, Exterior - Demais Continentes), conforme tabela na seção 6.4 e 6.5 do edital. A Fapes pode alterar as datas e prazos do cronograma, reabrir prazos em casos de força maior ou falhas de sistema, e dará publicidade a essas alterações. Recursos financeiros não utilizados em uma chamada podem ser aplicados em chamadas subsequentes. O beneficiário não poderá utilizar outros recursos da Fapes para cobrir despesas do estágio se o auxílio concedido for insuficiente. Auxílios em moeda estrangeira serão convertidos com base no câmbio oficial na data de aprovação. Cada proponente pode apresentar apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Não é permitida a contratação concomitante de estágio técnico-científico e visita técnico-científica para o mesmo período/chamada. O edital pode ser revogado ou anulado sem direito a indenização. Casos omissos e dúvidas de interpretação serão dirimidos pela Diretoria Executiva da Fapes.</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_04_2026_-_Estágio_Técnico_Cientifico.pdf</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_04_2026_-_ESTÁGIO_TÉCNICO-CIENTÍFICO.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Selecionar propostas para concessão de auxílio financeiro para a realização de visitas técnico-científicas em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, processos e adquirir conhecimentos específicos para projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas no Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>R$ 2.000.000,00</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>US$ 2.600,00</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 a 2026-03-12: Submissão de propostas (1ª Chamada) (Até as 17h59. Para visitas com início entre 01/05/2026 a 31/07/2026.)
-2026-03-05: Prazo final para impugnação do edital (Até o quinto dia útil que anteceder o prazo final de submissão da 1ª Chamada.)
-2026-03-10: Prazo para envio de dúvidas sobre o edital (1ª Chamada) (Até 2 dias antes do prazo final de submissão.)
-2026-03-17 a 2026-04-24: Submissão de propostas (2ª Chamada) (Para visitas com início entre 01/08/2026 a 31/12/2026.)
-2026-03-26: Prazo para interposição de recursos (1ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)
-2026-04-22: Prazo para envio de dúvidas sobre o edital (2ª Chamada) (Até 2 dias antes do prazo final de submissão.)
-2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)
-2026-07-01 a 2026-08-20: Submissão de propostas (3ª Chamada) (Para visitas com início entre 04/01/2027 a 30/04/2027.)
-2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)
-2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade institucional, podendo reabrir prazos em casos de força maior ou falhas de sistema, com publicidade das alterações. Cada proponente pode submeter apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Proponentes já contratados neste edital não poderão submeter nova proposta. Após a contratação, o beneficiário pode solicitar adiamento da data de início da visita por até 30 dias, mediante justificativa e autorização. Não será permitida a alteração da instituição de destino da visita técnico-científica após a contratação.</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2005_2026%20-%20Visita%20Técnico%20Cientifica%20(1).pdf</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_05_2026_-_VISITA_TÉCNICO-CIENTÍFICA.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59. A matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.)</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação, valorizando a relevância e o impacto da ciência, tecnologia e inovação para o desenvolvimento do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos fomentados.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>R$ 308.000,00</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>R$ 12.000,00</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)
 2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59. A matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.)
@@ -1085,70 +779,70 @@
 2026-11-03 a 2026-11-09: Votação popular – Categoria Jornalismo</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Edição em homenagem à Professora Jurema José de Oliveira. Os valores das premiações possuem natureza bruta e estão sujeitos à incidência do Imposto de Renda Retido na Fonte – IRRF, na forma da legislação tributária vigente. A premiação prevista neste edital possui caráter exclusivamente honorífico, meritório e eventual, destinando-se ao reconhecimento institucional dos trabalhos classificados. A Fapes pode alterar datas e prazos do cronograma por necessidade administrativa ou decisão institucional. O comparecimento do premiado é obrigatório. Caso não possa comparecer, deve indicar formalmente um representante para o recebimento da premiação, com comunicação prévia à Fapes, pelo e-mail gabinete@fapes.es.gov.br. Para as categorias Projetos e Destaque, as 3 (três) propostas com as maiores notas seguem para votação pelo Comitê de Especialistas. Para a categoria Jornalismo, as 3 (três) matérias com maiores notas seguem para votação popular.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 25/2025 - PARTICIPAÇÃO DE EQUIPES DE ESTUDANTES EM MOSTRAS E COMPETIÇÕES TÉCNICO-CIENTÍFICAS</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Conceder apoio financeiro a equipes formadas por estudantes de nível médio, de graduação e pós-graduação, coordenadas por um professor orientador. O objetivo é permitir a participação dessas equipes em mostras e competições técnico-científicas de âmbito regional, nacional ou internacional, visando a divulgação e difusão de resultados obtidos por instituições de ensino do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Professores(as) coordenadores(as) de equipes de 3 a 5 estudantes, vinculados(as) a instituições de ensino médio públicas ou instituições de ensino superior públicas ou privadas localizadas no estado do Espírito Santo. O proponente deve ter formação mínima de nível superior, vínculo ativo com a instituição, atuar em sala de aula na mesma instituição dos estudantes, ter Lattes atualizado há menos de 6 meses, estar regularizado junto à Fapes e morar no Espírito Santo ou municípios limítrofes. Estudantes de instituições privadas devem ser bolsistas integrais financiados por programas governamentais estaduais ou federais.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 500.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>?: Prazo para impugnação do edital (5 dias úteis antes do encerramento do prazo de submissão da 1ª Chamada)
 2025-11-10 a 2025-12-16: Submissão de propostas (Até as 17h:59. Para 1ª Chamada (eventos com início entre 01/03/2026 a 30/06/2026))
@@ -1162,70 +856,70 @@
 ?: Prazo para prestação de contas (Até 30 dias após o término da vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>O valor por proposta varia conforme a categoria do evento: R$ 500,00 para eventos regionais, R$ 1.200,00 para eventos nacionais e US$ 1.500,00 para eventos internacionais. O edital prevê três chamadas com períodos de submissão e eventos distintos. O início do evento proposto deve corresponder ao período da chamada selecionada. A Fapes pode alterar as datas e prazos definidos no cronograma. Cada coordenador pode apresentar apenas uma proposta. Não são contempladas propostas para participação em concursos ou premiações sem natureza acadêmica, técnico-científica ou tecnológica, ou competições esportivas.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_N_25_2025_Participação_Equipe_em_Mostras_e_Competições-2.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_N°_25_2025_-_PARTICIPAÇÃO_DE_EQUIPES_DE_ESTUDANTES_EM_MOSTRAS_E_COMPETIÇÕES_TÉCNICO-CIENTÍFICAS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-06-19 a 2026-08-25: Submissão de propostas (3ª Chamada, até as 17h59)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. A chamada pública visa selecionar propostas para concessão de auxílio financeiro para tal finalidade, valorizando a produção técnico-científica e ampliando a visibilidade das atividades de pesquisa e inovação.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2025-12-22 a 2026-02-25: Submissão de propostas (1ª Chamada, até as 17h59)
 2026-02-17: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada)
@@ -1241,66 +935,66 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga (prazo máximo de execução do projeto é de 12 meses))</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>O artigo deve ter sido aceito em periódico classificado entre A1 e A4 no Qualis-Capes (2021-2024) ou com percentil igual ou superior a 50% nas plataformas Scopus ou ISI Web of Science. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta por chamada; caso envie mais de uma, apenas a última será considerada. O prazo máximo para execução de cada projeto é de 12 meses.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Promover o aumento da competitividade dos setores econômicos capixabas por meio de projetos de inovação, desenvolvidos por empresas (incluindo cooperativas de trabalho) em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas. O apoio se dará por meio de um modelo de coinvestimento tripartite (FAPES, empresa/cooperativa, ICT/IES), com projetos alinhados ao Plano ES 500 Anos e ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas ou cooperativas de trabalho capixabas.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>R$ 500.000,00 a R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-03-30: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 ?: Prazo de submissão dos recursos administrativos (Habilitação) (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)
@@ -1309,19 +1003,267 @@
 ?: Submissão das documentações para contratação (Até 30 dias a partir da publicação do resultado homologado do julgamento de mérito.)</t>
         </is>
       </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>O prazo de execução do projeto é de 24 meses, com possibilidade de prorrogação por até 12 meses. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais; cooperativas de trabalho devem apresentar Demonstração de Sobras ou Perdas (DSP). As empresas devem estar ativas há pelo menos 6 meses e não podem ter sido contratadas em editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026, a menos que o projeto, coordenador e equipe executora sejam distintos. É permitida apenas uma proposta por empresa. Em caso de inabilitação ou desclassificação, a empresa poderá realizar uma nova submissão, exceto se reprovada pelo Comitê de Conformidade, o que impede nova submissão nesta chamada. A aprovação da proposta não garante a contratação, que está sujeita à disponibilidade financeira da FAPES, ordem de submissão e visita técnica. O critério de desempate é a data de submissão da proposta no SIGFAPES. Propostas com Nota Final inferior a 80 pontos ou notas individuais inferiores a 4 em critérios específicos serão desclassificadas. A impugnação dos termos do edital deve ser feita em até 5 dias úteis antes do encerramento do prazo de submissão das propostas do primeiro ciclo (considerando o fluxo contínuo, esta observação se refere a um prazo inicial para impugnação do edital em si).</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP CDTI 2026</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>€ 75.000,00</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+        </is>
+      </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>O prazo de execução do projeto é de 24 meses, com possibilidade de prorrogação por até 12 meses. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais; cooperativas de trabalho devem apresentar Demonstração de Sobras ou Perdas (DSP). As empresas devem estar ativas há pelo menos 6 meses e não podem ter sido contratadas em editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026, a menos que o projeto, coordenador e equipe executora sejam distintos. É permitida apenas uma proposta por empresa. Em caso de inabilitação ou desclassificação, a empresa poderá realizar uma nova submissão, exceto se reprovada pelo Comitê de Conformidade, o que impede nova submissão nesta chamada. A aprovação da proposta não garante a contratação, que está sujeita à disponibilidade financeira da FAPES, ordem de submissão e visita técnica. O critério de desempate é a data de submissão da proposta no SIGFAPES. Propostas com Nota Final inferior a 80 pontos ou notas individuais inferiores a 4 em critérios específicos serão desclassificadas. A impugnação dos termos do edital deve ser feita em até 5 dias úteis antes do encerramento do prazo de submissão das propostas do primeiro ciclo (considerando o fluxo contínuo, esta observação se refere a um prazo inicial para impugnação do edital em si).</t>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1275,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1341,51 +1283,52 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
+      <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="n"/>
+          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>US$ 6.000,00</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
+2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
+          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1397,7 +1340,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1405,55 +1348,49 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
-        </is>
-      </c>
+      <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
+?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
+?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
+          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
@@ -1465,7 +1402,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1473,277 +1410,34 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
+          <t>Este edital visa financiar projetos transnacionais de pesquisa e inovação em matérias-primas para a transição verde e digital. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
+          <t>Organizações de ensino superior e centros de pesquisa públicos. Os consórcios devem ser compostos por, no mínimo, três parceiros de três países diferentes (sendo pelo menos dois da UE ou países associados).</t>
         </is>
       </c>
       <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>EUR 100.000,00</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>US$ 6.000,00</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
-2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA HORIZON EUROPE</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>€ 25.000,00 por ano de projeto</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
-?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
-?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
-        </is>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Este edital visa financiar projetos transnacionais de pesquisa e inovação em matérias-primas para a transição verde e digital. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Organizações de ensino superior e centros de pesquisa públicos. Os consórcios devem ser compostos por, no mínimo, três parceiros de três países diferentes (sendo pelo menos dois da UE ou países associados).</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>EUR 100.000,00</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)
 2026-09-22: Submissão de propostas nacionais FAPES (Etapa 1) (Recomendado verificar requisitos da FAPES para submissão na plataforma nacional, prazo idêntico ao da submissão da pré-proposta internacional.)
@@ -1757,17 +1451,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional / Início dos projetos (esperado)</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>O edital é um Joint Transnational Call (JTC) 2026 da Parceria Europeia em Matérias-Primas para a Transição Verde e Digital (RAMP). A FAPES (Fundação de Amparo à Pesquisa e Inovação do Espírito Santo) participa sob o guarda-chuva do CONFAP. Cada parceiro de projeto é financiado diretamente por sua respectiva agência nacional/regional. A Comissão Europeia cofinancia os JTCs da RAMP, com o cofinanciamento sendo redistribuído pelas agências financiadoras aos seus beneficiários. A duração máxima dos projetos é de 36 meses. Propostas devem se enquadrar em um dos seis tópicos temáticos e adotar princípios de 'Safe and Sustainable by Design'. Conforme a tabela de elegibilidade de parceiros do CONFAP, empresas (SMEs e grandes) e entidades sem fins lucrativos (ONGs, associações, sociedades, fundações) não são elegíveis para financiamento pela FAPES.</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-25 08:21
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -656,51 +664,127 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Pesquisa</t>
+          <t>Formação Científica</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 21/2026 - REDES DE PESQUISA, DESENVOLVIMENTO E INOVAÇÃO EM SETORES ESTRATÉGICOS</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>EDITAL FAPES/CNPq/CAPES Nº 22/2026 - PROGRAMA DE APOIO À FIXAÇÃO DE DOUTORES NO BRASIL (PROFIX-CB)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 25/08/2026</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10: Envio de dúvidas sobre o edital (Até as 17h59)</t>
+          <t>2026-10-01: Submissão das propostas (Até as 17h59, via Sistema de Informação e Gestão de Projetos da Fapes)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
+          <t>O Programa de Apoio à Fixação de Doutores no Brasil – Conhecimento Brasil (PROFIX-CB) é uma iniciativa do CNPq, CAPES e FAPs para atrair, inserir e fixar pesquisadores doutores em instituições de pesquisa, universidades e centros de inovação no país. Seu propósito é criar condições para que o doutor estabeleça uma trajetória científica de médio prazo, contribuindo para a formação de recursos humanos, fortalecimento de programas de pós-graduação, consolidação de grupos de pesquisa e geração de conhecimento e inovação, especialmente em áreas estratégicas para o desenvolvimento científico, tecnológico e de inovação do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores doutores (com título obtido há no máximo 10 anos até a data limite de submissão da proposta), residentes no Espírito Santo, sem vínculo empregatício, que atuarão como coordenadores e bolsistas PROFIX-CB em Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no Espírito Santo, com um Programa de Pós-graduação (PPG) parceiro.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>R$ 31.803.200,00</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>R$ 400.000,00</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>bolsas.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01: Submissão das propostas (Até as 17h59, via Sistema de Informação e Gestão de Projetos da Fapes)
+?: Interposição de recursos (Até 5 dias úteis após a divulgação do resultado preliminar)
+2027-01-04: Contratação dos projetos e assinatura do Termo de Outorga (A partir de, via Acesso Cidadão e Sistema de Informação e Gestão de Projetos da Fapes)
+?: Envio de dados bancários para recebimento de recursos (Até 30 dias após a contratação)
+?: Indicação de bolsistas de mestrado e doutorado (Capes) (Até 12 meses após o início da vigência do projeto)
+?: Prestação de contas parcial (A cada 12 meses de vigência do projeto)
+?: Prestação de contas final (Até 30 dias após o término da vigência do Termo de Outorga)
+?: Envio de Relatório Técnico da Bolsa PROFIX-CB (Até 60 dias após o término da vigência do processo CNPq)
+?: Envio de Relatório Final de Bolsas de Pós-graduação (Capes) (Até 30 dias após o término da bolsa)</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>A proposta deve ter cronograma de atividades de 48 meses. O projeto tem vigência de 48 meses. A bolsa PROFIX-CB tem duração de 48 meses. As bolsas de doutorado (Capes) têm duração de até 48 meses, e as de mestrado (Capes) até 24 meses. As bolsas de Iniciação Científica e Tecnológica (Fapes) têm duração de até 12 meses, podendo ser prorrogadas por mais duas vezes. É obrigatório mencionar o apoio da Fapes, CNPq e Capes em todas as publicações e divulgações. Os resultados de propriedade intelectual devem ser comunicados à Fapes. A Fapes abre mão dos direitos de participação e propriedade sobre pesquisas e projetos que apoia, conforme previsto em legislação específica. A convocação de suplentes pode ocorrer por até 24 meses após a divulgação do resultado final. Os anexos do edital estão disponíveis no site da Fapes em 'Editais Abertos'. Dúvidas sobre a chamada devem ser enviadas em até 2 dias antes do término da submissão das propostas.</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2022.2026%20-%20PROFIX-CB.pdf</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>formacao_cientifica/EDITAL_FAPES_CNPq_CAPES_No_22_2026_-_PROGRAMA_DE_APOIO_À_FIXAÇÃO_DE_DOUTORES_NO_BRASIL_(PROFIX-CB).pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisa</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 21/2026 - REDES DE PESQUISA, DESENVOLVIMENTO E INOVAÇÃO EM SETORES ESTRATÉGICOS</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10: Envio de dúvidas sobre o edital (Até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>O edital Redes de Pesquisa, Desenvolvimento e Inovação (PD&amp;I) em Setores Estratégicos da Fapes tem como finalidade apoiar financeiramente a criação e o fortalecimento de redes que promovam ações coletivas de PD&amp;I. O objetivo geral é selecionar projetos para criar e fortalecer redes estruturantes de PD&amp;I em setores estratégicos e de interesse do Espírito Santo, consolidando grupos de referência em áreas do conhecimento.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores doutores vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo, que atuem como coordenadores de propostas.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000.000,00</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>R$ 1.200.000,00</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>2026-09-10: Envio de dúvidas sobre o edital (Até as 17h59)
 2026-08-07 a 2026-09-14: Submissão de propostas (Até as 17h59, via SigFapes)
@@ -708,70 +792,70 @@
 ?: Interposição de recursos (análise de mérito) (Até 5 dias úteis após a divulgação do resultado preliminar da análise de mérito)</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>As propostas devem ter prazo de execução de até 36 meses e prever no orçamento 1 bolsista pós-doutorado (POSDOC) e 1 estudante de graduação (ICT). As linhas temáticas incluem: Saúde Única, Saúde de Precisão, Imunobiológicos e Biofármacos, Preservação e Restauração ecológica do bioma da Mata Atlântica, Transformação digital e rastreabilidade ambiental, Economia Circular e Soberania digital e cibersegurança. A equipe executora deve ser exclusiva e composta por no mínimo 7 pesquisadores além do coordenador, com distribuição específica de doutores de diferentes IES/P e um pesquisador de órgão público estadual. Os recursos serão distribuídos garantindo ao menos uma proposta contemplada por linha temática, e as demais por ordem decrescente de nota final. Somente propostas com nota final igual ou superior a 70,0 pontos serão classificadas. Despesas de custeio com serviços de terceiros são limitadas a 30% do valor máximo por proposta. Despesas de capital financiáveis devem ter vida útil superior a dois anos e valor superior a 80 VRTEs. Não são financiáveis mobiliário (exceto se indispensável à pesquisa) e veículos motorizados (exceto se objeto da pesquisa).</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_21-2026_-_Redes_de_PDI_em_Setores_Estratégicos.pdf</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>pesquisa/EDITAL_FAPES_No_21_2026_-_REDES_DE_PESQUISA,_DESENVOLVIMENTO_E_INOVAÇÃO_EM_SETORES_ESTRATÉGICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59. A matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.)</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação, valorizando a relevância e o impacto da ciência, tecnologia e inovação para o desenvolvimento do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos fomentados.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 308.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000,00</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)
 2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59. A matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.)
@@ -779,70 +863,70 @@
 2026-11-03 a 2026-11-09: Votação popular – Categoria Jornalismo</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Edição em homenagem à Professora Jurema José de Oliveira. Os valores das premiações possuem natureza bruta e estão sujeitos à incidência do Imposto de Renda Retido na Fonte – IRRF, na forma da legislação tributária vigente. A premiação prevista neste edital possui caráter exclusivamente honorífico, meritório e eventual, destinando-se ao reconhecimento institucional dos trabalhos classificados. A Fapes pode alterar datas e prazos do cronograma por necessidade administrativa ou decisão institucional. O comparecimento do premiado é obrigatório. Caso não possa comparecer, deve indicar formalmente um representante para o recebimento da premiação, com comunicação prévia à Fapes, pelo e-mail gabinete@fapes.es.gov.br. Para as categorias Projetos e Destaque, as 3 (três) propostas com as maiores notas seguem para votação pelo Comitê de Especialistas. Para a categoria Jornalismo, as 3 (três) matérias com maiores notas seguem para votação popular.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 25/2025 - PARTICIPAÇÃO DE EQUIPES DE ESTUDANTES EM MOSTRAS E COMPETIÇÕES TÉCNICO-CIENTÍFICAS</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Conceder apoio financeiro a equipes formadas por estudantes de nível médio, de graduação e pós-graduação, coordenadas por um professor orientador. O objetivo é permitir a participação dessas equipes em mostras e competições técnico-científicas de âmbito regional, nacional ou internacional, visando a divulgação e difusão de resultados obtidos por instituições de ensino do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Professores(as) coordenadores(as) de equipes de 3 a 5 estudantes, vinculados(as) a instituições de ensino médio públicas ou instituições de ensino superior públicas ou privadas localizadas no estado do Espírito Santo. O proponente deve ter formação mínima de nível superior, vínculo ativo com a instituição, atuar em sala de aula na mesma instituição dos estudantes, ter Lattes atualizado há menos de 6 meses, estar regularizado junto à Fapes e morar no Espírito Santo ou municípios limítrofes. Estudantes de instituições privadas devem ser bolsistas integrais financiados por programas governamentais estaduais ou federais.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 500.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>?: Prazo para impugnação do edital (5 dias úteis antes do encerramento do prazo de submissão da 1ª Chamada)
 2025-11-10 a 2025-12-16: Submissão de propostas (Até as 17h:59. Para 1ª Chamada (eventos com início entre 01/03/2026 a 30/06/2026))
@@ -856,70 +940,70 @@
 ?: Prazo para prestação de contas (Até 30 dias após o término da vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>O valor por proposta varia conforme a categoria do evento: R$ 500,00 para eventos regionais, R$ 1.200,00 para eventos nacionais e US$ 1.500,00 para eventos internacionais. O edital prevê três chamadas com períodos de submissão e eventos distintos. O início do evento proposto deve corresponder ao período da chamada selecionada. A Fapes pode alterar as datas e prazos definidos no cronograma. Cada coordenador pode apresentar apenas uma proposta. Não são contempladas propostas para participação em concursos ou premiações sem natureza acadêmica, técnico-científica ou tecnológica, ou competições esportivas.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_N_25_2025_Participação_Equipe_em_Mostras_e_Competições-2.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_N°_25_2025_-_PARTICIPAÇÃO_DE_EQUIPES_DE_ESTUDANTES_EM_MOSTRAS_E_COMPETIÇÕES_TÉCNICO-CIENTÍFICAS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-06-19 a 2026-08-25: Submissão de propostas (3ª Chamada, até as 17h59)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. A chamada pública visa selecionar propostas para concessão de auxílio financeiro para tal finalidade, valorizando a produção técnico-científica e ampliando a visibilidade das atividades de pesquisa e inovação.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2025-12-22 a 2026-02-25: Submissão de propostas (1ª Chamada, até as 17h59)
 2026-02-17: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada)
@@ -935,66 +1019,66 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga (prazo máximo de execução do projeto é de 12 meses))</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>O artigo deve ter sido aceito em periódico classificado entre A1 e A4 no Qualis-Capes (2021-2024) ou com percentil igual ou superior a 50% nas plataformas Scopus ou ISI Web of Science. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta por chamada; caso envie mais de uma, apenas a última será considerada. O prazo máximo para execução de cada projeto é de 12 meses.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Promover o aumento da competitividade dos setores econômicos capixabas por meio de projetos de inovação, desenvolvidos por empresas (incluindo cooperativas de trabalho) em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas. O apoio se dará por meio de um modelo de coinvestimento tripartite (FAPES, empresa/cooperativa, ICT/IES), com projetos alinhados ao Plano ES 500 Anos e ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas ou cooperativas de trabalho capixabas.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 500.000,00 a R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-03-30: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 ?: Prazo de submissão dos recursos administrativos (Habilitação) (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)
@@ -1003,83 +1087,19 @@
 ?: Submissão das documentações para contratação (Até 30 dias a partir da publicação do resultado homologado do julgamento de mérito.)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução do projeto é de 24 meses, com possibilidade de prorrogação por até 12 meses. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais; cooperativas de trabalho devem apresentar Demonstração de Sobras ou Perdas (DSP). As empresas devem estar ativas há pelo menos 6 meses e não podem ter sido contratadas em editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026, a menos que o projeto, coordenador e equipe executora sejam distintos. É permitida apenas uma proposta por empresa. Em caso de inabilitação ou desclassificação, a empresa poderá realizar uma nova submissão, exceto se reprovada pelo Comitê de Conformidade, o que impede nova submissão nesta chamada. A aprovação da proposta não garante a contratação, que está sujeita à disponibilidade financeira da FAPES, ordem de submissão e visita técnica. O critério de desempate é a data de submissão da proposta no SIGFAPES. Propostas com Nota Final inferior a 80 pontos ou notas individuais inferiores a 4 em critérios específicos serão desclassificadas. A impugnação dos termos do edital deve ser feita em até 5 dias úteis antes do encerramento do prazo de submissão das propostas do primeiro ciclo (considerando o fluxo contínuo, esta observação se refere a um prazo inicial para impugnação do edital em si).</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>€ 75.000,00</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1111,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1101,53 +1121,49 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
+          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1159,7 +1175,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1167,20 +1183,32 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="n"/>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1188,22 +1216,22 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
+          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1243,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1223,47 +1251,43 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
+      <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
         </is>
       </c>
       <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="n"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1299,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1283,52 +1307,47 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+        </is>
+      </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>US$ 6.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
-2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1359,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1352,92 +1371,157 @@
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
+2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Este edital visa financiar projetos transnacionais de pesquisa e inovação em matérias-primas para a transição verde e digital. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Organizações de ensino superior e centros de pesquisa públicos. Os consórcios devem ser compostos por, no mínimo, três parceiros de três países diferentes (sendo pelo menos dois da UE ou países associados).</t>
         </is>
       </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)
 2026-09-22: Submissão de propostas nacionais FAPES (Etapa 1) (Recomendado verificar requisitos da FAPES para submissão na plataforma nacional, prazo idêntico ao da submissão da pré-proposta internacional.)
@@ -1451,17 +1535,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional / Início dos projetos (esperado)</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>O edital é um Joint Transnational Call (JTC) 2026 da Parceria Europeia em Matérias-Primas para a Transição Verde e Digital (RAMP). A FAPES (Fundação de Amparo à Pesquisa e Inovação do Espírito Santo) participa sob o guarda-chuva do CONFAP. Cada parceiro de projeto é financiado diretamente por sua respectiva agência nacional/regional. A Comissão Europeia cofinancia os JTCs da RAMP, com o cofinanciamento sendo redistribuído pelas agências financiadoras aos seus beneficiários. A duração máxima dos projetos é de 36 meses. Propostas devem se enquadrar em um dos seis tópicos temáticos e adotar princípios de 'Safe and Sustainable by Design'. Conforme a tabela de elegibilidade de parceiros do CONFAP, empresas (SMEs e grandes) e entidades sem fins lucrativos (ONGs, associações, sociedades, fundações) não são elegíveis para financiamento pela FAPES.</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-26 08:23
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -672,9 +672,9 @@
           <t>EDITAL FAPES/CNPq/CAPES Nº 22/2026 - PROGRAMA DE APOIO À FIXAÇÃO DE DOUTORES NO BRASIL (PROFIX-CB)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/08/2026</t>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -974,7 +974,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 a 2026-08-25: Submissão de propostas (3ª Chamada, até as 17h59)</t>
+          <t>2026-09-06 a 2026-10-26: Submissão de propostas (4ª Chamada, até as 17h59)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
@@ -1106,64 +1106,70 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Chamadas Internacionais</t>
+          <t>Inovação</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 26/08/2026</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-08-25 a 2026-09-24: Submissão de propostas (até as 17h59, via SigFapes)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
+          <t>Apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que ofereçam apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas com produtos, serviços ou modelos de negócio inovadores. O edital visa ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de empreendedores, a sustentabilidade econômica das empresas incubadas e o desenvolvimento socioeconômico do Espírito Santo.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="n"/>
+          <t>Incubadoras, sem fins lucrativos, sediadas no Espírito Santo, que atendam aos requisitos do edital.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>R$ 4.500.000,00</t>
+        </is>
+      </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>R$ 252.000,00</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-08-25 a 2026-09-24: Submissão de propostas (até as 17h59, via SigFapes)
+2026-10-16: Interposição de recursos (Até 5 dias úteis após a divulgação do resultado preliminar)
+2026-11-04: Contratação dos projetos selecionados</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
+          <t>O valor por proposta varia conforme o nível de maturidade da incubadora: Nível Avançado (R$ 252.000,00), Nível Intermediário (R$ 192.000,00) e Nível Básico (R$ 132.000,00). O projeto terá prazo de vigência de 24 meses, sem prorrogação. Propostas com nota final inferior a 70 pontos serão desclassificadas. A Fapes pode alterar o cronograma e redirecionar recursos remanescentes entre os níveis de maturidade. Os recursos de custeio (exceto bolsas) serão liberados em 2 parcelas. O orçamento do projeto pode ser aprovado parcial ou integralmente.</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
+          <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1181,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1185,53 +1191,49 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
+          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1245,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1251,20 +1253,32 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1272,22 +1286,22 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
+          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1299,7 +1313,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1307,47 +1321,43 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
+      <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
         </is>
       </c>
       <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="n"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1369,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1367,52 +1377,47 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>US$ 6.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
-2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1429,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1436,92 +1441,157 @@
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
+2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Este edital visa financiar projetos transnacionais de pesquisa e inovação em matérias-primas para a transição verde e digital. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Organizações de ensino superior e centros de pesquisa públicos. Os consórcios devem ser compostos por, no mínimo, três parceiros de três países diferentes (sendo pelo menos dois da UE ou países associados).</t>
         </is>
       </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)
 2026-09-22: Submissão de propostas nacionais FAPES (Etapa 1) (Recomendado verificar requisitos da FAPES para submissão na plataforma nacional, prazo idêntico ao da submissão da pré-proposta internacional.)
@@ -1535,17 +1605,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional / Início dos projetos (esperado)</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>O edital é um Joint Transnational Call (JTC) 2026 da Parceria Europeia em Matérias-Primas para a Transição Verde e Digital (RAMP). A FAPES (Fundação de Amparo à Pesquisa e Inovação do Espírito Santo) participa sob o guarda-chuva do CONFAP. Cada parceiro de projeto é financiado diretamente por sua respectiva agência nacional/regional. A Comissão Europeia cofinancia os JTCs da RAMP, com o cofinanciamento sendo redistribuído pelas agências financiadoras aos seus beneficiários. A duração máxima dos projetos é de 36 meses. Propostas devem se enquadrar em um dos seis tópicos temáticos e adotar princípios de 'Safe and Sustainable by Design'. Conforme a tabela de elegibilidade de parceiros do CONFAP, empresas (SMEs e grandes) e entidades sem fins lucrativos (ONGs, associações, sociedades, fundações) não são elegíveis para financiamento pela FAPES.</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-27 17:53
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1114,9 +1106,9 @@
           <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 26/08/2026</t>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-28 18:19
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -803,51 +811,123 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Difusão do Conhecimento</t>
+          <t>Pesquisa</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>EDITAL FAPES Nº 24/2026 - PRIMEIROS PROJETOS DE PESQUISA - ESPÍRITO SANTO (PPP-ES)</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 28/08/2026</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59. A matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.)</t>
+          <t>2026-09-28: Prazo para envio de dúvidas a respeito do edital (até as 17h59)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
+          <t>Apoiar o primeiro projeto de pesquisa científica de pesquisadores doutores em início de carreira, vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas no Espírito Santo. O edital visa fortalecer a pesquisa científica no estado, promover o acesso a recursos e consolidar novos grupos de pesquisa, com projetos de até 24 meses de duração.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores doutores em início de carreira, que tenham obtido o título de doutor a partir de 28/08/2018, vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo. Os proponentes não devem ter atuado como coordenadores de projetos de pesquisa, extensão ou inovação no âmbito da Fapes ou do CNPq, com exceção de projetos PICJr, PIBIC, PIBITI, auxílios e/ou bolsas de pós-graduação.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>R$ 4.000.000,00</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>R$ 180.000,00</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28: Prazo para envio de dúvidas a respeito do edital (até as 17h59)
+2026-08-29 a 2026-09-30: Envio da proposta e documentos via SigFapes (até as 17h59)
+?: Prazo para recorrer (habilitação) (5 dias úteis após a divulgação do resultado preliminar da habilitação)
+?: Prazo para recorrer (análise de mérito) (5 dias úteis após a divulgação do resultado preliminar de análise de mérito)
+2026-12-10: Início da contratação dos projetos selecionados (Prazo de até 30 dias para a Fapes contratar as propostas aprovadas após a publicação do resultado final homologado.)</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Os projetos aprovados terão duração de até 24 meses. Os coordenadores devem ter obtido o título de doutor a partir de 28/08/2018 e não podem ter atuado como coordenadores de projetos de pesquisa, extensão ou inovação no âmbito da Fapes ou do CNPq, exceto em projetos PICJr, PIBIC, PIBITI, auxílios e/ou bolsas de pós-graduação. As propostas devem estar enquadradas em uma das 8 grandes áreas do conhecimento do CNPq. Documentos de aprovação ética e legal, quando aplicáveis, devem estar emitidos ou aprovados no momento da contratação.</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2024-2026%20PPP-ES.pdf</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>pesquisa/EDITAL_FAPES_No_24_2026_-_PRIMEIROS_PROJETOS_DE_PESQUISA_-_ESPÍRITO_SANTO_(PPP-ES).pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59. A matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação, valorizando a relevância e o impacto da ciência, tecnologia e inovação para o desenvolvimento do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a projetos fomentados.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 308.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000,00</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)
 2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59. A matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.)
@@ -855,70 +935,70 @@
 2026-11-03 a 2026-11-09: Votação popular – Categoria Jornalismo</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Edição em homenagem à Professora Jurema José de Oliveira. Os valores das premiações possuem natureza bruta e estão sujeitos à incidência do Imposto de Renda Retido na Fonte – IRRF, na forma da legislação tributária vigente. A premiação prevista neste edital possui caráter exclusivamente honorífico, meritório e eventual, destinando-se ao reconhecimento institucional dos trabalhos classificados. A Fapes pode alterar datas e prazos do cronograma por necessidade administrativa ou decisão institucional. O comparecimento do premiado é obrigatório. Caso não possa comparecer, deve indicar formalmente um representante para o recebimento da premiação, com comunicação prévia à Fapes, pelo e-mail gabinete@fapes.es.gov.br. Para as categorias Projetos e Destaque, as 3 (três) propostas com as maiores notas seguem para votação pelo Comitê de Especialistas. Para a categoria Jornalismo, as 3 (três) matérias com maiores notas seguem para votação popular.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 25/2025 - PARTICIPAÇÃO DE EQUIPES DE ESTUDANTES EM MOSTRAS E COMPETIÇÕES TÉCNICO-CIENTÍFICAS</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Conceder apoio financeiro a equipes formadas por estudantes de nível médio, de graduação e pós-graduação, coordenadas por um professor orientador. O objetivo é permitir a participação dessas equipes em mostras e competições técnico-científicas de âmbito regional, nacional ou internacional, visando a divulgação e difusão de resultados obtidos por instituições de ensino do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Professores(as) coordenadores(as) de equipes de 3 a 5 estudantes, vinculados(as) a instituições de ensino médio públicas ou instituições de ensino superior públicas ou privadas localizadas no estado do Espírito Santo. O proponente deve ter formação mínima de nível superior, vínculo ativo com a instituição, atuar em sala de aula na mesma instituição dos estudantes, ter Lattes atualizado há menos de 6 meses, estar regularizado junto à Fapes e morar no Espírito Santo ou municípios limítrofes. Estudantes de instituições privadas devem ser bolsistas integrais financiados por programas governamentais estaduais ou federais.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 500.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>?: Prazo para impugnação do edital (5 dias úteis antes do encerramento do prazo de submissão da 1ª Chamada)
 2025-11-10 a 2025-12-16: Submissão de propostas (Até as 17h:59. Para 1ª Chamada (eventos com início entre 01/03/2026 a 30/06/2026))
@@ -932,70 +1012,70 @@
 ?: Prazo para prestação de contas (Até 30 dias após o término da vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>O valor por proposta varia conforme a categoria do evento: R$ 500,00 para eventos regionais, R$ 1.200,00 para eventos nacionais e US$ 1.500,00 para eventos internacionais. O edital prevê três chamadas com períodos de submissão e eventos distintos. O início do evento proposto deve corresponder ao período da chamada selecionada. A Fapes pode alterar as datas e prazos definidos no cronograma. Cada coordenador pode apresentar apenas uma proposta. Não são contempladas propostas para participação em concursos ou premiações sem natureza acadêmica, técnico-científica ou tecnológica, ou competições esportivas.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_N_25_2025_Participação_Equipe_em_Mostras_e_Competições-2.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_N°_25_2025_-_PARTICIPAÇÃO_DE_EQUIPES_DE_ESTUDANTES_EM_MOSTRAS_E_COMPETIÇÕES_TÉCNICO-CIENTÍFICAS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>2026-09-06 a 2026-10-26: Submissão de propostas (4ª Chamada, até as 17h59)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. A chamada pública visa selecionar propostas para concessão de auxílio financeiro para tal finalidade, valorizando a produção técnico-científica e ampliando a visibilidade das atividades de pesquisa e inovação.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2025-12-22 a 2026-02-25: Submissão de propostas (1ª Chamada, até as 17h59)
 2026-02-17: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada)
@@ -1011,66 +1091,66 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga (prazo máximo de execução do projeto é de 12 meses))</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>O artigo deve ter sido aceito em periódico classificado entre A1 e A4 no Qualis-Capes (2021-2024) ou com percentil igual ou superior a 50% nas plataformas Scopus ou ISI Web of Science. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta por chamada; caso envie mais de uma, apenas a última será considerada. O prazo máximo para execução de cada projeto é de 12 meses.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Promover o aumento da competitividade dos setores econômicos capixabas por meio de projetos de inovação, desenvolvidos por empresas (incluindo cooperativas de trabalho) em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas. O apoio se dará por meio de um modelo de coinvestimento tripartite (FAPES, empresa/cooperativa, ICT/IES), com projetos alinhados ao Plano ES 500 Anos e ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas ou cooperativas de trabalho capixabas.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 500.000,00 a R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-03-30: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 ?: Prazo de submissão dos recursos administrativos (Habilitação) (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)
@@ -1079,153 +1159,89 @@
 ?: Submissão das documentações para contratação (Até 30 dias a partir da publicação do resultado homologado do julgamento de mérito.)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução do projeto é de 24 meses, com possibilidade de prorrogação por até 12 meses. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais; cooperativas de trabalho devem apresentar Demonstração de Sobras ou Perdas (DSP). As empresas devem estar ativas há pelo menos 6 meses e não podem ter sido contratadas em editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026, a menos que o projeto, coordenador e equipe executora sejam distintos. É permitida apenas uma proposta por empresa. Em caso de inabilitação ou desclassificação, a empresa poderá realizar uma nova submissão, exceto se reprovada pelo Comitê de Conformidade, o que impede nova submissão nesta chamada. A aprovação da proposta não garante a contratação, que está sujeita à disponibilidade financeira da FAPES, ordem de submissão e visita técnica. O critério de desempate é a data de submissão da proposta no SIGFAPES. Propostas com Nota Final inferior a 80 pontos ou notas individuais inferiores a 4 em critérios específicos serão desclassificadas. A impugnação dos termos do edital deve ser feita em até 5 dias úteis antes do encerramento do prazo de submissão das propostas do primeiro ciclo (considerando o fluxo contínuo, esta observação se refere a um prazo inicial para impugnação do edital em si).</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-08-25 a 2026-09-24: Submissão de propostas (até as 17h59, via SigFapes)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que ofereçam apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas com produtos, serviços ou modelos de negócio inovadores. O edital visa ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de empreendedores, a sustentabilidade econômica das empresas incubadas e o desenvolvimento socioeconômico do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Incubadoras, sem fins lucrativos, sediadas no Espírito Santo, que atendam aos requisitos do edital.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 252.000,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-08-25 a 2026-09-24: Submissão de propostas (até as 17h59, via SigFapes)
 2026-10-16: Interposição de recursos (Até 5 dias úteis após a divulgação do resultado preliminar)
 2026-11-04: Contratação dos projetos selecionados</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>O valor por proposta varia conforme o nível de maturidade da incubadora: Nível Avançado (R$ 252.000,00), Nível Intermediário (R$ 192.000,00) e Nível Básico (R$ 132.000,00). O projeto terá prazo de vigência de 24 meses, sem prorrogação. Propostas com nota final inferior a 70 pontos serão desclassificadas. A Fapes pode alterar o cronograma e redirecionar recursos remanescentes entre os níveis de maturidade. Os recursos de custeio (exceto bolsas) serão liberados em 2 parcelas. O orçamento do projeto pode ser aprovado parcial ou integralmente.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>€ 75.000,00</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1237,7 +1253,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1247,53 +1263,49 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
+          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1305,7 +1317,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1313,20 +1325,32 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1334,22 +1358,22 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
+          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1385,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1369,47 +1393,43 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
+      <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
         </is>
       </c>
       <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1441,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1429,52 +1449,47 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>US$ 6.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
-2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1486,7 +1501,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1498,92 +1513,157 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
+2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Este edital visa financiar projetos transnacionais de pesquisa e inovação em matérias-primas para a transição verde e digital. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Organizações de ensino superior e centros de pesquisa públicos. Os consórcios devem ser compostos por, no mínimo, três parceiros de três países diferentes (sendo pelo menos dois da UE ou países associados).</t>
         </is>
       </c>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)
 2026-09-22: Submissão de propostas nacionais FAPES (Etapa 1) (Recomendado verificar requisitos da FAPES para submissão na plataforma nacional, prazo idêntico ao da submissão da pré-proposta internacional.)
@@ -1597,17 +1677,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional / Início dos projetos (esperado)</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>O edital é um Joint Transnational Call (JTC) 2026 da Parceria Europeia em Matérias-Primas para a Transição Verde e Digital (RAMP). A FAPES (Fundação de Amparo à Pesquisa e Inovação do Espírito Santo) participa sob o guarda-chuva do CONFAP. Cada parceiro de projeto é financiado diretamente por sua respectiva agência nacional/regional. A Comissão Europeia cofinancia os JTCs da RAMP, com o cofinanciamento sendo redistribuído pelas agências financiadoras aos seus beneficiários. A duração máxima dos projetos é de 36 meses. Propostas devem se enquadrar em um dos seis tópicos temáticos e adotar princípios de 'Safe and Sustainable by Design'. Conforme a tabela de elegibilidade de parceiros do CONFAP, empresas (SMEs e grandes) e entidades sem fins lucrativos (ONGs, associações, sociedades, fundações) não são elegíveis para financiamento pela FAPES.</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-29 12:24
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -819,9 +811,9 @@
           <t>EDITAL FAPES Nº 24/2026 - PRIMEIROS PROJETOS DE PESQUISA - ESPÍRITO SANTO (PPP-ES)</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 28/08/2026</t>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-01 12:21
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1023,12 +1023,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Difusão do Conhecimento</t>
+          <t>Inovação</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
+          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1036,113 +1036,34 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-06 a 2026-10-26: Submissão de propostas (4ª Chamada, até as 17h59)</t>
-        </is>
-      </c>
+      <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. A chamada pública visa selecionar propostas para concessão de auxílio financeiro para tal finalidade, valorizando a produção técnico-científica e ampliando a visibilidade das atividades de pesquisa e inovação.</t>
+          <t>Promover o aumento da competitividade dos setores econômicos capixabas por meio de projetos de inovação, desenvolvidos por empresas (incluindo cooperativas de trabalho) em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas. O apoio se dará por meio de um modelo de coinvestimento tripartite (FAPES, empresa/cooperativa, ICT/IES), com projetos alinhados ao Plano ES 500 Anos e ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
+          <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas ou cooperativas de trabalho capixabas.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>R$ 800.000,00</t>
+          <t>R$ 40.000.000,00</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>US$ 1.500,00</t>
+          <t>R$ 500.000,00 a R$ 3.000.000,00</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>editais.duvidas@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>2025-12-22 a 2026-02-25: Submissão de propostas (1ª Chamada, até as 17h59)
-2026-02-17: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada)
-?: Interposição de recursos (1ª Chamada, 5 dias úteis após a publicação do resultado preliminar)
-2026-03-19 a 2026-05-25: Submissão de propostas (2ª Chamada, até as 17h59)
-?: Interposição de recursos (2ª Chamada, 5 dias úteis após a publicação do resultado preliminar)
-2026-06-19 a 2026-08-25: Submissão de propostas (3ª Chamada, até as 17h59)
-?: Interposição de recursos (3ª Chamada, 5 dias úteis após a publicação do resultado preliminar)
-2026-09-06 a 2026-10-26: Submissão de propostas (4ª Chamada, até as 17h59)
-?: Interposição de recursos (4ª Chamada, 5 dias úteis após a publicação do resultado preliminar)
-?: Contratação das propostas aprovadas (Até 30 dias após a publicação do resultado final homologado de cada chamada)
-?: Informar dados bancários (Até 30 dias após a assinatura e publicação do Termo de Outorga de cada projeto)
-?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga (prazo máximo de execução do projeto é de 12 meses))</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>O artigo deve ter sido aceito em periódico classificado entre A1 e A4 no Qualis-Capes (2021-2024) ou com percentil igual ou superior a 50% nas plataformas Scopus ou ISI Web of Science. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta por chamada; caso envie mais de uma, apenas a última será considerada. O prazo máximo para execução de cada projeto é de 12 meses.</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Inovação</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Promover o aumento da competitividade dos setores econômicos capixabas por meio de projetos de inovação, desenvolvidos por empresas (incluindo cooperativas de trabalho) em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas. O apoio se dará por meio de um modelo de coinvestimento tripartite (FAPES, empresa/cooperativa, ICT/IES), com projetos alinhados ao Plano ES 500 Anos e ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas ou cooperativas de trabalho capixabas.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>R$ 40.000.000,00</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>R$ 500.000,00 a R$ 3.000.000,00</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-03-30: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 ?: Prazo de submissão dos recursos administrativos (Habilitação) (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)
@@ -1151,31 +1072,101 @@
 ?: Submissão das documentações para contratação (Até 30 dias a partir da publicação do resultado homologado do julgamento de mérito.)</t>
         </is>
       </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>O prazo de execução do projeto é de 24 meses, com possibilidade de prorrogação por até 12 meses. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais; cooperativas de trabalho devem apresentar Demonstração de Sobras ou Perdas (DSP). As empresas devem estar ativas há pelo menos 6 meses e não podem ter sido contratadas em editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026, a menos que o projeto, coordenador e equipe executora sejam distintos. É permitida apenas uma proposta por empresa. Em caso de inabilitação ou desclassificação, a empresa poderá realizar uma nova submissão, exceto se reprovada pelo Comitê de Conformidade, o que impede nova submissão nesta chamada. A aprovação da proposta não garante a contratação, que está sujeita à disponibilidade financeira da FAPES, ordem de submissão e visita técnica. O critério de desempate é a data de submissão da proposta no SIGFAPES. Propostas com Nota Final inferior a 80 pontos ou notas individuais inferiores a 4 em critérios específicos serão desclassificadas. A impugnação dos termos do edital deve ser feita em até 5 dias úteis antes do encerramento do prazo de submissão das propostas do primeiro ciclo (considerando o fluxo contínuo, esta observação se refere a um prazo inicial para impugnação do edital em si).</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Inovação</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25 a 2026-09-24: Submissão de propostas (até as 17h59, via SigFapes)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que ofereçam apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas com produtos, serviços ou modelos de negócio inovadores. O edital visa ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de empreendedores, a sustentabilidade econômica das empresas incubadas e o desenvolvimento socioeconômico do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Incubadoras, sem fins lucrativos, sediadas no Espírito Santo, que atendam aos requisitos do edital.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>R$ 4.500.000,00</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>R$ 252.000,00</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>duvidas.inovacao@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25 a 2026-09-24: Submissão de propostas (até as 17h59, via SigFapes)
+2026-10-16: Interposição de recursos (Até 5 dias úteis após a divulgação do resultado preliminar)
+2026-11-04: Contratação dos projetos selecionados</t>
+        </is>
+      </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>O prazo de execução do projeto é de 24 meses, com possibilidade de prorrogação por até 12 meses. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais; cooperativas de trabalho devem apresentar Demonstração de Sobras ou Perdas (DSP). As empresas devem estar ativas há pelo menos 6 meses e não podem ter sido contratadas em editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026, a menos que o projeto, coordenador e equipe executora sejam distintos. É permitida apenas uma proposta por empresa. Em caso de inabilitação ou desclassificação, a empresa poderá realizar uma nova submissão, exceto se reprovada pelo Comitê de Conformidade, o que impede nova submissão nesta chamada. A aprovação da proposta não garante a contratação, que está sujeita à disponibilidade financeira da FAPES, ordem de submissão e visita técnica. O critério de desempate é a data de submissão da proposta no SIGFAPES. Propostas com Nota Final inferior a 80 pontos ou notas individuais inferiores a 4 em critérios específicos serão desclassificadas. A impugnação dos termos do edital deve ser feita em até 5 dias úteis antes do encerramento do prazo de submissão das propostas do primeiro ciclo (considerando o fluxo contínuo, esta observação se refere a um prazo inicial para impugnação do edital em si).</t>
+          <t>O valor por proposta varia conforme o nível de maturidade da incubadora: Nível Avançado (R$ 252.000,00), Nível Intermediário (R$ 192.000,00) e Nível Básico (R$ 132.000,00). O projeto terá prazo de vigência de 24 meses, sem prorrogação. Propostas com nota final inferior a 70 pontos serão desclassificadas. A Fapes pode alterar o cronograma e redirecionar recursos remanescentes entre os níveis de maturidade. Os recursos de custeio (exceto bolsas) serão liberados em 2 parcelas. O orçamento do projeto pode ser aprovado parcial ou integralmente.</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
+          <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Inovação</t>
+          <t>Chamadas Internacionais</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
+          <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1185,55 +1176,49 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 a 2026-09-24: Submissão de propostas (até as 17h59, via SigFapes)</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que ofereçam apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas com produtos, serviços ou modelos de negócio inovadores. O edital visa ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de empreendedores, a sustentabilidade econômica das empresas incubadas e o desenvolvimento socioeconômico do Espírito Santo.</t>
+          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Incubadoras, sem fins lucrativos, sediadas no Espírito Santo, que atendam aos requisitos do edital.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>R$ 4.500.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>R$ 252.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>duvidas.inovacao@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 a 2026-09-24: Submissão de propostas (até as 17h59, via SigFapes)
-2026-10-16: Interposição de recursos (Até 5 dias úteis após a divulgação do resultado preliminar)
-2026-11-04: Contratação dos projetos selecionados</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>O valor por proposta varia conforme o nível de maturidade da incubadora: Nível Avançado (R$ 252.000,00), Nível Intermediário (R$ 192.000,00) e Nível Básico (R$ 132.000,00). O projeto terá prazo de vigência de 24 meses, sem prorrogação. Propostas com nota final inferior a 70 pontos serão desclassificadas. A Fapes pode alterar o cronograma e redirecionar recursos remanescentes entre os níveis de maturidade. Os recursos de custeio (exceto bolsas) serão liberados em 2 parcelas. O orçamento do projeto pode ser aprovado parcial ou integralmente.</t>
+          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1230,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1255,49 +1240,53 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="n"/>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>R$ 150.000,00</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
+          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1298,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1317,32 +1306,20 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
-        </is>
-      </c>
+      <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>R$ 150.000,00</t>
-        </is>
-      </c>
+          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1350,22 +1327,22 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1354,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1385,43 +1362,47 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
         </is>
       </c>
       <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1433,7 +1414,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1441,47 +1422,52 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
+      <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
+          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
+2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
+          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1493,7 +1479,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1505,48 +1491,45 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>US$ 6.000,00</t>
+          <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
-2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
+?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
+?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
+          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1541,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1566,96 +1549,34 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)</t>
+        </is>
+      </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
+          <t>Este edital visa financiar projetos transnacionais de pesquisa e inovação em matérias-primas para a transição verde e digital. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
+          <t>Organizações de ensino superior e centros de pesquisa públicos. Os consórcios devem ser compostos por, no mínimo, três parceiros de três países diferentes (sendo pelo menos dois da UE ou países associados).</t>
         </is>
       </c>
       <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>€ 25.000,00 por ano de projeto</t>
+          <t>EUR 100.000,00</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
-?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
-?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Este edital visa financiar projetos transnacionais de pesquisa e inovação em matérias-primas para a transição verde e digital. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Organizações de ensino superior e centros de pesquisa públicos. Os consórcios devem ser compostos por, no mínimo, três parceiros de três países diferentes (sendo pelo menos dois da UE ou países associados).</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>EUR 100.000,00</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)
 2026-09-22: Submissão de propostas nacionais FAPES (Etapa 1) (Recomendado verificar requisitos da FAPES para submissão na plataforma nacional, prazo idêntico ao da submissão da pré-proposta internacional.)
@@ -1669,17 +1590,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional / Início dos projetos (esperado)</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>O edital é um Joint Transnational Call (JTC) 2026 da Parceria Europeia em Matérias-Primas para a Transição Verde e Digital (RAMP). A FAPES (Fundação de Amparo à Pesquisa e Inovação do Espírito Santo) participa sob o guarda-chuva do CONFAP. Cada parceiro de projeto é financiado diretamente por sua respectiva agência nacional/regional. A Comissão Europeia cofinancia os JTCs da RAMP, com o cofinanciamento sendo redistribuído pelas agências financiadoras aos seus beneficiários. A duração máxima dos projetos é de 36 meses. Propostas devem se enquadrar em um dos seis tópicos temáticos e adotar princípios de 'Safe and Sustainable by Design'. Conforme a tabela de elegibilidade de parceiros do CONFAP, empresas (SMEs e grandes) e entidades sem fins lucrativos (ONGs, associações, sociedades, fundações) não são elegíveis para financiamento pela FAPES.</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-04 11:46
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,22 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +59,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -524,25 +540,32 @@
           <t>EDITAL FAPES Nº 19/2026 - PIC JR 2027</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 04/09/2026</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09: Submissão de propostas (Até as 17h59)</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr"/>
+          <t>2026-09-14: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas.)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "O objetivo geral deste edital é selecionar projetos que despertem nos estudantes da Rede Pública de Educação Básica do Espírito Santo o interesse pela ciência, pelo desenvolvimento tecnológico e por ações de inovação. O programa apoia financeiramente projetos de pesquisa desenvolvidos em parceria entre escolas públicas de Educação Básica e Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo. Destina-se a pesquisadores, IES/P, professores e estudantes da Rede Pública de Educação Básica do Estado do Espírito Santo." → "Selecionar projetos que promovam o interesse pela ciência, desenvolvimento tecnológico e inovação em estudantes da Rede Pública de Educação Básica do Espírito Santo. O programa visa incentivar a participação ativa dos estudantes em pesquisa, popularizar a ciência na comunidade escolar, e fortalecer parcerias entre IES/P e escolas públicas para a formação de qualidade e inclusão social."
+Público-alvo: "Pesquisadores (mínimo mestre) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo, em parceria com professores e estudantes da Rede Pública de Educação Básica do Estado do Espírito Santo." → "Pesquisadores (mínimo mestre, com vínculo estatutário ou celetista por tempo indeterminado) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo."
+Valor por proposta: "R$ 10.000,00" → "-"
+Submissão (removida): Submissão de propostas — ? a 2026-09-09</t>
+        </is>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>O objetivo geral deste edital é selecionar projetos que despertem nos estudantes da Rede Pública de Educação Básica do Espírito Santo o interesse pela ciência, pelo desenvolvimento tecnológico e por ações de inovação. O programa apoia financeiramente projetos de pesquisa desenvolvidos em parceria entre escolas públicas de Educação Básica e Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo. Destina-se a pesquisadores, IES/P, professores e estudantes da Rede Pública de Educação Básica do Estado do Espírito Santo.</t>
+          <t>Selecionar projetos que promovam o interesse pela ciência, desenvolvimento tecnológico e inovação em estudantes da Rede Pública de Educação Básica do Espírito Santo. O programa visa incentivar a participação ativa dos estudantes em pesquisa, popularizar a ciência na comunidade escolar, e fortalecer parcerias entre IES/P e escolas públicas para a formação de qualidade e inclusão social.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores (mínimo mestre) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo, em parceria com professores e estudantes da Rede Pública de Educação Básica do Estado do Espírito Santo.</t>
+          <t>Pesquisadores (mínimo mestre, com vínculo estatutário ou celetista por tempo indeterminado) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -550,11 +573,7 @@
           <t>R$ 8.887.500,00</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>R$ 10.000,00</t>
-        </is>
-      </c>
+      <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
           <t>bolsas.duvidas@fapes.es.gov.br</t>
@@ -562,15 +581,16 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09: Submissão de propostas (Até as 17h59)
-?: Interposição de recursos (habilitação) (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação)
-?: Interposição de recursos (análise de mérito) (Até 5 dias úteis após a divulgação do resultado preliminar de análise de mérito)
+          <t>2026-09-14: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas.)
+2026-09-21: Envio da proposta e documentos (até as 17h59)
+?: Prazo para recorrer (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação)
+?: Prazo para recorrer (Até 5 dias úteis após a divulgação do resultado preliminar de análise de mérito)
 2027-02-09: Contratação dos projetos selecionados</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>O valor total do edital é distribuído por faixas (Educação Ambiental Formal, Práticas de Ciências da Natureza e Matemática, Bairros do Programa Estado Presente, Ampla Concorrência), com possibilidade de transferência de recursos entre elas. Além do auxílio financeiro de R$ 10.000,00 por projeto, são concedidas bolsas para coordenador (BCO), tutor (BTU), iniciação científica e tecnológica (ICT) e iniciação científica júnior (ICJr). Apenas as cinco bolsas de ICJr são obrigatórias. As bolsas BCO, BTU e ICT têm duração de até 10 meses, e as bolsas ICJr, até 9 meses. Os projetos devem ser inéditos para a Fapes. A Fapes abre mão dos direitos de participação e propriedade sobre pesquisas e projetos apoiados, mas os resultados econômicos da exploração comercial de criações protegidas serão partilhados.</t>
+          <t>O coordenador de cada projeto contratado recebe um auxílio financeiro de R$ 10.000,00. Somente as cinco bolsas de Iniciação Científica Júnior (ICJr) são obrigatórias para implementação; as demais modalidades (BCO, BTU e ICT) são opcionais. Os valores mensais das bolsas são definidos na Tabela de Valores de Bolsas e Auxílios da Fapes. Cada coordenador pode apresentar apenas uma proposta. É obrigatório mencionar o apoio da Fapes e Sedu em todas as publicações e divulgações de atividades. É obrigatória a comunicação formal à Fapes sobre criações intelectuais resultantes do projeto e a partilha de resultados econômicos.</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -595,25 +615,30 @@
           <t>EDITAL FAPES Nº 20/2026 - BOLSAS DE PÓS-DOUTORADO SÊNIOR</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 04/09/2026</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14: Solicitação de recursos de acessibilidade (Até 10 dias do término de submissão das propostas, via e-mail bolsas.duvidas@fapes.es.gov.br.)</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr"/>
+          <t>2026-09-19: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao término da submissão das propostas.)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Selecionar propostas para concessão de bolsas de pós-doutorado sênior, a serem realizadas em instituições de excelência no país ou no exterior. O objetivo é aprimorar a qualificação de pesquisadores, fortalecer as atividades de pesquisa científica e tecnológica, e ampliar a cooperação acadêmica nacional e internacional, contribuindo para o desenvolvimento científico e tecnológico no Espírito Santo e no Brasil." → "A presente chamada pública tem por objetivo selecionar propostas para concessão de bolsas de pós-doutorado sênior, a serem realizadas em instituições de excelência, no país ou no exterior. Visa o aprimoramento da qualificação de pesquisadores, o fortalecimento das atividades de pesquisa científica e tecnológica e a ampliação da cooperação acadêmica nacional e internacional. O edital apoia projetos de pesquisa que contribuam para o desenvolvimento científico e tecnológico no Espírito Santo e do Brasil."
+Público-alvo: "Pesquisadores doutores vinculados a Instituições de Ensino e/ou Pesquisa (IES/P), públicas ou privadas, sediadas no estado do Espírito Santo, que tenham obtido o título de doutor há mais de 8 anos, conforme faixas de titulação especificadas no edital." → "Pesquisador com título de doutor conforme discriminado nas faixas descritas no edital e com vínculo em Instituição de Ensino ou Pesquisa (IES/P), pública ou privada, sediada no estado do Espírito Santo."</t>
+        </is>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Selecionar propostas para concessão de bolsas de pós-doutorado sênior, a serem realizadas em instituições de excelência no país ou no exterior. O objetivo é aprimorar a qualificação de pesquisadores, fortalecer as atividades de pesquisa científica e tecnológica, e ampliar a cooperação acadêmica nacional e internacional, contribuindo para o desenvolvimento científico e tecnológico no Espírito Santo e no Brasil.</t>
+          <t>A presente chamada pública tem por objetivo selecionar propostas para concessão de bolsas de pós-doutorado sênior, a serem realizadas em instituições de excelência, no país ou no exterior. Visa o aprimoramento da qualificação de pesquisadores, o fortalecimento das atividades de pesquisa científica e tecnológica e a ampliação da cooperação acadêmica nacional e internacional. O edital apoia projetos de pesquisa que contribuam para o desenvolvimento científico e tecnológico no Espírito Santo e do Brasil.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores doutores vinculados a Instituições de Ensino e/ou Pesquisa (IES/P), públicas ou privadas, sediadas no estado do Espírito Santo, que tenham obtido o título de doutor há mais de 8 anos, conforme faixas de titulação especificadas no edital.</t>
+          <t>Pesquisador com título de doutor conforme discriminado nas faixas descritas no edital e com vínculo em Instituição de Ensino ou Pesquisa (IES/P), pública ou privada, sediada no estado do Espírito Santo.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -629,17 +654,16 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao término da submissão das propostas, via Formulário de Impugnação de Edital no E-Flow.)
-2026-09-14: Solicitação de recursos de acessibilidade (Até 10 dias do término de submissão das propostas, via e-mail bolsas.duvidas@fapes.es.gov.br.)
-2026-09-24: Submissão de propostas (Até as 17h59, via Sistema de Informação e Gestão de Projetos da Fapes.)
-?: Prazo para recurso administrativo (habilitação) (5 dias úteis após a publicação do resultado preliminar de habilitação, via Formulário de Recurso Administrativo no E-Flow.)
-?: Prazo para recurso administrativo (classificação) (5 dias úteis após a publicação do resultado preliminar de classificação, via Formulário de Recurso Administrativo no E-Flow.)
-2027-01-18: Contratação das propostas (A partir desta data, com assinatura eletrônica do Termo de Outorga via E-Docs (Acesso Cidadão).)</t>
+          <t>2026-09-19: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao término da submissão das propostas.)
+2026-09-24: Submissão das propostas (Até as 17h59)
+?: Prazo para recurso administrativo (5 dias após a publicação do resultado preliminar de habilitação)
+?: Prazo para recurso administrativo (5 dias após a publicação do resultado preliminar de classificação)
+2027-01-18: Contratação das propostas</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>O prazo de execução do projeto é de 16 meses, improrrogáveis, exceto em caso de Advento de Prole. Cada proponente pode apresentar apenas uma proposta; a última enviada será considerada. Os resultados são publicados no Diário Oficial do Estado do Espírito Santo (DIO-ES) e detalhados no site da Fapes. O beneficiário tem um interstício de 16 meses a partir do início da vigência do Termo de Outorga para iniciar e finalizar a bolsa. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. As atividades de pesquisa devem ser realizadas presencialmente na Instituição de Destino, sem modalidade à distância. Não é permitida a alteração da Instituição de Destino ou do Supervisor após a submissão da proposta. O proponente deve ser o bolsista POSDOC. A duração mínima do estágio pós-doutoral é de 6 meses e máxima de 10 meses. Casos omissos e dúvidas de interpretação serão dirimidos pela Direx.</t>
+          <t>Cada proponente deve apresentar apenas uma proposta. Caso envie mais de uma, apenas a última será considerada. Não é admitida a alteração da Instituição Destino ou do Supervisor após a submissão da proposta. O proponente pode solicitar correção de erros materiais na proposta ou documentação, desde que não comprometam a análise ou representem vantagem competitiva. A concessão de recursos de acessibilidade é avaliada por viabilidade e razoabilidade, se solicitada em até 10 dias do término da submissão. Recursos administrativos não podem envolver mudanças na proposta original, ser apresentados fora do prazo ou incluir/substituir documentos após o envio da proposta. A convocação de suplentes pode ocorrer em casos de desistência, não contratação ou ampliação de recursos. O beneficiário tem um interstício de 16 meses a partir do início da vigência do Termo de Outorga para iniciar e finalizar a bolsa. Não haverá prorrogação do prazo de vigência do Termo de Outorga, exceto em caso de Advento de Prole. O bolsista pode ser penalizado mesmo que a inadimplência seja regularizada.</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -664,25 +688,32 @@
           <t>EDITAL FAPES/CNPq/CAPES Nº 22/2026 - PROGRAMA DE APOIO À FIXAÇÃO DE DOUTORES NO BRASIL (PROFIX-CB)</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 04/09/2026</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01: Submissão das propostas (Até as 17h59, via Sistema de Informação e Gestão de Projetos da Fapes)</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr"/>
+          <t>2026-09-24: Prazo para impugnação do edital (até 5 dias úteis anteriores ao encerramento do prazo de submissão das propostas)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "O Programa de Apoio à Fixação de Doutores no Brasil – Conhecimento Brasil (PROFIX-CB) é uma iniciativa do CNPq, CAPES e FAPs para atrair, inserir e fixar pesquisadores doutores em instituições de pesquisa, universidades e centros de inovação no país. Seu propósito é criar condições para que o doutor estabeleça uma trajetória científica de médio prazo, contribuindo para a formação de recursos humanos, fortalecimento de programas de pós-graduação, consolidação de grupos de pesquisa e geração de conhecimento e inovação, especialmente em áreas estratégicas para o desenvolvimento científico, tecnológico e de inovação do Espírito Santo." → "O Programa de Apoio à Fixação de Doutores no Brasil – Conhecimento Brasil (PROFIX-CB) é uma iniciativa do CNPq, CAPES e FAPs para atrair, inserir e fixar pesquisadores doutores em instituições de pesquisa, universidades e centros de inovação no país, especialmente em áreas estratégicas para o desenvolvimento científico, tecnológico e de inovação. O objetivo é apoiar projetos de pesquisa que criem condições para que recém-doutores sem vínculo empregatício desenvolvam uma trajetória científica de médio prazo no Espírito Santo, contribuindo para a formação de recursos humanos, fortalecimento de programas de pós-graduação, consolidação de grupos de pesquisa e geração de conhecimento e inovação, alinhado ao Plano Estadual de CT&amp;I do Espírito Santo (PCTI-ES) 2026–2035."
+Público-alvo: "Pesquisadores doutores (com título obtido há no máximo 10 anos até a data limite de submissão da proposta), residentes no Espírito Santo, sem vínculo empregatício, que atuarão como coordenadores e bolsistas PROFIX-CB em Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no Espírito Santo, com um Programa de Pós-graduação (PPG) parceiro." → "Pesquisadores doutores com título obtido há no máximo 10 anos, residentes no Espírito Santo durante a execução do projeto, com disponibilidade de 40 horas semanais presenciais, não aposentados, sem vínculo empregatício ou acúmulo de bolsas no momento da contratação e durante as atividades como bolsista PROFIX-CB. Devem estar vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, com registro ativo no Diretório de Instituições do CNPq e anuência do PPG parceiro."
+Valor por proposta: "R$ 400.000,00" → "R$ 400.000,00 (auxílio financeiro da Fapes)"
+Contato: "bolsas.duvidas@fapes.es.gov.br" → "bolsas.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br"</t>
+        </is>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>O Programa de Apoio à Fixação de Doutores no Brasil – Conhecimento Brasil (PROFIX-CB) é uma iniciativa do CNPq, CAPES e FAPs para atrair, inserir e fixar pesquisadores doutores em instituições de pesquisa, universidades e centros de inovação no país. Seu propósito é criar condições para que o doutor estabeleça uma trajetória científica de médio prazo, contribuindo para a formação de recursos humanos, fortalecimento de programas de pós-graduação, consolidação de grupos de pesquisa e geração de conhecimento e inovação, especialmente em áreas estratégicas para o desenvolvimento científico, tecnológico e de inovação do Espírito Santo.</t>
+          <t>O Programa de Apoio à Fixação de Doutores no Brasil – Conhecimento Brasil (PROFIX-CB) é uma iniciativa do CNPq, CAPES e FAPs para atrair, inserir e fixar pesquisadores doutores em instituições de pesquisa, universidades e centros de inovação no país, especialmente em áreas estratégicas para o desenvolvimento científico, tecnológico e de inovação. O objetivo é apoiar projetos de pesquisa que criem condições para que recém-doutores sem vínculo empregatício desenvolvam uma trajetória científica de médio prazo no Espírito Santo, contribuindo para a formação de recursos humanos, fortalecimento de programas de pós-graduação, consolidação de grupos de pesquisa e geração de conhecimento e inovação, alinhado ao Plano Estadual de CT&amp;I do Espírito Santo (PCTI-ES) 2026–2035.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores doutores (com título obtido há no máximo 10 anos até a data limite de submissão da proposta), residentes no Espírito Santo, sem vínculo empregatício, que atuarão como coordenadores e bolsistas PROFIX-CB em Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no Espírito Santo, com um Programa de Pós-graduação (PPG) parceiro.</t>
+          <t>Pesquisadores doutores com título obtido há no máximo 10 anos, residentes no Espírito Santo durante a execução do projeto, com disponibilidade de 40 horas semanais presenciais, não aposentados, sem vínculo empregatício ou acúmulo de bolsas no momento da contratação e durante as atividades como bolsista PROFIX-CB. Devem estar vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, com registro ativo no Diretório de Instituições do CNPq e anuência do PPG parceiro.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -692,30 +723,25 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>R$ 400.000,00</t>
+          <t>R$ 400.000,00 (auxílio financeiro da Fapes)</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>bolsas.duvidas@fapes.es.gov.br</t>
+          <t>bolsas.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01: Submissão das propostas (Até as 17h59, via Sistema de Informação e Gestão de Projetos da Fapes)
-?: Interposição de recursos (Até 5 dias úteis após a divulgação do resultado preliminar)
-2027-01-04: Contratação dos projetos e assinatura do Termo de Outorga (A partir de, via Acesso Cidadão e Sistema de Informação e Gestão de Projetos da Fapes)
-?: Envio de dados bancários para recebimento de recursos (Até 30 dias após a contratação)
-?: Indicação de bolsistas de mestrado e doutorado (Capes) (Até 12 meses após o início da vigência do projeto)
-?: Prestação de contas parcial (A cada 12 meses de vigência do projeto)
-?: Prestação de contas final (Até 30 dias após o término da vigência do Termo de Outorga)
-?: Envio de Relatório Técnico da Bolsa PROFIX-CB (Até 60 dias após o término da vigência do processo CNPq)
-?: Envio de Relatório Final de Bolsas de Pós-graduação (Capes) (Até 30 dias após o término da bolsa)</t>
+          <t>2026-09-24: Prazo para impugnação do edital (até 5 dias úteis anteriores ao encerramento do prazo de submissão das propostas)
+2026-10-01: Submissão de propostas (até as 17h59)
+?: Interposição de recursos (seleção) (até 5 dias úteis após a divulgação do resultado preliminar)
+2027-01-04: Contratação dos projetos (A partir de)</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>A proposta deve ter cronograma de atividades de 48 meses. O projeto tem vigência de 48 meses. A bolsa PROFIX-CB tem duração de 48 meses. As bolsas de doutorado (Capes) têm duração de até 48 meses, e as de mestrado (Capes) até 24 meses. As bolsas de Iniciação Científica e Tecnológica (Fapes) têm duração de até 12 meses, podendo ser prorrogadas por mais duas vezes. É obrigatório mencionar o apoio da Fapes, CNPq e Capes em todas as publicações e divulgações. Os resultados de propriedade intelectual devem ser comunicados à Fapes. A Fapes abre mão dos direitos de participação e propriedade sobre pesquisas e projetos que apoia, conforme previsto em legislação específica. A convocação de suplentes pode ocorrer por até 24 meses após a divulgação do resultado final. Os anexos do edital estão disponíveis no site da Fapes em 'Editais Abertos'. Dúvidas sobre a chamada devem ser enviadas em até 2 dias antes do término da submissão das propostas.</t>
+          <t>É permitida a participação do mesmo coordenador em Chamadas Públicas PROFIX-CB promovidas por diferentes Fundações de Amparo à Pesquisa. Entretanto, é vedada sua contratação pela Fapes caso tenha sido contratado no âmbito do Programa PROFIX-CB por Fundação de Amparo à Pesquisa de qualquer outra Unidade da Federação ou do Distrito Federal. Constatada, a qualquer tempo, a contratação do coordenador por outra Fundação de Amparo à Pesquisa no âmbito do Programa PROFIX-CB, sua proposta é eliminada desta Chamada e, caso a concessão pela Fapes já tenha sido implementada, é cancelada, sem prejuízo da comunicação ao CNPq, à Capes e à respectiva Fundação de Amparo à Pesquisa para adoção das providências cabíveis. Cada proposta deve contemplar 1 bolsa PROFIX-CB e pode ainda, contemplar: Até 1 bolsa de doutorado (48 meses), Até 1 bolsa de mestrado (24 meses), Até 4 bolsas de Iniciação Científica e Tecnológica (ICT) (12 meses). A bolsa PROFIX-CB é destinada obrigatoriamente ao coordenador do projeto e tem duração de 48 meses. Não é permitida a substituição do bolsista coordenador em caso de cancelamento da bolsa. Os anexos do edital estão disponíveis no site da Fapes (Fapes - Editais Abertos) em formato Word para facilitar a edição pelos proponentes. A prestação de contas parcial deve ser apresentada a cada 12 meses de vigência e a final em até 30 dias após o término da vigência do Termo de Outorga. O coordenador deve encaminhar o Relatório de Execução do Objeto (REO) ao CNPq em até 60 dias após o término da vigência do processo do CNPq. Bolsistas de pós-graduação devem enviar o Relatório Final à Capes em até 30 dias após o término da bolsa. É obrigatório mencionar o apoio da Fapes, CNPq e Capes em todas as publicações e divulgações. A Fapes abre mão dos direitos de participação e propriedade sobre pesquisas e projetos que apoia, conforme Lei Complementar nº 978/2021, mas os resultados econômicos da exploração comercial da criação protegida são partilhados com a Fapes. A convocação de suplentes pode ocorrer em casos de desistência, não contratação ou ampliação de recursos, com validade de 24 meses a contar da divulgação do resultado final. A concessão de adaptações para acessibilidade é avaliada segundo critérios de viabilidade e razoabilidade, mediante solicitação em até 10 dias do término de submissão das propostas.</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -1023,47 +1049,127 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Inovação</t>
+          <t>Extensão</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr"/>
+          <t>EDITAL FAPES Nº 01/2026 – TCC EMPREENDEDOR INOVADOR</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 04/09/2026</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02 a 2026-10-27: Período de submissão das propostas (Segunda Chamada) (Até 17h59)</t>
+        </is>
+      </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
+          <t>Incentivar o desenvolvimento de Trabalhos de Conclusão de Curso (TCCs) com foco em inovação, empreendedorismo e aplicabilidade prática. O edital visa a concessão de Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC) para a execução de TCCs que apresentem soluções inovadoras e empreendedoras. As propostas devem ter fundamentação teórico-metodológica consistente, voltadas para aplicação prática e impacto econômico, social e/ou ambiental no Estado do Espírito Santo, alinhados aos ODS da ONU e ao Plano ES 500 Anos.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Professores orientadores com vínculo estatutário ou celetista por tempo indeterminado com Instituição de Ensino Superior (IES) reconhecida pelo Ministério da Educação (MEC), localizada no Espírito Santo, que submetam entre 3 (três) e 5 (cinco) propostas.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 1.600.000,00</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 11.000,00</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>?: Impugnação do Edital (Até 5 (cinco) dias úteis antes do encerramento do prazo de submissão das propostas de cada chamada.)
+2026-02-02 a 2026-03-30: Período de submissão das propostas (Primeira Chamada) (Até 17h59)
+?: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 (cinco) dias úteis a partir da publicação do resultado de seleção da Primeira Chamada.)
+?: Prazo de contratação (Primeira Chamada) (Até 5 (cinco) dias úteis da publicação do resultado homologado da Primeira Chamada.)
+2026-09-02 a 2026-10-27: Período de submissão das propostas (Segunda Chamada) (Até 17h59)
+?: Prazo para interposição de recursos administrativos (Segunda Chamada) (5 (cinco) dias úteis a partir da publicação do resultado de seleção da Segunda Chamada.)
+?: Prazo de contratação (Segunda Chamada) (Até 5 (cinco) dias úteis da publicação do resultado homologado da Segunda Chamada.)
+2027-02-02 a 2027-03-30: Período de submissão das propostas (Terceira Chamada) (Até 17h59)
+?: Prazo para interposição de recursos administrativos (Terceira Chamada) (5 (cinco) dias úteis a partir da publicação do resultado de seleção da Terceira Chamada.)
+?: Prazo de contratação (Terceira Chamada) (Até 5 (cinco) dias úteis da publicação do resultado homologado da Terceira Chamada.)
+XX.XX.20XX: Contratação de suplentes (Período de, se aplicável.)
+?: Prazo para envio de dados bancários (Até 30 (trinta) dias corridos, contados a partir da data de início da vigência do Termo de Outorga publicada no Diário Oficial do Espírito Santo.)
+?: Prazo para solicitação de ofício para abertura de conta (Até 3 (três) dias úteis para o Outorgado.)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>O prazo de execução dos projetos será de um semestre letivo, acrescido de até 3 (três) meses apenas para apresentação da Declaração ou Ata de Defesa do TCC. Cada projeto de TCC deve demonstrar potencial de geração de valor, criação de negócios ou produtos inovadores; estar alinhado aos ODS da ONU (especialmente ODS 4, 8, 9, 10 e 17) e ao Plano ES 500 Anos, e ser desenvolvido em consonância com os Projetos Pedagógicos dos respectivos cursos de graduação. As propostas concorrerão com as demais de suas respectivas microrregiões, sendo apoiados, na primeira chamada, no máximo 20 (vinte) projetos de TCC por microrregião e, na segunda e terceira chamadas, até 10 (dez) projetos de TCC por microrregião. Recursos remanescentes serão destinados a projetos em ampla concorrência por ordem decrescente de nota. Propostas submetidas a mais de uma microrregião serão desclassificadas. Cada proposta deverá vincular um único aluno sob orientação do proponente. O proponente que indicar alunos orientados vinculados a outra IES deverá apresentar declaração de autorização tanto da sua IES de vínculo quanto da IES à qual os alunos orientados estão vinculados. Propostas com Nota Final (NF) inferior a 70 (setenta) pontos serão desclassificadas. Não será permitido o acúmulo de bolsas Fapes pelo aluno orientado, exceto com bolsas do Programa Nossa Bolsa, do Programa Universidade para Todos (Prouni) e com Bolsas de Extensão (Ext-E e Ext-F) da Fapes.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_01.2026_TCC_EMPREENDEDOR_INOVADOR-2.pdf</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>extensao/EDITAL_FAPES_No_01_2026_–_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Inovação</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>Promover o aumento da competitividade dos setores econômicos capixabas por meio de projetos de inovação, desenvolvidos por empresas (incluindo cooperativas de trabalho) em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas. O apoio se dará por meio de um modelo de coinvestimento tripartite (FAPES, empresa/cooperativa, ICT/IES), com projetos alinhados ao Plano ES 500 Anos e ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas ou cooperativas de trabalho capixabas.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 500.000,00 a R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-03-30: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 ?: Prazo de submissão dos recursos administrativos (Habilitação) (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)
@@ -1072,153 +1178,95 @@
 ?: Submissão das documentações para contratação (Até 30 dias a partir da publicação do resultado homologado do julgamento de mérito.)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução do projeto é de 24 meses, com possibilidade de prorrogação por até 12 meses. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais; cooperativas de trabalho devem apresentar Demonstração de Sobras ou Perdas (DSP). As empresas devem estar ativas há pelo menos 6 meses e não podem ter sido contratadas em editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026, a menos que o projeto, coordenador e equipe executora sejam distintos. É permitida apenas uma proposta por empresa. Em caso de inabilitação ou desclassificação, a empresa poderá realizar uma nova submissão, exceto se reprovada pelo Comitê de Conformidade, o que impede nova submissão nesta chamada. A aprovação da proposta não garante a contratação, que está sujeita à disponibilidade financeira da FAPES, ordem de submissão e visita técnica. O critério de desempate é a data de submissão da proposta no SIGFAPES. Propostas com Nota Final inferior a 80 pontos ou notas individuais inferiores a 4 em critérios específicos serão desclassificadas. A impugnação dos termos do edital deve ser feita em até 5 dias úteis antes do encerramento do prazo de submissão das propostas do primeiro ciclo (considerando o fluxo contínuo, esta observação se refere a um prazo inicial para impugnação do edital em si).</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Inovação</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-25 a 2026-09-24: Submissão de propostas (até as 17h59, via SigFapes)</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que ofereçam apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas com produtos, serviços ou modelos de negócio inovadores. O edital visa ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de empreendedores, a sustentabilidade econômica das empresas incubadas e o desenvolvimento socioeconômico do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Incubadoras, sem fins lucrativos, sediadas no Espírito Santo, que atendam aos requisitos do edital.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>R$ 4.500.000,00</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>R$ 252.000,00</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>duvidas.inovacao@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-25 a 2026-09-24: Submissão de propostas (até as 17h59, via SigFapes)
-2026-10-16: Interposição de recursos (Até 5 dias úteis após a divulgação do resultado preliminar)
-2026-11-04: Contratação dos projetos selecionados</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>O valor por proposta varia conforme o nível de maturidade da incubadora: Nível Avançado (R$ 252.000,00), Nível Intermediário (R$ 192.000,00) e Nível Básico (R$ 132.000,00). O projeto terá prazo de vigência de 24 meses, sem prorrogação. Propostas com nota final inferior a 70 pontos serão desclassificadas. A Fapes pode alterar o cronograma e redirecionar recursos remanescentes entre os níveis de maturidade. Os recursos de custeio (exceto bolsas) serão liberados em 2 parcelas. O orçamento do projeto pode ser aprovado parcial ou integralmente.</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Chamadas Internacionais</t>
+          <t>Inovação</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 04/09/2026</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
+          <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas. O pedido deve ser enviado no E-Flow por meio do Formulário de Impugnação de Edital.)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que ofereçam apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas com produtos, serviços ou modelos de negócio inovadores. O edital visa ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de empreendedores, a sustentabilidade econômica das empresas incubadas e o desenvolvimento socioeconômico do Espírito Santo." → "O edital visa apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que buscam estimular e prestar apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas com produtos, serviços ou modelos de negócio inovadores. Este apoio busca ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de novos empreendedores e o desenvolvimento socioeconômico do estado."
+Submissão (removida): Submissão de propostas — 2026-08-25 a 2026-09-24</t>
+        </is>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
+          <t>O edital visa apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que buscam estimular e prestar apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas com produtos, serviços ou modelos de negócio inovadores. Este apoio busca ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de novos empreendedores e o desenvolvimento socioeconômico do estado.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="n"/>
+          <t>Incubadoras, sem fins lucrativos, sediadas no Espírito Santo, que atendam aos requisitos do edital.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>R$ 4.500.000,00</t>
+        </is>
+      </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>R$ 252.000,00</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas. O pedido deve ser enviado no E-Flow por meio do Formulário de Impugnação de Edital.)
+2026-08-25 a 2026-09-24: Envio da proposta e documentos (Até as 17h59, via SigFapes)
+?: Prazo para recorrer (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação e análise de mérito)
+2026-11-04: Contratação dos projetos selecionados (A partir desta data)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
+          <t>O projeto terá prazo de vigência de 24 meses, sem prorrogação. Os recursos financeiros remanescentes, caso o número de propostas previstas para contratação nos níveis de maturidade I, II ou III não seja alcançado, serão redirecionados para propostas suplentes. Os recursos destinados ao custeio (exceto bolsas) serão liberados em 2 parcelas. Caso a proposta seja enquadrada em nível de maturidade distinto do indicado pelo proponente, os valores financiáveis serão ajustados proporcionalmente. É obrigatório destinar no mínimo 20% do valor total solicitado para bolsas. As incubadoras beneficiárias devem destinar parte dos recursos de custeio à associação à Anprotec. Propostas com nota final inferior a 60 pontos serão desclassificadas. A classificação por nível de maturidade é a seguinte: Nível Avançado (86 a 100 pontos), Nível Intermediário (76 a 85 pontos), Nível Básico (60 a 75 pontos).</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
+          <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1278,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1240,53 +1288,49 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Apoiar projetos colaborativos de pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. Destina-se a profissionais vinculados a universidades, centros de pesquisa ou empresas do Espírito Santo que desenvolvam atividades de P,D&amp;I e que apresentem propostas conjuntas com empresas espanholas.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, residentes no Espírito Santo, com vínculo ativo a universidades, centros de pesquisa ou empresas localizadas no estado do Espírito Santo, que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica e que integrem proposta conjunta com empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+          <t>2026-10-08: Submissão de propostas (Até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Os formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
+          <t>A FAPES apoiará um único projeto. Os projetos terão duração de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. Cada proponente pode submeter apenas uma proposta. A submissão à FAPES (via SigFapes) para contratação ocorrerá somente após a aprovação da proposta pelo CDTI. Os projetos devem ter um orçamento total mínimo de € 250.000,00, e o apoio da FAPES deve corresponder a no mínimo 30% da contrapartida do valor total da proposta.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1342,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1306,20 +1350,32 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
+        </is>
+      </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1327,22 +1383,22 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília), exclusivamente por meio da plataforma https://sistema.confap.org.br.)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
+          <t>Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas. O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, excluindo bolsas. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, apenas a última será considerada. As propostas devem ser submetidas utilizando o modelo do Anexo I (Application Form Template) em ambas as plataformas (CONFAP).</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1410,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1362,47 +1418,43 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
+      <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
+          <t>Apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem selecionados pelo Serviço Alemão de Intercâmbio Acadêmico (DAAD). O suporte visa permitir que esses bolsistas realizem suas pesquisas em instituições na Alemanha, no âmbito da Chamada DAAD 2026.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+          <t>Bolsistas de doutorado da FAPES que forem selecionados pelo DAAD, que estejam adimplentes junto à FAPES e que não estejam no primeiro nem no último ano do doutorado.</t>
         </is>
       </c>
       <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+          <t>?: Submissão de propostas (As propostas deverão ser submetidas na Plataforma do DAAD, conforme item 3.1.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada DAAD 2026, complementando o edital completo disponível no site do CONFAP.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1466,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1422,52 +1474,47 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+          <t>O edital MOBILITY CONFAP ITALY CALL 2026 visa apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa brasileiras, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação por meio da mobilidade de estudantes de doutorado, mestrado e pós-doutorado. O suporte é oferecido na forma de bolsas de estudo para fortalecer grupos de pesquisa brasileiros através de colaborações e visitas a grupos de pesquisa na Itália, parte da rede MCI.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>US$ 6.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa nos Estados brasileiros participantes, que possuam um supervisor associado a uma universidade italiana parte da rede MCI.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
-2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
+          <t>As FAPs participantes podem exigir critérios de elegibilidade adicionais e definir as modalidades de apoio, incluindo os valores das bolsas mensais, em suas próprias diretrizes ou orientações, devendo ser consultadas pelos candidatos antes da preparação da proposta. Não serão cobradas taxas de matrícula por nenhuma das partes para qualquer mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio deverão assinar um acordo de colaboração específico. As propostas devem incluir: projeto de pesquisa, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do supervisor (Itália) e carta de apoio do supervisor na universidade italiana. As FAPs podem solicitar documentos adicionais. As vagas e oportunidades de pesquisa nas universidades italianas da rede MCI estão disponíveis em https://site.unibo.it/mobility-confap-italy/en/research-opportunity-offers-in-italy. Detalhes da rede MCI italiana em https://site.unibo.it/mobility-confap-italy/en/mci-program/network-of-italian-university. As FAPs associadas a esta chamada são: Alagoas - FAPEAL, Amazonas - FAPEAM, Bahia - FAPESB, Ceará - FUNCAP, Espírito Santo – FAPES, Goiás - FAPEG, Maranhão - FAPEMA, Pará - FAPESPA, Paraná - Fundação Araucária, Pernambuco – FACEPE, Rio Grande do Sul - FAPERGS, Santa Catarina - FAPESC. Outras FAPs podem confirmar sua participação.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1526,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1491,92 +1538,157 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O objetivo é possibilitar colaborações de pesquisa, promover oportunidades em equipes internacionais de excelência e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de doutor, que implementam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros. Para FAPES, o proponente deve ser pesquisador principal ou coordenador do projeto, vinculado a IES/P no Espírito Santo, residente no estado, brasileiro ou estrangeiro com visto permanente, com currículo Lattes atualizado, adimplente com a FAPES e em regularidade perante as normas legais vigentes.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Propostas completas, incluindo todos os documentos solicitados no Item 6 do edital geral, devem ser submetidas via portal https://sistema.confap.org.br/.)
+2026-08-10: Submissão de documentação para verificação de elegibilidade (FAPES) (Submeter via SigFapes a documentação exigida conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B do edital específico da FAPES.)</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará até 3 projetos selecionados. Os recursos podem ser usados como auxílios individuais para estágios ou visitas técnicas de curta duração. O acesso à lista de projetos ERC é liberado após análise de elegibilidade básica pelo CONFAP. Os pesquisadores devem contatar os PIs dos projetos ERC para definir o Plano de Trabalho e condições.</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Este edital visa financiar projetos transnacionais de pesquisa e inovação em matérias-primas para a transição verde e digital. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Organizações de ensino superior e centros de pesquisa públicos. Os consórcios devem ser compostos por, no mínimo, três parceiros de três países diferentes (sendo pelo menos dois da UE ou países associados).</t>
         </is>
       </c>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (Até as 15:00 CEST)
 2026-09-22: Submissão de propostas nacionais FAPES (Etapa 1) (Recomendado verificar requisitos da FAPES para submissão na plataforma nacional, prazo idêntico ao da submissão da pré-proposta internacional.)
@@ -1590,17 +1702,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional / Início dos projetos (esperado)</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>O edital é um Joint Transnational Call (JTC) 2026 da Parceria Europeia em Matérias-Primas para a Transição Verde e Digital (RAMP). A FAPES (Fundação de Amparo à Pesquisa e Inovação do Espírito Santo) participa sob o guarda-chuva do CONFAP. Cada parceiro de projeto é financiado diretamente por sua respectiva agência nacional/regional. A Comissão Europeia cofinancia os JTCs da RAMP, com o cofinanciamento sendo redistribuído pelas agências financiadoras aos seus beneficiários. A duração máxima dos projetos é de 36 meses. Propostas devem se enquadrar em um dos seis tópicos temáticos e adotar princípios de 'Safe and Sustainable by Design'. Conforme a tabela de elegibilidade de parceiros do CONFAP, empresas (SMEs e grandes) e entidades sem fins lucrativos (ONGs, associações, sociedades, fundações) não são elegíveis para financiamento pela FAPES.</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-05 10:39
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,7 +29,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -39,11 +39,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -59,7 +54,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -68,9 +63,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -542,30 +534,28 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Atualizado - e-mail enviado em 04/09/2026</t>
+          <t>Atualizado - e-mail enviado em 05/09/2026</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas.)</t>
+          <t>2026-09-21: Submissão de propostas e documentos (Até as 17h59)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Objetivo: "O objetivo geral deste edital é selecionar projetos que despertem nos estudantes da Rede Pública de Educação Básica do Espírito Santo o interesse pela ciência, pelo desenvolvimento tecnológico e por ações de inovação. O programa apoia financeiramente projetos de pesquisa desenvolvidos em parceria entre escolas públicas de Educação Básica e Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo. Destina-se a pesquisadores, IES/P, professores e estudantes da Rede Pública de Educação Básica do Estado do Espírito Santo." → "Selecionar projetos que promovam o interesse pela ciência, desenvolvimento tecnológico e inovação em estudantes da Rede Pública de Educação Básica do Espírito Santo. O programa visa incentivar a participação ativa dos estudantes em pesquisa, popularizar a ciência na comunidade escolar, e fortalecer parcerias entre IES/P e escolas públicas para a formação de qualidade e inclusão social."
-Público-alvo: "Pesquisadores (mínimo mestre) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo, em parceria com professores e estudantes da Rede Pública de Educação Básica do Estado do Espírito Santo." → "Pesquisadores (mínimo mestre, com vínculo estatutário ou celetista por tempo indeterminado) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo."
-Valor por proposta: "R$ 10.000,00" → "-"
-Submissão (removida): Submissão de propostas — ? a 2026-09-09</t>
+          <t>Objetivo: "Selecionar projetos que promovam o interesse pela ciência, desenvolvimento tecnológico e inovação em estudantes da Rede Pública de Educação Básica do Espírito Santo. O programa visa incentivar a participação ativa dos estudantes em pesquisa, popularizar a ciência na comunidade escolar, e fortalecer parcerias entre IES/P e escolas públicas para a formação de qualidade e inclusão social." → "O Programa de Iniciação Científica Júnior (PICJr) visa apoiar financeiramente projetos de pesquisa desenvolvidos em parceria entre escolas públicas de Educação Básica e Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo. O objetivo é aproximar estudantes da rede pública de práticas científicas, sob a orientação de um pesquisador coordenador e a coorientação de um professor tutor, despertando o interesse pela ciência, desenvolvimento tecnológico e inovação."
+Público-alvo: "Pesquisadores (mínimo mestre, com vínculo estatutário ou celetista por tempo indeterminado) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo." → "Pesquisadores (mínimo mestre) vinculados a IES/P do Espírito Santo, professores (tutores) e estudantes da Rede Pública de Educação Básica do Espírito Santo."</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Selecionar projetos que promovam o interesse pela ciência, desenvolvimento tecnológico e inovação em estudantes da Rede Pública de Educação Básica do Espírito Santo. O programa visa incentivar a participação ativa dos estudantes em pesquisa, popularizar a ciência na comunidade escolar, e fortalecer parcerias entre IES/P e escolas públicas para a formação de qualidade e inclusão social.</t>
+          <t>O Programa de Iniciação Científica Júnior (PICJr) visa apoiar financeiramente projetos de pesquisa desenvolvidos em parceria entre escolas públicas de Educação Básica e Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo. O objetivo é aproximar estudantes da rede pública de práticas científicas, sob a orientação de um pesquisador coordenador e a coorientação de um professor tutor, despertando o interesse pela ciência, desenvolvimento tecnológico e inovação.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores (mínimo mestre, com vínculo estatutário ou celetista por tempo indeterminado) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo.</t>
+          <t>Pesquisadores (mínimo mestre) vinculados a IES/P do Espírito Santo, professores (tutores) e estudantes da Rede Pública de Educação Básica do Espírito Santo.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -581,21 +571,20 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas.)
-2026-09-21: Envio da proposta e documentos (até as 17h59)
-?: Prazo para recorrer (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação)
-?: Prazo para recorrer (Até 5 dias úteis após a divulgação do resultado preliminar de análise de mérito)
-2027-02-09: Contratação dos projetos selecionados</t>
+          <t>2026-09-21: Submissão de propostas e documentos (Até as 17h59)
+?: Interposição de recursos (habilitação) (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação)
+?: Interposição de recursos (análise de mérito) (Até 5 dias úteis após a divulgação do resultado preliminar de análise de mérito)
+2027-02-09: Contratação dos projetos selecionados (A partir de)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>O coordenador de cada projeto contratado recebe um auxílio financeiro de R$ 10.000,00. Somente as cinco bolsas de Iniciação Científica Júnior (ICJr) são obrigatórias para implementação; as demais modalidades (BCO, BTU e ICT) são opcionais. Os valores mensais das bolsas são definidos na Tabela de Valores de Bolsas e Auxílios da Fapes. Cada coordenador pode apresentar apenas uma proposta. É obrigatório mencionar o apoio da Fapes e Sedu em todas as publicações e divulgações de atividades. É obrigatória a comunicação formal à Fapes sobre criações intelectuais resultantes do projeto e a partilha de resultados econômicos.</t>
+          <t>O coordenador de cada projeto contratado recebe um auxílio financeiro de R$ 10.000,00 para desenvolver o projeto de pesquisa, além das bolsas. As modalidades de bolsas incluem uma bolsa de coordenador (BCO), uma de tutor (BTU), uma de iniciação científica e tecnológica (ICT) e cinco de iniciação científica júnior (ICJr), sendo apenas as cinco bolsas de ICJr obrigatórias. A Fapes pode alterar as datas e prazos do cronograma. Cada coordenador pode apresentar apenas uma proposta. A etapa de habilitação é eliminatória. Propostas com nota final inferior a 70 pontos são desclassificadas. É proibido acumular bolsas da Fapes com outras bolsas (exceto as de inclusão social) e não implementar as bolsas de ICJr. É obrigatório mencionar o apoio da Fapes e da Sedu em todas as publicações e divulgações. A Fapes abre mão dos direitos de participação e propriedade sobre pesquisas e projetos que apoia, mas os resultados econômicos da exploração comercial serão partilhados.</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/PIC_JR_2027%20-.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Ed.%2019.2026%20PIC%20JR%202027%20-%201ª%20Alteração%20-%20Publicada.pdf</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -615,9 +604,9 @@
           <t>EDITAL FAPES Nº 20/2026 - BOLSAS DE PÓS-DOUTORADO SÊNIOR</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 04/09/2026</t>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -625,12 +614,7 @@
           <t>2026-09-19: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao término da submissão das propostas.)</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "Selecionar propostas para concessão de bolsas de pós-doutorado sênior, a serem realizadas em instituições de excelência no país ou no exterior. O objetivo é aprimorar a qualificação de pesquisadores, fortalecer as atividades de pesquisa científica e tecnológica, e ampliar a cooperação acadêmica nacional e internacional, contribuindo para o desenvolvimento científico e tecnológico no Espírito Santo e no Brasil." → "A presente chamada pública tem por objetivo selecionar propostas para concessão de bolsas de pós-doutorado sênior, a serem realizadas em instituições de excelência, no país ou no exterior. Visa o aprimoramento da qualificação de pesquisadores, o fortalecimento das atividades de pesquisa científica e tecnológica e a ampliação da cooperação acadêmica nacional e internacional. O edital apoia projetos de pesquisa que contribuam para o desenvolvimento científico e tecnológico no Espírito Santo e do Brasil."
-Público-alvo: "Pesquisadores doutores vinculados a Instituições de Ensino e/ou Pesquisa (IES/P), públicas ou privadas, sediadas no estado do Espírito Santo, que tenham obtido o título de doutor há mais de 8 anos, conforme faixas de titulação especificadas no edital." → "Pesquisador com título de doutor conforme discriminado nas faixas descritas no edital e com vínculo em Instituição de Ensino ou Pesquisa (IES/P), pública ou privada, sediada no estado do Espírito Santo."</t>
-        </is>
-      </c>
+      <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>A presente chamada pública tem por objetivo selecionar propostas para concessão de bolsas de pós-doutorado sênior, a serem realizadas em instituições de excelência, no país ou no exterior. Visa o aprimoramento da qualificação de pesquisadores, o fortalecimento das atividades de pesquisa científica e tecnológica e a ampliação da cooperação acadêmica nacional e internacional. O edital apoia projetos de pesquisa que contribuam para o desenvolvimento científico e tecnológico no Espírito Santo e do Brasil.</t>
@@ -688,9 +672,9 @@
           <t>EDITAL FAPES/CNPq/CAPES Nº 22/2026 - PROGRAMA DE APOIO À FIXAÇÃO DE DOUTORES NO BRASIL (PROFIX-CB)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 04/09/2026</t>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -698,14 +682,7 @@
           <t>2026-09-24: Prazo para impugnação do edital (até 5 dias úteis anteriores ao encerramento do prazo de submissão das propostas)</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "O Programa de Apoio à Fixação de Doutores no Brasil – Conhecimento Brasil (PROFIX-CB) é uma iniciativa do CNPq, CAPES e FAPs para atrair, inserir e fixar pesquisadores doutores em instituições de pesquisa, universidades e centros de inovação no país. Seu propósito é criar condições para que o doutor estabeleça uma trajetória científica de médio prazo, contribuindo para a formação de recursos humanos, fortalecimento de programas de pós-graduação, consolidação de grupos de pesquisa e geração de conhecimento e inovação, especialmente em áreas estratégicas para o desenvolvimento científico, tecnológico e de inovação do Espírito Santo." → "O Programa de Apoio à Fixação de Doutores no Brasil – Conhecimento Brasil (PROFIX-CB) é uma iniciativa do CNPq, CAPES e FAPs para atrair, inserir e fixar pesquisadores doutores em instituições de pesquisa, universidades e centros de inovação no país, especialmente em áreas estratégicas para o desenvolvimento científico, tecnológico e de inovação. O objetivo é apoiar projetos de pesquisa que criem condições para que recém-doutores sem vínculo empregatício desenvolvam uma trajetória científica de médio prazo no Espírito Santo, contribuindo para a formação de recursos humanos, fortalecimento de programas de pós-graduação, consolidação de grupos de pesquisa e geração de conhecimento e inovação, alinhado ao Plano Estadual de CT&amp;I do Espírito Santo (PCTI-ES) 2026–2035."
-Público-alvo: "Pesquisadores doutores (com título obtido há no máximo 10 anos até a data limite de submissão da proposta), residentes no Espírito Santo, sem vínculo empregatício, que atuarão como coordenadores e bolsistas PROFIX-CB em Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no Espírito Santo, com um Programa de Pós-graduação (PPG) parceiro." → "Pesquisadores doutores com título obtido há no máximo 10 anos, residentes no Espírito Santo durante a execução do projeto, com disponibilidade de 40 horas semanais presenciais, não aposentados, sem vínculo empregatício ou acúmulo de bolsas no momento da contratação e durante as atividades como bolsista PROFIX-CB. Devem estar vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, com registro ativo no Diretório de Instituições do CNPq e anuência do PPG parceiro."
-Valor por proposta: "R$ 400.000,00" → "R$ 400.000,00 (auxílio financeiro da Fapes)"
-Contato: "bolsas.duvidas@fapes.es.gov.br" → "bolsas.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br"</t>
-        </is>
-      </c>
+      <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>O Programa de Apoio à Fixação de Doutores no Brasil – Conhecimento Brasil (PROFIX-CB) é uma iniciativa do CNPq, CAPES e FAPs para atrair, inserir e fixar pesquisadores doutores em instituições de pesquisa, universidades e centros de inovação no país, especialmente em áreas estratégicas para o desenvolvimento científico, tecnológico e de inovação. O objetivo é apoiar projetos de pesquisa que criem condições para que recém-doutores sem vínculo empregatício desenvolvam uma trajetória científica de médio prazo no Espírito Santo, contribuindo para a formação de recursos humanos, fortalecimento de programas de pós-graduação, consolidação de grupos de pesquisa e geração de conhecimento e inovação, alinhado ao Plano Estadual de CT&amp;I do Espírito Santo (PCTI-ES) 2026–2035.</t>
@@ -1057,9 +1034,9 @@
           <t>EDITAL FAPES Nº 01/2026 – TCC EMPREENDEDOR INOVADOR</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 04/09/2026</t>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1205,9 +1182,9 @@
           <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 04/09/2026</t>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1215,12 +1192,7 @@
           <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas. O pedido deve ser enviado no E-Flow por meio do Formulário de Impugnação de Edital.)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "Apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que ofereçam apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas com produtos, serviços ou modelos de negócio inovadores. O edital visa ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de empreendedores, a sustentabilidade econômica das empresas incubadas e o desenvolvimento socioeconômico do Espírito Santo." → "O edital visa apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que buscam estimular e prestar apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas com produtos, serviços ou modelos de negócio inovadores. Este apoio busca ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de novos empreendedores e o desenvolvimento socioeconômico do estado."
-Submissão (removida): Submissão de propostas — 2026-08-25 a 2026-09-24</t>
-        </is>
-      </c>
+      <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
           <t>O edital visa apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que buscam estimular e prestar apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas com produtos, serviços ou modelos de negócio inovadores. Este apoio busca ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de novos empreendedores e o desenvolvimento socioeconômico do estado.</t>
@@ -1474,11 +1446,7 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Submissão de propostas (Até as 11:59 (horário de Brasília) via https://sistema.confap.org.br. Proponentes devem verificar com suas FAPs sobre submissão em plataformas próprias.)</t>
-        </is>
-      </c>
+      <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-06 10:52
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -532,9 +524,9 @@
           <t>EDITAL FAPES Nº 19/2026 - PIC JR 2027</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 05/09/2026</t>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -542,12 +534,7 @@
           <t>2026-09-21: Submissão de propostas e documentos (Até as 17h59)</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "Selecionar projetos que promovam o interesse pela ciência, desenvolvimento tecnológico e inovação em estudantes da Rede Pública de Educação Básica do Espírito Santo. O programa visa incentivar a participação ativa dos estudantes em pesquisa, popularizar a ciência na comunidade escolar, e fortalecer parcerias entre IES/P e escolas públicas para a formação de qualidade e inclusão social." → "O Programa de Iniciação Científica Júnior (PICJr) visa apoiar financeiramente projetos de pesquisa desenvolvidos em parceria entre escolas públicas de Educação Básica e Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo. O objetivo é aproximar estudantes da rede pública de práticas científicas, sob a orientação de um pesquisador coordenador e a coorientação de um professor tutor, despertando o interesse pela ciência, desenvolvimento tecnológico e inovação."
-Público-alvo: "Pesquisadores (mínimo mestre, com vínculo estatutário ou celetista por tempo indeterminado) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo." → "Pesquisadores (mínimo mestre) vinculados a IES/P do Espírito Santo, professores (tutores) e estudantes da Rede Pública de Educação Básica do Espírito Santo."</t>
-        </is>
-      </c>
+      <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>O Programa de Iniciação Científica Júnior (PICJr) visa apoiar financeiramente projetos de pesquisa desenvolvidos em parceria entre escolas públicas de Educação Básica e Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo. O objetivo é aproximar estudantes da rede pública de práticas científicas, sob a orientação de um pesquisador coordenador e a coorientação de um professor tutor, despertando o interesse pela ciência, desenvolvimento tecnológico e inovação.</t>

</xml_diff>